<commit_message>
Is takibi: Is Listesi'ne tarih/kapanis/commit sutunlari + CLAUDE.md takip kurallari
- BETAVUS_Is_Listesi.xlsx: Eklenme Tarihi, Kapanis Tarihi, Commit / Yapilan
  sutunlari; '3 - Genel / Diger' segmenti (+Ozet satiri); durum renkleri;
  acilir listeler 500. satira kadar
- CLAUDE.md: iki bilgisayardaki Claude oturumu icin is listesi protokolu
- HANDOVER.md: calisma dizini guncellendi, baslangic sirasina is listesi
- .vercelignore: is listesi ve CLAUDE.md sitede yayinlanmaz

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Özet" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'İş Listesi'!$A$4:$K$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'İş Listesi'!$A$4:$N$500</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,8 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
+    <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -110,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -156,10 +157,88 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="007F6000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF2CC"/>
+          <bgColor rgb="00FFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="001F3864"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00DDEBF7"/>
+          <bgColor rgb="00DDEBF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00833C0B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FCE4D6"/>
+          <bgColor rgb="00FCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="004B2E83"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00EDE7F6"/>
+          <bgColor rgb="00EDE7F6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00375623"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E2EFDA"/>
+          <bgColor rgb="00E2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="007F7F7F"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00EDEDED"/>
+          <bgColor rgb="00EDEDED"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -521,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:N500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -535,6 +614,9 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -544,10 +626,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sıra: önce Faz 1 (teknik veri doğruluğu), sonra Faz 2 (arayüz). Durum, Öncelik, Sorumlu, Hedef Tarih ve Not sütunları doldurulmak içindir. "Öneri" durumundaki satırlar ekip listesinde yoktu; onay bekliyor.</t>
+          <t>Nasıl kullanılır: Yeni fikir = yeni satır, Durum "Öneri" (karar bekliyor). Claude her oturumda listeyi okur ve "Öneri" satırlarını "şimdi yapayım mı, plana mı alayım?" diye sorar. Plana alınan iş = "Açık", üzerinde çalışılan = "Devam ediyor", iş bitince Claude "Tamamlandı" yapar, Kapanış Tarihi ile Commit'i doldurur. Önce Faz 1 (teknik veri doğruluğu), sonra Faz 2 (arayüz). Excel'de düzenlemeden önce Pull, kaydettikten hemen sonra Commit + Push.</t>
         </is>
       </c>
     </row>
@@ -605,6 +687,21 @@
       <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Not</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Eklenme Tarihi</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Kapanış Tarihi</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>Commit / Yapılan</t>
         </is>
       </c>
     </row>
@@ -650,6 +747,11 @@
       <c r="I5" s="7" t="inlineStr"/>
       <c r="J5" s="8" t="inlineStr"/>
       <c r="K5" s="7" t="inlineStr"/>
+      <c r="L5" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M5" s="19" t="n"/>
+      <c r="N5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -693,6 +795,11 @@
       <c r="I6" s="7" t="inlineStr"/>
       <c r="J6" s="8" t="inlineStr"/>
       <c r="K6" s="7" t="inlineStr"/>
+      <c r="L6" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M6" s="19" t="n"/>
+      <c r="N6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -736,6 +843,11 @@
       <c r="I7" s="7" t="inlineStr"/>
       <c r="J7" s="8" t="inlineStr"/>
       <c r="K7" s="7" t="inlineStr"/>
+      <c r="L7" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M7" s="19" t="n"/>
+      <c r="N7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -779,6 +891,11 @@
       <c r="I8" s="7" t="inlineStr"/>
       <c r="J8" s="8" t="inlineStr"/>
       <c r="K8" s="7" t="inlineStr"/>
+      <c r="L8" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M8" s="19" t="n"/>
+      <c r="N8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -822,6 +939,11 @@
       <c r="I9" s="7" t="inlineStr"/>
       <c r="J9" s="8" t="inlineStr"/>
       <c r="K9" s="7" t="inlineStr"/>
+      <c r="L9" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M9" s="19" t="n"/>
+      <c r="N9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -865,6 +987,11 @@
       <c r="I10" s="7" t="inlineStr"/>
       <c r="J10" s="8" t="inlineStr"/>
       <c r="K10" s="7" t="inlineStr"/>
+      <c r="L10" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M10" s="19" t="n"/>
+      <c r="N10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -908,6 +1035,11 @@
       <c r="I11" s="7" t="inlineStr"/>
       <c r="J11" s="8" t="inlineStr"/>
       <c r="K11" s="7" t="inlineStr"/>
+      <c r="L11" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M11" s="19" t="n"/>
+      <c r="N11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -951,6 +1083,11 @@
       <c r="I12" s="7" t="inlineStr"/>
       <c r="J12" s="8" t="inlineStr"/>
       <c r="K12" s="7" t="inlineStr"/>
+      <c r="L12" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M12" s="19" t="n"/>
+      <c r="N12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -994,6 +1131,11 @@
       <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="8" t="inlineStr"/>
       <c r="K13" s="7" t="inlineStr"/>
+      <c r="L13" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M13" s="19" t="n"/>
+      <c r="N13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -1037,6 +1179,11 @@
       <c r="I14" s="7" t="inlineStr"/>
       <c r="J14" s="8" t="inlineStr"/>
       <c r="K14" s="7" t="inlineStr"/>
+      <c r="L14" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M14" s="19" t="n"/>
+      <c r="N14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1080,6 +1227,11 @@
       <c r="I15" s="7" t="inlineStr"/>
       <c r="J15" s="8" t="inlineStr"/>
       <c r="K15" s="7" t="inlineStr"/>
+      <c r="L15" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M15" s="19" t="n"/>
+      <c r="N15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -1123,6 +1275,11 @@
       <c r="I16" s="7" t="inlineStr"/>
       <c r="J16" s="8" t="inlineStr"/>
       <c r="K16" s="7" t="inlineStr"/>
+      <c r="L16" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M16" s="19" t="n"/>
+      <c r="N16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -1166,24 +1323,1504 @@
       <c r="I17" s="7" t="inlineStr"/>
       <c r="J17" s="8" t="inlineStr"/>
       <c r="K17" s="7" t="inlineStr"/>
+      <c r="L17" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M17" s="19" t="n"/>
+      <c r="N17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="L18" s="20" t="n"/>
+    </row>
+    <row r="19">
+      <c r="L19" s="20" t="n"/>
+    </row>
+    <row r="20">
+      <c r="L20" s="20" t="n"/>
+    </row>
+    <row r="21">
+      <c r="L21" s="20" t="n"/>
+    </row>
+    <row r="22">
+      <c r="L22" s="20" t="n"/>
+    </row>
+    <row r="23">
+      <c r="L23" s="20" t="n"/>
+    </row>
+    <row r="24">
+      <c r="L24" s="20" t="n"/>
+    </row>
+    <row r="25">
+      <c r="L25" s="20" t="n"/>
+    </row>
+    <row r="26">
+      <c r="L26" s="20" t="n"/>
+    </row>
+    <row r="27">
+      <c r="L27" s="20" t="n"/>
+    </row>
+    <row r="28">
+      <c r="L28" s="20" t="n"/>
+    </row>
+    <row r="29">
+      <c r="L29" s="20" t="n"/>
+    </row>
+    <row r="30">
+      <c r="L30" s="20" t="n"/>
+    </row>
+    <row r="31">
+      <c r="L31" s="20" t="n"/>
+    </row>
+    <row r="32">
+      <c r="L32" s="20" t="n"/>
+    </row>
+    <row r="33">
+      <c r="L33" s="20" t="n"/>
+    </row>
+    <row r="34">
+      <c r="L34" s="20" t="n"/>
+    </row>
+    <row r="35">
+      <c r="L35" s="20" t="n"/>
+    </row>
+    <row r="36">
+      <c r="L36" s="20" t="n"/>
+    </row>
+    <row r="37">
+      <c r="L37" s="20" t="n"/>
+    </row>
+    <row r="38">
+      <c r="L38" s="20" t="n"/>
+    </row>
+    <row r="39">
+      <c r="L39" s="20" t="n"/>
+    </row>
+    <row r="40">
+      <c r="L40" s="20" t="n"/>
+    </row>
+    <row r="41">
+      <c r="L41" s="20" t="n"/>
+    </row>
+    <row r="42">
+      <c r="L42" s="20" t="n"/>
+    </row>
+    <row r="43">
+      <c r="L43" s="20" t="n"/>
+    </row>
+    <row r="44">
+      <c r="L44" s="20" t="n"/>
+    </row>
+    <row r="45">
+      <c r="L45" s="20" t="n"/>
+    </row>
+    <row r="46">
+      <c r="L46" s="20" t="n"/>
+    </row>
+    <row r="47">
+      <c r="L47" s="20" t="n"/>
+    </row>
+    <row r="48">
+      <c r="L48" s="20" t="n"/>
+    </row>
+    <row r="49">
+      <c r="L49" s="20" t="n"/>
+    </row>
+    <row r="50">
+      <c r="L50" s="20" t="n"/>
+    </row>
+    <row r="51">
+      <c r="L51" s="20" t="n"/>
+    </row>
+    <row r="52">
+      <c r="L52" s="20" t="n"/>
+    </row>
+    <row r="53">
+      <c r="L53" s="20" t="n"/>
+    </row>
+    <row r="54">
+      <c r="L54" s="20" t="n"/>
+    </row>
+    <row r="55">
+      <c r="L55" s="20" t="n"/>
+    </row>
+    <row r="56">
+      <c r="L56" s="20" t="n"/>
+    </row>
+    <row r="57">
+      <c r="L57" s="20" t="n"/>
+    </row>
+    <row r="58">
+      <c r="L58" s="20" t="n"/>
+    </row>
+    <row r="59">
+      <c r="L59" s="20" t="n"/>
+    </row>
+    <row r="60">
+      <c r="L60" s="20" t="n"/>
+    </row>
+    <row r="61">
+      <c r="L61" s="20" t="n"/>
+    </row>
+    <row r="62">
+      <c r="L62" s="20" t="n"/>
+    </row>
+    <row r="63">
+      <c r="L63" s="20" t="n"/>
+    </row>
+    <row r="64">
+      <c r="L64" s="20" t="n"/>
+    </row>
+    <row r="65">
+      <c r="L65" s="20" t="n"/>
+    </row>
+    <row r="66">
+      <c r="L66" s="20" t="n"/>
+    </row>
+    <row r="67">
+      <c r="L67" s="20" t="n"/>
+    </row>
+    <row r="68">
+      <c r="L68" s="20" t="n"/>
+    </row>
+    <row r="69">
+      <c r="L69" s="20" t="n"/>
+    </row>
+    <row r="70">
+      <c r="L70" s="20" t="n"/>
+    </row>
+    <row r="71">
+      <c r="L71" s="20" t="n"/>
+    </row>
+    <row r="72">
+      <c r="L72" s="20" t="n"/>
+    </row>
+    <row r="73">
+      <c r="L73" s="20" t="n"/>
+    </row>
+    <row r="74">
+      <c r="L74" s="20" t="n"/>
+    </row>
+    <row r="75">
+      <c r="L75" s="20" t="n"/>
+    </row>
+    <row r="76">
+      <c r="L76" s="20" t="n"/>
+    </row>
+    <row r="77">
+      <c r="L77" s="20" t="n"/>
+    </row>
+    <row r="78">
+      <c r="L78" s="20" t="n"/>
+    </row>
+    <row r="79">
+      <c r="L79" s="20" t="n"/>
+    </row>
+    <row r="80">
+      <c r="L80" s="20" t="n"/>
+    </row>
+    <row r="81">
+      <c r="L81" s="20" t="n"/>
+    </row>
+    <row r="82">
+      <c r="L82" s="20" t="n"/>
+    </row>
+    <row r="83">
+      <c r="L83" s="20" t="n"/>
+    </row>
+    <row r="84">
+      <c r="L84" s="20" t="n"/>
+    </row>
+    <row r="85">
+      <c r="L85" s="20" t="n"/>
+    </row>
+    <row r="86">
+      <c r="L86" s="20" t="n"/>
+    </row>
+    <row r="87">
+      <c r="L87" s="20" t="n"/>
+    </row>
+    <row r="88">
+      <c r="L88" s="20" t="n"/>
+    </row>
+    <row r="89">
+      <c r="L89" s="20" t="n"/>
+    </row>
+    <row r="90">
+      <c r="L90" s="20" t="n"/>
+    </row>
+    <row r="91">
+      <c r="L91" s="20" t="n"/>
+    </row>
+    <row r="92">
+      <c r="L92" s="20" t="n"/>
+    </row>
+    <row r="93">
+      <c r="L93" s="20" t="n"/>
+    </row>
+    <row r="94">
+      <c r="L94" s="20" t="n"/>
+    </row>
+    <row r="95">
+      <c r="L95" s="20" t="n"/>
+    </row>
+    <row r="96">
+      <c r="L96" s="20" t="n"/>
+    </row>
+    <row r="97">
+      <c r="L97" s="20" t="n"/>
+    </row>
+    <row r="98">
+      <c r="L98" s="20" t="n"/>
+    </row>
+    <row r="99">
+      <c r="L99" s="20" t="n"/>
+    </row>
+    <row r="100">
+      <c r="L100" s="20" t="n"/>
+    </row>
+    <row r="101">
+      <c r="L101" s="20" t="n"/>
+    </row>
+    <row r="102">
+      <c r="L102" s="20" t="n"/>
+    </row>
+    <row r="103">
+      <c r="L103" s="20" t="n"/>
+    </row>
+    <row r="104">
+      <c r="L104" s="20" t="n"/>
+    </row>
+    <row r="105">
+      <c r="L105" s="20" t="n"/>
+    </row>
+    <row r="106">
+      <c r="L106" s="20" t="n"/>
+    </row>
+    <row r="107">
+      <c r="L107" s="20" t="n"/>
+    </row>
+    <row r="108">
+      <c r="L108" s="20" t="n"/>
+    </row>
+    <row r="109">
+      <c r="L109" s="20" t="n"/>
+    </row>
+    <row r="110">
+      <c r="L110" s="20" t="n"/>
+    </row>
+    <row r="111">
+      <c r="L111" s="20" t="n"/>
+    </row>
+    <row r="112">
+      <c r="L112" s="20" t="n"/>
+    </row>
+    <row r="113">
+      <c r="L113" s="20" t="n"/>
+    </row>
+    <row r="114">
+      <c r="L114" s="20" t="n"/>
+    </row>
+    <row r="115">
+      <c r="L115" s="20" t="n"/>
+    </row>
+    <row r="116">
+      <c r="L116" s="20" t="n"/>
+    </row>
+    <row r="117">
+      <c r="L117" s="20" t="n"/>
+    </row>
+    <row r="118">
+      <c r="L118" s="20" t="n"/>
+    </row>
+    <row r="119">
+      <c r="L119" s="20" t="n"/>
+    </row>
+    <row r="120">
+      <c r="L120" s="20" t="n"/>
+    </row>
+    <row r="121">
+      <c r="L121" s="20" t="n"/>
+    </row>
+    <row r="122">
+      <c r="L122" s="20" t="n"/>
+    </row>
+    <row r="123">
+      <c r="L123" s="20" t="n"/>
+    </row>
+    <row r="124">
+      <c r="L124" s="20" t="n"/>
+    </row>
+    <row r="125">
+      <c r="L125" s="20" t="n"/>
+    </row>
+    <row r="126">
+      <c r="L126" s="20" t="n"/>
+    </row>
+    <row r="127">
+      <c r="L127" s="20" t="n"/>
+    </row>
+    <row r="128">
+      <c r="L128" s="20" t="n"/>
+    </row>
+    <row r="129">
+      <c r="L129" s="20" t="n"/>
+    </row>
+    <row r="130">
+      <c r="L130" s="20" t="n"/>
+    </row>
+    <row r="131">
+      <c r="L131" s="20" t="n"/>
+    </row>
+    <row r="132">
+      <c r="L132" s="20" t="n"/>
+    </row>
+    <row r="133">
+      <c r="L133" s="20" t="n"/>
+    </row>
+    <row r="134">
+      <c r="L134" s="20" t="n"/>
+    </row>
+    <row r="135">
+      <c r="L135" s="20" t="n"/>
+    </row>
+    <row r="136">
+      <c r="L136" s="20" t="n"/>
+    </row>
+    <row r="137">
+      <c r="L137" s="20" t="n"/>
+    </row>
+    <row r="138">
+      <c r="L138" s="20" t="n"/>
+    </row>
+    <row r="139">
+      <c r="L139" s="20" t="n"/>
+    </row>
+    <row r="140">
+      <c r="L140" s="20" t="n"/>
+    </row>
+    <row r="141">
+      <c r="L141" s="20" t="n"/>
+    </row>
+    <row r="142">
+      <c r="L142" s="20" t="n"/>
+    </row>
+    <row r="143">
+      <c r="L143" s="20" t="n"/>
+    </row>
+    <row r="144">
+      <c r="L144" s="20" t="n"/>
+    </row>
+    <row r="145">
+      <c r="L145" s="20" t="n"/>
+    </row>
+    <row r="146">
+      <c r="L146" s="20" t="n"/>
+    </row>
+    <row r="147">
+      <c r="L147" s="20" t="n"/>
+    </row>
+    <row r="148">
+      <c r="L148" s="20" t="n"/>
+    </row>
+    <row r="149">
+      <c r="L149" s="20" t="n"/>
+    </row>
+    <row r="150">
+      <c r="L150" s="20" t="n"/>
+    </row>
+    <row r="151">
+      <c r="L151" s="20" t="n"/>
+    </row>
+    <row r="152">
+      <c r="L152" s="20" t="n"/>
+    </row>
+    <row r="153">
+      <c r="L153" s="20" t="n"/>
+    </row>
+    <row r="154">
+      <c r="L154" s="20" t="n"/>
+    </row>
+    <row r="155">
+      <c r="L155" s="20" t="n"/>
+    </row>
+    <row r="156">
+      <c r="L156" s="20" t="n"/>
+    </row>
+    <row r="157">
+      <c r="L157" s="20" t="n"/>
+    </row>
+    <row r="158">
+      <c r="L158" s="20" t="n"/>
+    </row>
+    <row r="159">
+      <c r="L159" s="20" t="n"/>
+    </row>
+    <row r="160">
+      <c r="L160" s="20" t="n"/>
+    </row>
+    <row r="161">
+      <c r="L161" s="20" t="n"/>
+    </row>
+    <row r="162">
+      <c r="L162" s="20" t="n"/>
+    </row>
+    <row r="163">
+      <c r="L163" s="20" t="n"/>
+    </row>
+    <row r="164">
+      <c r="L164" s="20" t="n"/>
+    </row>
+    <row r="165">
+      <c r="L165" s="20" t="n"/>
+    </row>
+    <row r="166">
+      <c r="L166" s="20" t="n"/>
+    </row>
+    <row r="167">
+      <c r="L167" s="20" t="n"/>
+    </row>
+    <row r="168">
+      <c r="L168" s="20" t="n"/>
+    </row>
+    <row r="169">
+      <c r="L169" s="20" t="n"/>
+    </row>
+    <row r="170">
+      <c r="L170" s="20" t="n"/>
+    </row>
+    <row r="171">
+      <c r="L171" s="20" t="n"/>
+    </row>
+    <row r="172">
+      <c r="L172" s="20" t="n"/>
+    </row>
+    <row r="173">
+      <c r="L173" s="20" t="n"/>
+    </row>
+    <row r="174">
+      <c r="L174" s="20" t="n"/>
+    </row>
+    <row r="175">
+      <c r="L175" s="20" t="n"/>
+    </row>
+    <row r="176">
+      <c r="L176" s="20" t="n"/>
+    </row>
+    <row r="177">
+      <c r="L177" s="20" t="n"/>
+    </row>
+    <row r="178">
+      <c r="L178" s="20" t="n"/>
+    </row>
+    <row r="179">
+      <c r="L179" s="20" t="n"/>
+    </row>
+    <row r="180">
+      <c r="L180" s="20" t="n"/>
+    </row>
+    <row r="181">
+      <c r="L181" s="20" t="n"/>
+    </row>
+    <row r="182">
+      <c r="L182" s="20" t="n"/>
+    </row>
+    <row r="183">
+      <c r="L183" s="20" t="n"/>
+    </row>
+    <row r="184">
+      <c r="L184" s="20" t="n"/>
+    </row>
+    <row r="185">
+      <c r="L185" s="20" t="n"/>
+    </row>
+    <row r="186">
+      <c r="L186" s="20" t="n"/>
+    </row>
+    <row r="187">
+      <c r="L187" s="20" t="n"/>
+    </row>
+    <row r="188">
+      <c r="L188" s="20" t="n"/>
+    </row>
+    <row r="189">
+      <c r="L189" s="20" t="n"/>
+    </row>
+    <row r="190">
+      <c r="L190" s="20" t="n"/>
+    </row>
+    <row r="191">
+      <c r="L191" s="20" t="n"/>
+    </row>
+    <row r="192">
+      <c r="L192" s="20" t="n"/>
+    </row>
+    <row r="193">
+      <c r="L193" s="20" t="n"/>
+    </row>
+    <row r="194">
+      <c r="L194" s="20" t="n"/>
+    </row>
+    <row r="195">
+      <c r="L195" s="20" t="n"/>
+    </row>
+    <row r="196">
+      <c r="L196" s="20" t="n"/>
+    </row>
+    <row r="197">
+      <c r="L197" s="20" t="n"/>
+    </row>
+    <row r="198">
+      <c r="L198" s="20" t="n"/>
+    </row>
+    <row r="199">
+      <c r="L199" s="20" t="n"/>
+    </row>
+    <row r="200">
+      <c r="L200" s="20" t="n"/>
+    </row>
+    <row r="201">
+      <c r="L201" s="20" t="n"/>
+    </row>
+    <row r="202">
+      <c r="L202" s="20" t="n"/>
+    </row>
+    <row r="203">
+      <c r="L203" s="20" t="n"/>
+    </row>
+    <row r="204">
+      <c r="L204" s="20" t="n"/>
+    </row>
+    <row r="205">
+      <c r="L205" s="20" t="n"/>
+    </row>
+    <row r="206">
+      <c r="L206" s="20" t="n"/>
+    </row>
+    <row r="207">
+      <c r="L207" s="20" t="n"/>
+    </row>
+    <row r="208">
+      <c r="L208" s="20" t="n"/>
+    </row>
+    <row r="209">
+      <c r="L209" s="20" t="n"/>
+    </row>
+    <row r="210">
+      <c r="L210" s="20" t="n"/>
+    </row>
+    <row r="211">
+      <c r="L211" s="20" t="n"/>
+    </row>
+    <row r="212">
+      <c r="L212" s="20" t="n"/>
+    </row>
+    <row r="213">
+      <c r="L213" s="20" t="n"/>
+    </row>
+    <row r="214">
+      <c r="L214" s="20" t="n"/>
+    </row>
+    <row r="215">
+      <c r="L215" s="20" t="n"/>
+    </row>
+    <row r="216">
+      <c r="L216" s="20" t="n"/>
+    </row>
+    <row r="217">
+      <c r="L217" s="20" t="n"/>
+    </row>
+    <row r="218">
+      <c r="L218" s="20" t="n"/>
+    </row>
+    <row r="219">
+      <c r="L219" s="20" t="n"/>
+    </row>
+    <row r="220">
+      <c r="L220" s="20" t="n"/>
+    </row>
+    <row r="221">
+      <c r="L221" s="20" t="n"/>
+    </row>
+    <row r="222">
+      <c r="L222" s="20" t="n"/>
+    </row>
+    <row r="223">
+      <c r="L223" s="20" t="n"/>
+    </row>
+    <row r="224">
+      <c r="L224" s="20" t="n"/>
+    </row>
+    <row r="225">
+      <c r="L225" s="20" t="n"/>
+    </row>
+    <row r="226">
+      <c r="L226" s="20" t="n"/>
+    </row>
+    <row r="227">
+      <c r="L227" s="20" t="n"/>
+    </row>
+    <row r="228">
+      <c r="L228" s="20" t="n"/>
+    </row>
+    <row r="229">
+      <c r="L229" s="20" t="n"/>
+    </row>
+    <row r="230">
+      <c r="L230" s="20" t="n"/>
+    </row>
+    <row r="231">
+      <c r="L231" s="20" t="n"/>
+    </row>
+    <row r="232">
+      <c r="L232" s="20" t="n"/>
+    </row>
+    <row r="233">
+      <c r="L233" s="20" t="n"/>
+    </row>
+    <row r="234">
+      <c r="L234" s="20" t="n"/>
+    </row>
+    <row r="235">
+      <c r="L235" s="20" t="n"/>
+    </row>
+    <row r="236">
+      <c r="L236" s="20" t="n"/>
+    </row>
+    <row r="237">
+      <c r="L237" s="20" t="n"/>
+    </row>
+    <row r="238">
+      <c r="L238" s="20" t="n"/>
+    </row>
+    <row r="239">
+      <c r="L239" s="20" t="n"/>
+    </row>
+    <row r="240">
+      <c r="L240" s="20" t="n"/>
+    </row>
+    <row r="241">
+      <c r="L241" s="20" t="n"/>
+    </row>
+    <row r="242">
+      <c r="L242" s="20" t="n"/>
+    </row>
+    <row r="243">
+      <c r="L243" s="20" t="n"/>
+    </row>
+    <row r="244">
+      <c r="L244" s="20" t="n"/>
+    </row>
+    <row r="245">
+      <c r="L245" s="20" t="n"/>
+    </row>
+    <row r="246">
+      <c r="L246" s="20" t="n"/>
+    </row>
+    <row r="247">
+      <c r="L247" s="20" t="n"/>
+    </row>
+    <row r="248">
+      <c r="L248" s="20" t="n"/>
+    </row>
+    <row r="249">
+      <c r="L249" s="20" t="n"/>
+    </row>
+    <row r="250">
+      <c r="L250" s="20" t="n"/>
+    </row>
+    <row r="251">
+      <c r="L251" s="20" t="n"/>
+    </row>
+    <row r="252">
+      <c r="L252" s="20" t="n"/>
+    </row>
+    <row r="253">
+      <c r="L253" s="20" t="n"/>
+    </row>
+    <row r="254">
+      <c r="L254" s="20" t="n"/>
+    </row>
+    <row r="255">
+      <c r="L255" s="20" t="n"/>
+    </row>
+    <row r="256">
+      <c r="L256" s="20" t="n"/>
+    </row>
+    <row r="257">
+      <c r="L257" s="20" t="n"/>
+    </row>
+    <row r="258">
+      <c r="L258" s="20" t="n"/>
+    </row>
+    <row r="259">
+      <c r="L259" s="20" t="n"/>
+    </row>
+    <row r="260">
+      <c r="L260" s="20" t="n"/>
+    </row>
+    <row r="261">
+      <c r="L261" s="20" t="n"/>
+    </row>
+    <row r="262">
+      <c r="L262" s="20" t="n"/>
+    </row>
+    <row r="263">
+      <c r="L263" s="20" t="n"/>
+    </row>
+    <row r="264">
+      <c r="L264" s="20" t="n"/>
+    </row>
+    <row r="265">
+      <c r="L265" s="20" t="n"/>
+    </row>
+    <row r="266">
+      <c r="L266" s="20" t="n"/>
+    </row>
+    <row r="267">
+      <c r="L267" s="20" t="n"/>
+    </row>
+    <row r="268">
+      <c r="L268" s="20" t="n"/>
+    </row>
+    <row r="269">
+      <c r="L269" s="20" t="n"/>
+    </row>
+    <row r="270">
+      <c r="L270" s="20" t="n"/>
+    </row>
+    <row r="271">
+      <c r="L271" s="20" t="n"/>
+    </row>
+    <row r="272">
+      <c r="L272" s="20" t="n"/>
+    </row>
+    <row r="273">
+      <c r="L273" s="20" t="n"/>
+    </row>
+    <row r="274">
+      <c r="L274" s="20" t="n"/>
+    </row>
+    <row r="275">
+      <c r="L275" s="20" t="n"/>
+    </row>
+    <row r="276">
+      <c r="L276" s="20" t="n"/>
+    </row>
+    <row r="277">
+      <c r="L277" s="20" t="n"/>
+    </row>
+    <row r="278">
+      <c r="L278" s="20" t="n"/>
+    </row>
+    <row r="279">
+      <c r="L279" s="20" t="n"/>
+    </row>
+    <row r="280">
+      <c r="L280" s="20" t="n"/>
+    </row>
+    <row r="281">
+      <c r="L281" s="20" t="n"/>
+    </row>
+    <row r="282">
+      <c r="L282" s="20" t="n"/>
+    </row>
+    <row r="283">
+      <c r="L283" s="20" t="n"/>
+    </row>
+    <row r="284">
+      <c r="L284" s="20" t="n"/>
+    </row>
+    <row r="285">
+      <c r="L285" s="20" t="n"/>
+    </row>
+    <row r="286">
+      <c r="L286" s="20" t="n"/>
+    </row>
+    <row r="287">
+      <c r="L287" s="20" t="n"/>
+    </row>
+    <row r="288">
+      <c r="L288" s="20" t="n"/>
+    </row>
+    <row r="289">
+      <c r="L289" s="20" t="n"/>
+    </row>
+    <row r="290">
+      <c r="L290" s="20" t="n"/>
+    </row>
+    <row r="291">
+      <c r="L291" s="20" t="n"/>
+    </row>
+    <row r="292">
+      <c r="L292" s="20" t="n"/>
+    </row>
+    <row r="293">
+      <c r="L293" s="20" t="n"/>
+    </row>
+    <row r="294">
+      <c r="L294" s="20" t="n"/>
+    </row>
+    <row r="295">
+      <c r="L295" s="20" t="n"/>
+    </row>
+    <row r="296">
+      <c r="L296" s="20" t="n"/>
+    </row>
+    <row r="297">
+      <c r="L297" s="20" t="n"/>
+    </row>
+    <row r="298">
+      <c r="L298" s="20" t="n"/>
+    </row>
+    <row r="299">
+      <c r="L299" s="20" t="n"/>
+    </row>
+    <row r="300">
+      <c r="L300" s="20" t="n"/>
+    </row>
+    <row r="301">
+      <c r="L301" s="20" t="n"/>
+    </row>
+    <row r="302">
+      <c r="L302" s="20" t="n"/>
+    </row>
+    <row r="303">
+      <c r="L303" s="20" t="n"/>
+    </row>
+    <row r="304">
+      <c r="L304" s="20" t="n"/>
+    </row>
+    <row r="305">
+      <c r="L305" s="20" t="n"/>
+    </row>
+    <row r="306">
+      <c r="L306" s="20" t="n"/>
+    </row>
+    <row r="307">
+      <c r="L307" s="20" t="n"/>
+    </row>
+    <row r="308">
+      <c r="L308" s="20" t="n"/>
+    </row>
+    <row r="309">
+      <c r="L309" s="20" t="n"/>
+    </row>
+    <row r="310">
+      <c r="L310" s="20" t="n"/>
+    </row>
+    <row r="311">
+      <c r="L311" s="20" t="n"/>
+    </row>
+    <row r="312">
+      <c r="L312" s="20" t="n"/>
+    </row>
+    <row r="313">
+      <c r="L313" s="20" t="n"/>
+    </row>
+    <row r="314">
+      <c r="L314" s="20" t="n"/>
+    </row>
+    <row r="315">
+      <c r="L315" s="20" t="n"/>
+    </row>
+    <row r="316">
+      <c r="L316" s="20" t="n"/>
+    </row>
+    <row r="317">
+      <c r="L317" s="20" t="n"/>
+    </row>
+    <row r="318">
+      <c r="L318" s="20" t="n"/>
+    </row>
+    <row r="319">
+      <c r="L319" s="20" t="n"/>
+    </row>
+    <row r="320">
+      <c r="L320" s="20" t="n"/>
+    </row>
+    <row r="321">
+      <c r="L321" s="20" t="n"/>
+    </row>
+    <row r="322">
+      <c r="L322" s="20" t="n"/>
+    </row>
+    <row r="323">
+      <c r="L323" s="20" t="n"/>
+    </row>
+    <row r="324">
+      <c r="L324" s="20" t="n"/>
+    </row>
+    <row r="325">
+      <c r="L325" s="20" t="n"/>
+    </row>
+    <row r="326">
+      <c r="L326" s="20" t="n"/>
+    </row>
+    <row r="327">
+      <c r="L327" s="20" t="n"/>
+    </row>
+    <row r="328">
+      <c r="L328" s="20" t="n"/>
+    </row>
+    <row r="329">
+      <c r="L329" s="20" t="n"/>
+    </row>
+    <row r="330">
+      <c r="L330" s="20" t="n"/>
+    </row>
+    <row r="331">
+      <c r="L331" s="20" t="n"/>
+    </row>
+    <row r="332">
+      <c r="L332" s="20" t="n"/>
+    </row>
+    <row r="333">
+      <c r="L333" s="20" t="n"/>
+    </row>
+    <row r="334">
+      <c r="L334" s="20" t="n"/>
+    </row>
+    <row r="335">
+      <c r="L335" s="20" t="n"/>
+    </row>
+    <row r="336">
+      <c r="L336" s="20" t="n"/>
+    </row>
+    <row r="337">
+      <c r="L337" s="20" t="n"/>
+    </row>
+    <row r="338">
+      <c r="L338" s="20" t="n"/>
+    </row>
+    <row r="339">
+      <c r="L339" s="20" t="n"/>
+    </row>
+    <row r="340">
+      <c r="L340" s="20" t="n"/>
+    </row>
+    <row r="341">
+      <c r="L341" s="20" t="n"/>
+    </row>
+    <row r="342">
+      <c r="L342" s="20" t="n"/>
+    </row>
+    <row r="343">
+      <c r="L343" s="20" t="n"/>
+    </row>
+    <row r="344">
+      <c r="L344" s="20" t="n"/>
+    </row>
+    <row r="345">
+      <c r="L345" s="20" t="n"/>
+    </row>
+    <row r="346">
+      <c r="L346" s="20" t="n"/>
+    </row>
+    <row r="347">
+      <c r="L347" s="20" t="n"/>
+    </row>
+    <row r="348">
+      <c r="L348" s="20" t="n"/>
+    </row>
+    <row r="349">
+      <c r="L349" s="20" t="n"/>
+    </row>
+    <row r="350">
+      <c r="L350" s="20" t="n"/>
+    </row>
+    <row r="351">
+      <c r="L351" s="20" t="n"/>
+    </row>
+    <row r="352">
+      <c r="L352" s="20" t="n"/>
+    </row>
+    <row r="353">
+      <c r="L353" s="20" t="n"/>
+    </row>
+    <row r="354">
+      <c r="L354" s="20" t="n"/>
+    </row>
+    <row r="355">
+      <c r="L355" s="20" t="n"/>
+    </row>
+    <row r="356">
+      <c r="L356" s="20" t="n"/>
+    </row>
+    <row r="357">
+      <c r="L357" s="20" t="n"/>
+    </row>
+    <row r="358">
+      <c r="L358" s="20" t="n"/>
+    </row>
+    <row r="359">
+      <c r="L359" s="20" t="n"/>
+    </row>
+    <row r="360">
+      <c r="L360" s="20" t="n"/>
+    </row>
+    <row r="361">
+      <c r="L361" s="20" t="n"/>
+    </row>
+    <row r="362">
+      <c r="L362" s="20" t="n"/>
+    </row>
+    <row r="363">
+      <c r="L363" s="20" t="n"/>
+    </row>
+    <row r="364">
+      <c r="L364" s="20" t="n"/>
+    </row>
+    <row r="365">
+      <c r="L365" s="20" t="n"/>
+    </row>
+    <row r="366">
+      <c r="L366" s="20" t="n"/>
+    </row>
+    <row r="367">
+      <c r="L367" s="20" t="n"/>
+    </row>
+    <row r="368">
+      <c r="L368" s="20" t="n"/>
+    </row>
+    <row r="369">
+      <c r="L369" s="20" t="n"/>
+    </row>
+    <row r="370">
+      <c r="L370" s="20" t="n"/>
+    </row>
+    <row r="371">
+      <c r="L371" s="20" t="n"/>
+    </row>
+    <row r="372">
+      <c r="L372" s="20" t="n"/>
+    </row>
+    <row r="373">
+      <c r="L373" s="20" t="n"/>
+    </row>
+    <row r="374">
+      <c r="L374" s="20" t="n"/>
+    </row>
+    <row r="375">
+      <c r="L375" s="20" t="n"/>
+    </row>
+    <row r="376">
+      <c r="L376" s="20" t="n"/>
+    </row>
+    <row r="377">
+      <c r="L377" s="20" t="n"/>
+    </row>
+    <row r="378">
+      <c r="L378" s="20" t="n"/>
+    </row>
+    <row r="379">
+      <c r="L379" s="20" t="n"/>
+    </row>
+    <row r="380">
+      <c r="L380" s="20" t="n"/>
+    </row>
+    <row r="381">
+      <c r="L381" s="20" t="n"/>
+    </row>
+    <row r="382">
+      <c r="L382" s="20" t="n"/>
+    </row>
+    <row r="383">
+      <c r="L383" s="20" t="n"/>
+    </row>
+    <row r="384">
+      <c r="L384" s="20" t="n"/>
+    </row>
+    <row r="385">
+      <c r="L385" s="20" t="n"/>
+    </row>
+    <row r="386">
+      <c r="L386" s="20" t="n"/>
+    </row>
+    <row r="387">
+      <c r="L387" s="20" t="n"/>
+    </row>
+    <row r="388">
+      <c r="L388" s="20" t="n"/>
+    </row>
+    <row r="389">
+      <c r="L389" s="20" t="n"/>
+    </row>
+    <row r="390">
+      <c r="L390" s="20" t="n"/>
+    </row>
+    <row r="391">
+      <c r="L391" s="20" t="n"/>
+    </row>
+    <row r="392">
+      <c r="L392" s="20" t="n"/>
+    </row>
+    <row r="393">
+      <c r="L393" s="20" t="n"/>
+    </row>
+    <row r="394">
+      <c r="L394" s="20" t="n"/>
+    </row>
+    <row r="395">
+      <c r="L395" s="20" t="n"/>
+    </row>
+    <row r="396">
+      <c r="L396" s="20" t="n"/>
+    </row>
+    <row r="397">
+      <c r="L397" s="20" t="n"/>
+    </row>
+    <row r="398">
+      <c r="L398" s="20" t="n"/>
+    </row>
+    <row r="399">
+      <c r="L399" s="20" t="n"/>
+    </row>
+    <row r="400">
+      <c r="L400" s="20" t="n"/>
+    </row>
+    <row r="401">
+      <c r="L401" s="20" t="n"/>
+    </row>
+    <row r="402">
+      <c r="L402" s="20" t="n"/>
+    </row>
+    <row r="403">
+      <c r="L403" s="20" t="n"/>
+    </row>
+    <row r="404">
+      <c r="L404" s="20" t="n"/>
+    </row>
+    <row r="405">
+      <c r="L405" s="20" t="n"/>
+    </row>
+    <row r="406">
+      <c r="L406" s="20" t="n"/>
+    </row>
+    <row r="407">
+      <c r="L407" s="20" t="n"/>
+    </row>
+    <row r="408">
+      <c r="L408" s="20" t="n"/>
+    </row>
+    <row r="409">
+      <c r="L409" s="20" t="n"/>
+    </row>
+    <row r="410">
+      <c r="L410" s="20" t="n"/>
+    </row>
+    <row r="411">
+      <c r="L411" s="20" t="n"/>
+    </row>
+    <row r="412">
+      <c r="L412" s="20" t="n"/>
+    </row>
+    <row r="413">
+      <c r="L413" s="20" t="n"/>
+    </row>
+    <row r="414">
+      <c r="L414" s="20" t="n"/>
+    </row>
+    <row r="415">
+      <c r="L415" s="20" t="n"/>
+    </row>
+    <row r="416">
+      <c r="L416" s="20" t="n"/>
+    </row>
+    <row r="417">
+      <c r="L417" s="20" t="n"/>
+    </row>
+    <row r="418">
+      <c r="L418" s="20" t="n"/>
+    </row>
+    <row r="419">
+      <c r="L419" s="20" t="n"/>
+    </row>
+    <row r="420">
+      <c r="L420" s="20" t="n"/>
+    </row>
+    <row r="421">
+      <c r="L421" s="20" t="n"/>
+    </row>
+    <row r="422">
+      <c r="L422" s="20" t="n"/>
+    </row>
+    <row r="423">
+      <c r="L423" s="20" t="n"/>
+    </row>
+    <row r="424">
+      <c r="L424" s="20" t="n"/>
+    </row>
+    <row r="425">
+      <c r="L425" s="20" t="n"/>
+    </row>
+    <row r="426">
+      <c r="L426" s="20" t="n"/>
+    </row>
+    <row r="427">
+      <c r="L427" s="20" t="n"/>
+    </row>
+    <row r="428">
+      <c r="L428" s="20" t="n"/>
+    </row>
+    <row r="429">
+      <c r="L429" s="20" t="n"/>
+    </row>
+    <row r="430">
+      <c r="L430" s="20" t="n"/>
+    </row>
+    <row r="431">
+      <c r="L431" s="20" t="n"/>
+    </row>
+    <row r="432">
+      <c r="L432" s="20" t="n"/>
+    </row>
+    <row r="433">
+      <c r="L433" s="20" t="n"/>
+    </row>
+    <row r="434">
+      <c r="L434" s="20" t="n"/>
+    </row>
+    <row r="435">
+      <c r="L435" s="20" t="n"/>
+    </row>
+    <row r="436">
+      <c r="L436" s="20" t="n"/>
+    </row>
+    <row r="437">
+      <c r="L437" s="20" t="n"/>
+    </row>
+    <row r="438">
+      <c r="L438" s="20" t="n"/>
+    </row>
+    <row r="439">
+      <c r="L439" s="20" t="n"/>
+    </row>
+    <row r="440">
+      <c r="L440" s="20" t="n"/>
+    </row>
+    <row r="441">
+      <c r="L441" s="20" t="n"/>
+    </row>
+    <row r="442">
+      <c r="L442" s="20" t="n"/>
+    </row>
+    <row r="443">
+      <c r="L443" s="20" t="n"/>
+    </row>
+    <row r="444">
+      <c r="L444" s="20" t="n"/>
+    </row>
+    <row r="445">
+      <c r="L445" s="20" t="n"/>
+    </row>
+    <row r="446">
+      <c r="L446" s="20" t="n"/>
+    </row>
+    <row r="447">
+      <c r="L447" s="20" t="n"/>
+    </row>
+    <row r="448">
+      <c r="L448" s="20" t="n"/>
+    </row>
+    <row r="449">
+      <c r="L449" s="20" t="n"/>
+    </row>
+    <row r="450">
+      <c r="L450" s="20" t="n"/>
+    </row>
+    <row r="451">
+      <c r="L451" s="20" t="n"/>
+    </row>
+    <row r="452">
+      <c r="L452" s="20" t="n"/>
+    </row>
+    <row r="453">
+      <c r="L453" s="20" t="n"/>
+    </row>
+    <row r="454">
+      <c r="L454" s="20" t="n"/>
+    </row>
+    <row r="455">
+      <c r="L455" s="20" t="n"/>
+    </row>
+    <row r="456">
+      <c r="L456" s="20" t="n"/>
+    </row>
+    <row r="457">
+      <c r="L457" s="20" t="n"/>
+    </row>
+    <row r="458">
+      <c r="L458" s="20" t="n"/>
+    </row>
+    <row r="459">
+      <c r="L459" s="20" t="n"/>
+    </row>
+    <row r="460">
+      <c r="L460" s="20" t="n"/>
+    </row>
+    <row r="461">
+      <c r="L461" s="20" t="n"/>
+    </row>
+    <row r="462">
+      <c r="L462" s="20" t="n"/>
+    </row>
+    <row r="463">
+      <c r="L463" s="20" t="n"/>
+    </row>
+    <row r="464">
+      <c r="L464" s="20" t="n"/>
+    </row>
+    <row r="465">
+      <c r="L465" s="20" t="n"/>
+    </row>
+    <row r="466">
+      <c r="L466" s="20" t="n"/>
+    </row>
+    <row r="467">
+      <c r="L467" s="20" t="n"/>
+    </row>
+    <row r="468">
+      <c r="L468" s="20" t="n"/>
+    </row>
+    <row r="469">
+      <c r="L469" s="20" t="n"/>
+    </row>
+    <row r="470">
+      <c r="L470" s="20" t="n"/>
+    </row>
+    <row r="471">
+      <c r="L471" s="20" t="n"/>
+    </row>
+    <row r="472">
+      <c r="L472" s="20" t="n"/>
+    </row>
+    <row r="473">
+      <c r="L473" s="20" t="n"/>
+    </row>
+    <row r="474">
+      <c r="L474" s="20" t="n"/>
+    </row>
+    <row r="475">
+      <c r="L475" s="20" t="n"/>
+    </row>
+    <row r="476">
+      <c r="L476" s="20" t="n"/>
+    </row>
+    <row r="477">
+      <c r="L477" s="20" t="n"/>
+    </row>
+    <row r="478">
+      <c r="L478" s="20" t="n"/>
+    </row>
+    <row r="479">
+      <c r="L479" s="20" t="n"/>
+    </row>
+    <row r="480">
+      <c r="L480" s="20" t="n"/>
+    </row>
+    <row r="481">
+      <c r="L481" s="20" t="n"/>
+    </row>
+    <row r="482">
+      <c r="L482" s="20" t="n"/>
+    </row>
+    <row r="483">
+      <c r="L483" s="20" t="n"/>
+    </row>
+    <row r="484">
+      <c r="L484" s="20" t="n"/>
+    </row>
+    <row r="485">
+      <c r="L485" s="20" t="n"/>
+    </row>
+    <row r="486">
+      <c r="L486" s="20" t="n"/>
+    </row>
+    <row r="487">
+      <c r="L487" s="20" t="n"/>
+    </row>
+    <row r="488">
+      <c r="L488" s="20" t="n"/>
+    </row>
+    <row r="489">
+      <c r="L489" s="20" t="n"/>
+    </row>
+    <row r="490">
+      <c r="L490" s="20" t="n"/>
+    </row>
+    <row r="491">
+      <c r="L491" s="20" t="n"/>
+    </row>
+    <row r="492">
+      <c r="L492" s="20" t="n"/>
+    </row>
+    <row r="493">
+      <c r="L493" s="20" t="n"/>
+    </row>
+    <row r="494">
+      <c r="L494" s="20" t="n"/>
+    </row>
+    <row r="495">
+      <c r="L495" s="20" t="n"/>
+    </row>
+    <row r="496">
+      <c r="L496" s="20" t="n"/>
+    </row>
+    <row r="497">
+      <c r="L497" s="20" t="n"/>
+    </row>
+    <row r="498">
+      <c r="L498" s="20" t="n"/>
+    </row>
+    <row r="499">
+      <c r="L499" s="20" t="n"/>
+    </row>
+    <row r="500">
+      <c r="L500" s="20" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K17"/>
+  <autoFilter ref="A4:N500"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A2:N2"/>
   </mergeCells>
-  <dataValidations count="4">
-    <dataValidation sqref="H5:H67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <conditionalFormatting sqref="H5:H500">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$H5="Öneri"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>$H5="Açık"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>$H5="Devam ediyor"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>$H5="Test"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="4">
+      <formula>$H5="Tamamlandı"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="5">
+      <formula>$H5="İptal"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="6">
+    <dataValidation sqref="H5:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Öneri,Açık,Devam ediyor,Test,Tamamlandı,İptal"</formula1>
     </dataValidation>
-    <dataValidation sqref="F5:F67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yüksek,Orta,Düşük"</formula1>
     </dataValidation>
-    <dataValidation sqref="G5:G67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G5:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Faz 1,Faz 2"</formula1>
     </dataValidation>
-    <dataValidation sqref="B5:B67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"1 - Teknik: Veri Doğruluğu,2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm"</formula1>
+    <dataValidation sqref="B5:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 - Teknik: Veri Doğruluğu,2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm,3 - Genel / Diğer"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L5:L500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Tarih" error="Tarih girin (GG.AA.YYYY)" type="date" operator="greaterThan">
+      <formula1>DATE(2026,1,1)</formula1>
+    </dataValidation>
+    <dataValidation sqref="M5:M500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Tarih" error="Tarih girin (GG.AA.YYYY)" type="date" operator="greaterThan">
+      <formula1>DATE(2026,1,1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1197,7 +2834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1344,46 +2981,85 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>3 - Genel / Diğer</t>
+        </is>
+      </c>
+      <c r="B6" s="13">
+        <f>COUNTIFS('İş Listesi'!$B$5:$B$500,$A6,'İş Listesi'!$H$5:$H$500,B$3)</f>
+        <v/>
+      </c>
+      <c r="C6" s="13">
+        <f>COUNTIFS('İş Listesi'!$B$5:$B$500,$A6,'İş Listesi'!$H$5:$H$500,C$3)</f>
+        <v/>
+      </c>
+      <c r="D6" s="13">
+        <f>COUNTIFS('İş Listesi'!$B$5:$B$500,$A6,'İş Listesi'!$H$5:$H$500,D$3)</f>
+        <v/>
+      </c>
+      <c r="E6" s="13">
+        <f>COUNTIFS('İş Listesi'!$B$5:$B$500,$A6,'İş Listesi'!$H$5:$H$500,E$3)</f>
+        <v/>
+      </c>
+      <c r="F6" s="13">
+        <f>COUNTIFS('İş Listesi'!$B$5:$B$500,$A6,'İş Listesi'!$H$5:$H$500,F$3)</f>
+        <v/>
+      </c>
+      <c r="G6" s="13">
+        <f>COUNTIFS('İş Listesi'!$B$5:$B$500,$A6,'İş Listesi'!$H$5:$H$500,G$3)</f>
+        <v/>
+      </c>
+      <c r="H6" s="13">
+        <f>SUM(B6:G6)</f>
+        <v/>
+      </c>
+      <c r="I6" s="14">
+        <f>IF(H6-G6=0,0,F6/(H6-G6))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Toplam</t>
         </is>
       </c>
-      <c r="B6" s="16">
-        <f>SUM(B4:B5)</f>
-        <v/>
-      </c>
-      <c r="C6" s="16">
-        <f>SUM(C4:C5)</f>
-        <v/>
-      </c>
-      <c r="D6" s="16">
-        <f>SUM(D4:D5)</f>
-        <v/>
-      </c>
-      <c r="E6" s="16">
-        <f>SUM(E4:E5)</f>
-        <v/>
-      </c>
-      <c r="F6" s="16">
-        <f>SUM(F4:F5)</f>
-        <v/>
-      </c>
-      <c r="G6" s="16">
-        <f>SUM(G4:G5)</f>
-        <v/>
-      </c>
-      <c r="H6" s="16">
-        <f>SUM(H4:H5)</f>
-        <v/>
-      </c>
-      <c r="I6" s="17">
-        <f>IF(H6-G6=0,0,F6/(H6-G6))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="B7" s="16">
+        <f>SUM(B4:B6)</f>
+        <v/>
+      </c>
+      <c r="C7" s="16">
+        <f>SUM(C4:C6)</f>
+        <v/>
+      </c>
+      <c r="D7" s="16">
+        <f>SUM(D4:D6)</f>
+        <v/>
+      </c>
+      <c r="E7" s="16">
+        <f>SUM(E4:E6)</f>
+        <v/>
+      </c>
+      <c r="F7" s="16">
+        <f>SUM(F4:F6)</f>
+        <v/>
+      </c>
+      <c r="G7" s="16">
+        <f>SUM(G4:G6)</f>
+        <v/>
+      </c>
+      <c r="H7" s="16">
+        <f>SUM(H4:H6)</f>
+        <v/>
+      </c>
+      <c r="I7" s="17">
+        <f>IF(H7-G7=0,0,F7/(H7-G7))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Tamamlanma % = Tamamlandı / (Toplam − İptal)</t>
         </is>

</xml_diff>

<commit_message>
Sanal Kasa: Duygusal Denge Koçu (EI cash-out) — stres/anapara/zirveden düşüş/kazanç serisi sinyalleri, risk profili seçenekli kenara koyma, yol haritası, tabloda Kenarda sütunu (TR/EN/NL)
İş listesi #1 → Test; Cash-out Kuralları sayfası eklendi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="İş Listesi" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Özet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cash-out Kuralları" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'İş Listesi'!$A$4:$N$500</definedName>
@@ -23,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
     <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +62,16 @@
       <b val="1"/>
       <sz val="13"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -85,7 +96,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -107,11 +118,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -161,6 +216,24 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -741,17 +814,29 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Açık</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr"/>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Claude (Murat)</t>
+        </is>
+      </c>
       <c r="J5" s="8" t="inlineStr"/>
-      <c r="K5" s="7" t="inlineStr"/>
+      <c r="K5" s="21" t="inlineStr">
+        <is>
+          <t>Duygusal Denge Koçu olarak yapıldı; kurallar ve örnek yol haritası 'Cash-out Kuralları' sayfasında. Eşikler varsayımdır, kullanıcı testinden sonra ayarlanabilir.</t>
+        </is>
+      </c>
       <c r="L5" s="19" t="n">
         <v>46291</v>
       </c>
       <c r="M5" s="19" t="n"/>
-      <c r="N5" s="7" t="n"/>
+      <c r="N5" s="21" t="inlineStr">
+        <is>
+          <t>Sanal Kasa'ya Duygusal Denge Koçu: stres eşiği / anapara / zirveden düşüş / kazanç serisi sinyalleri, risk profili seçenekli cash-out, elle kenara koyma, geri alma, yol haritası; tablo+grafikte 'Kenarda' (js/paper_engine.js, js/paper_ui.js)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -3068,4 +3153,641 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sanal Kasa — Duygusal Denge Koçu (EI Cash-out) Kuralları</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="58" customHeight="1">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>Temel fikir: paranın insan üzerindeki etkisi kasanın yüzdesine değil, tek kuponda riske edilen MUTLAK tutara bağlıdır. Kişinin başlarken tamamını kaybetmeyi göze aldığı tutar (başlangıç kasası) 'konfor tutarı' kabul edilir. Koç her gün girilen gerçek kasaya bakar, öneri sunar; para hareketini kullanıcı onaylar (otomatik uygulamaz).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Öncelik</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Sinyal</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Tetikleme koşulu</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Önerilen aksiyon</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Davranışsal gerekçe</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Varsayılan değer</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>Zirveden düşüş</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>Toplam varlık, son cash-out'tan beri görülen zirvenin %30 altına indi (Minimum riskte değilken)</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>Risk bir kademe düşür, bugün mola ver (para kenara konmaz)</t>
+        </is>
+      </c>
+      <c r="E5" s="21" t="inlineStr">
+        <is>
+          <t>Kaybı kovalama / başa baş etkisi: kayıptan sonra risk artırma eğilimi</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="inlineStr">
+        <is>
+          <t>drawdownPct = %30</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Stres eşiği</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>Tek kupon riski ≥ 2 × konfor tutarı</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>Kasanın bir kısmını kenara koy + risk bir kademe düşür; tek kupon riski yeniden konfor tutarına iner. Her risk profili için ayrı seçenek gösterilir.</t>
+        </is>
+      </c>
+      <c r="E6" s="21" t="inlineStr">
+        <is>
+          <t>Kayıptan kaçınma: büyük mutlak kayıp, kazancın keyfinden ~2 kat daha güçlü hissedilir</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>stressMultiple = 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Anapara güvencesi</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>Henüz hiç kenara konmadı ve toplam varlık ≥ 2 × başlangıç kasası</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>Başlangıç parasını kenara koy (risk aynı veya bir kademe düşük)</t>
+        </is>
+      </c>
+      <c r="E7" s="21" t="inlineStr">
+        <is>
+          <t>Masada yalnızca kazanç kalır; en kötü günde bile kendi para güvende</t>
+        </is>
+      </c>
+      <c r="F7" s="21" t="inlineStr">
+        <is>
+          <t>principalMultiple = 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Kazanç serisi (heyecan)</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>3 gün üst üste büyüme ve bu sürede oyundaki kasa ≥ %50 arttı</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>Serinin kazancının yarısını kenara koy</t>
+        </is>
+      </c>
+      <c r="E8" s="21" t="inlineStr">
+        <is>
+          <t>'Kasa parası' etkisi: seri kazançta risk iştahı artar</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>streakDays = 3, streakGain = %50, streakSecure = %50</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Tanım</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Formül / değer</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>Tek kupon riski</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>Oyundaki kasa × (1 − Kasa Rezerv Oranı)  →  Minimum %25, Medium %50, High %50</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="n"/>
+      <c r="D11" s="24" t="n"/>
+      <c r="E11" s="24" t="n"/>
+      <c r="F11" s="25" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>Konfor tutarı</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>Başlangıç kasası + %25 × kenara konan toplam (kenara konan para güvence verdiği için konfor biraz büyür: alışma katsayısı = 0,25)</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="n"/>
+      <c r="D12" s="24" t="n"/>
+      <c r="E12" s="24" t="n"/>
+      <c r="F12" s="25" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>Stres seviyesi göstergesi</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>Sakin: risk ≤ 1,25 × konfor · Dikkat: 1,25–2 × konfor · Yüksek stres: ≥ 2 × konfor</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="n"/>
+      <c r="D13" s="24" t="n"/>
+      <c r="E13" s="24" t="n"/>
+      <c r="F13" s="25" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>Kenara konacak tutar (stres)</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>x = (f·W − S − 0,25·Kenarda) / (f + 0,25)  →  sonrasında f·(W−x) = konfor tutarı. 100 € üstü 10'luk yuvarlanır; kasanın %5'inden küçükse yalnızca risk değişir.</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="n"/>
+      <c r="D14" s="24" t="n"/>
+      <c r="E14" s="24" t="n"/>
+      <c r="F14" s="25" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>Hedef</t>
+        </is>
+      </c>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>Toplam varlık (oyundaki + kenarda) hedefe ulaşınca kasa tamamlanır. Cash-out günü yol haritası yeni risk faktörüyle o günden yeniden kurulur: Hedef(gün) = Kenarda + W·(1+g)^(gün−d)</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="n"/>
+      <c r="D15" s="24" t="n"/>
+      <c r="E15" s="24" t="n"/>
+      <c r="F15" s="25" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>Tekrar önerme</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>Aynı gün cash-out yapıldıysa o gün yeni öneri yok. "Şimdilik devam et" o günün önerisini gizler; ertesi gün yeniden değerlendirilir. Son cash-out geri alınabilir.</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="n"/>
+      <c r="D16" s="24" t="n"/>
+      <c r="E16" s="24" t="n"/>
+      <c r="F16" s="25" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="26" t="inlineStr">
+        <is>
+          <t>Örnek yol haritası: 100 € → 5.000 € (her gün teorik büyüme gerçekleşirse, önerilen seçenek uygulanarak)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Risk profili</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Koçsuz: hedefe gün</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Koçsuz: en yüksek tek kupon (€)</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Koçla: hedefe gün</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Koçla: en yüksek tek kupon (€)</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Koçla: seviye sayısı</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="n">
+        <v>18</v>
+      </c>
+      <c r="C20" s="27" t="n">
+        <v>2220</v>
+      </c>
+      <c r="D20" s="21" t="n">
+        <v>39</v>
+      </c>
+      <c r="E20" s="27" t="n">
+        <v>805</v>
+      </c>
+      <c r="F20" s="21" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="n">
+        <v>28</v>
+      </c>
+      <c r="C21" s="27" t="n">
+        <v>2177</v>
+      </c>
+      <c r="D21" s="21" t="n">
+        <v>47</v>
+      </c>
+      <c r="E21" s="27" t="n">
+        <v>855</v>
+      </c>
+      <c r="F21" s="21" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Minimum</t>
+        </is>
+      </c>
+      <c r="B22" s="21" t="n">
+        <v>42</v>
+      </c>
+      <c r="C22" s="27" t="n">
+        <v>1245</v>
+      </c>
+      <c r="D22" s="21" t="n">
+        <v>54</v>
+      </c>
+      <c r="E22" s="27" t="n">
+        <v>841</v>
+      </c>
+      <c r="F22" s="21" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>Kaynak: js/paper_engine.js buildEIRoadmap, 2026-09-26. Koçla hedefe ulaşmak daha uzun sürer ama tek kuponda riske edilen en yüksek tutar ~%60-65 düşer ve hedefe varırken paranın bir kısmı zaten güvendedir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>Detay: High risk, 100 € → 5.000 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Gün</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Tetikleyici</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Toplam varlık (€)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Kenara (€) / Kenarda toplam (€)</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Tek kupon riski (€): önce → sonra</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B27" s="21" t="inlineStr">
+        <is>
+          <t>Anapara güvencesi</t>
+        </is>
+      </c>
+      <c r="C27" s="27" t="n">
+        <v>244</v>
+      </c>
+      <c r="D27" s="21" t="inlineStr">
+        <is>
+          <t>100 / 100</t>
+        </is>
+      </c>
+      <c r="E27" s="21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="inlineStr">
+        <is>
+          <t>122 → 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="B28" s="21" t="inlineStr">
+        <is>
+          <t>Stres eşiği</t>
+        </is>
+      </c>
+      <c r="C28" s="27" t="n">
+        <v>650</v>
+      </c>
+      <c r="D28" s="21" t="inlineStr">
+        <is>
+          <t>190 / 290</t>
+        </is>
+      </c>
+      <c r="E28" s="21" t="inlineStr">
+        <is>
+          <t>High → Medium</t>
+        </is>
+      </c>
+      <c r="F28" s="21" t="inlineStr">
+        <is>
+          <t>275 → 180</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="21" t="n">
+        <v>15</v>
+      </c>
+      <c r="B29" s="21" t="inlineStr">
+        <is>
+          <t>Stres eşiği</t>
+        </is>
+      </c>
+      <c r="C29" s="27" t="n">
+        <v>1014</v>
+      </c>
+      <c r="D29" s="21" t="inlineStr">
+        <is>
+          <t>0 / 290</t>
+        </is>
+      </c>
+      <c r="E29" s="21" t="inlineStr">
+        <is>
+          <t>Medium → Minimum</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="inlineStr">
+        <is>
+          <t>362 → 181</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="n">
+        <v>22</v>
+      </c>
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>Stres eşiği</t>
+        </is>
+      </c>
+      <c r="C30" s="27" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>360 / 650</t>
+        </is>
+      </c>
+      <c r="E30" s="21" t="inlineStr">
+        <is>
+          <t>Minimum</t>
+        </is>
+      </c>
+      <c r="F30" s="21" t="inlineStr">
+        <is>
+          <t>353 → 263</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="21" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>Stres eşiği</t>
+        </is>
+      </c>
+      <c r="C31" s="27" t="n">
+        <v>2902</v>
+      </c>
+      <c r="D31" s="21" t="inlineStr">
+        <is>
+          <t>600 / 1.250</t>
+        </is>
+      </c>
+      <c r="E31" s="21" t="inlineStr">
+        <is>
+          <t>Minimum</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="inlineStr">
+        <is>
+          <t>563 → 413</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="21" t="n">
+        <v>38</v>
+      </c>
+      <c r="B32" s="21" t="inlineStr">
+        <is>
+          <t>Stres eşiği</t>
+        </is>
+      </c>
+      <c r="C32" s="27" t="n">
+        <v>4791</v>
+      </c>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>940 / 2.190</t>
+        </is>
+      </c>
+      <c r="E32" s="21" t="inlineStr">
+        <is>
+          <t>Minimum</t>
+        </is>
+      </c>
+      <c r="F32" s="21" t="inlineStr">
+        <is>
+          <t>885 → 650</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="28" t="inlineStr">
+        <is>
+          <t>Kullanıcının örneği (koçu dinlemeden 1.000 €'ya gelmiş, High): tek kupon 500 € = konforun 5 katı → seçenekler: 530 € kenara + High (11 gün), 530 € kenara + Medium (önerilen, 17 gün), 300 € kenara + Minimum (20 gün).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B13:F13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Sanal Kasa: güven payı kazanç eğrisi ve hedef dışında; Güven Payı İşlemleri (kenara koy / kasaya geri al); Tab/Enter ile sonraki güne geçiş; girişte sayfa kaymıyor
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -834,7 +834,7 @@
       <c r="M5" s="19" t="n"/>
       <c r="N5" s="21" t="inlineStr">
         <is>
-          <t>d8d4301 — Sanal Kasa'ya Duygusal Denge Koçu: stres eşiği / anapara / zirveden düşüş / kazanç serisi sinyalleri, risk profili seçenekli cash-out, elle kenara koyma, geri alma, yol haritası; tablo+grafikte 'Kenarda' (js/paper_engine.js, js/paper_ui.js)</t>
+          <t>d8d4301 — Sanal Kasa'ya Duygusal Denge Koçu: stres eşiği / anapara / zirveden düşüş / kazanç serisi sinyalleri, risk profili seçenekli cash-out, elle kenara koyma, geri alma, yol haritası; tablo+grafikte 'Kenarda' (js/paper_engine.js, js/paper_ui.js). Sonraki commit: güven payı kazanç eğrisi/hedef dışında; Güven Payı İşlemleri (kenara koy / kasaya geri al); Tab/Enter ile sonraki gün; girişte sayfa kaymıyor.</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3229,7 +3229,7 @@
       </c>
       <c r="C5" s="21" t="inlineStr">
         <is>
-          <t>Toplam varlık, son cash-out'tan beri görülen zirvenin %30 altına indi (Minimum riskte değilken)</t>
+          <t>Oyundaki kasa, son cash-out'tan beri görülen zirvesinin %30 altına indi (Minimum riskte değilken)</t>
         </is>
       </c>
       <c r="D5" s="21" t="inlineStr">
@@ -3289,7 +3289,7 @@
       </c>
       <c r="C7" s="21" t="inlineStr">
         <is>
-          <t>Henüz hiç kenara konmadı ve toplam varlık ≥ 2 × başlangıç kasası</t>
+          <t>Henüz hiç kenara konmadı ve oyundaki kasa ≥ 2 × başlangıç kasası</t>
         </is>
       </c>
       <c r="D7" s="21" t="inlineStr">
@@ -3421,12 +3421,12 @@
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
         <is>
-          <t>Hedef</t>
+          <t>Güven payı ve hedef</t>
         </is>
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>Toplam varlık (oyundaki + kenarda) hedefe ulaşınca kasa tamamlanır. Cash-out günü yol haritası yeni risk faktörüyle o günden yeniden kurulur: Hedef(gün) = Kenarda + W·(1+g)^(gün−d)</t>
+          <t>Kenara konan para kişinin güven payıdır: kazanç eğrisine, büyüme yüzdelerine ve hedefe dahil edilmez (grafikte mavi sütunun üstünde yeşil olarak ayrıca gösterilir). Hedef, OYUNDAKİ kasanın hedef kasaya ulaşmasıdır. Cash-out günü yol haritası kalan oyundaki kasa ve yeni risk faktörüyle o günden yeniden kurulur: Hedef(gün) = W·(1+g)^(gün−d)</t>
         </is>
       </c>
       <c r="C15" s="24" t="n"/>
@@ -3442,7 +3442,7 @@
       </c>
       <c r="B16" s="21" t="inlineStr">
         <is>
-          <t>Aynı gün cash-out yapıldıysa o gün yeni öneri yok. "Şimdilik devam et" o günün önerisini gizler; ertesi gün yeniden değerlendirilir. Son cash-out geri alınabilir.</t>
+          <t>Aynı gün kenara koyma/geri alma yapıldıysa o gün yeni öneri yok. "Şimdilik devam et" o günün önerisini gizler; ertesi gün yeniden değerlendirilir. Kullanıcı istediği zaman Güven Payı İşlemleri ile kenara koyabilir veya güven payından kasaya geri alabilir; son işlem geri alınabilir.</t>
         </is>
       </c>
       <c r="C16" s="24" t="n"/>
@@ -3502,10 +3502,10 @@
         <v>2220</v>
       </c>
       <c r="D20" s="21" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E20" s="27" t="n">
-        <v>805</v>
+        <v>1152</v>
       </c>
       <c r="F20" s="21" t="n">
         <v>6</v>
@@ -3524,13 +3524,13 @@
         <v>2177</v>
       </c>
       <c r="D21" s="21" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="E21" s="27" t="n">
-        <v>855</v>
+        <v>1223</v>
       </c>
       <c r="F21" s="21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
@@ -3546,10 +3546,10 @@
         <v>1245</v>
       </c>
       <c r="D22" s="21" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="E22" s="27" t="n">
-        <v>841</v>
+        <v>1200</v>
       </c>
       <c r="F22" s="21" t="n">
         <v>4</v>
@@ -3558,7 +3558,7 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="28" t="inlineStr">
         <is>
-          <t>Kaynak: js/paper_engine.js buildEIRoadmap, 2026-09-26. Koçla hedefe ulaşmak daha uzun sürer ama tek kuponda riske edilen en yüksek tutar ~%60-65 düşer ve hedefe varırken paranın bir kısmı zaten güvendedir.</t>
+          <t>Kaynak: js/paper_engine.js buildEIRoadmap, 2026-09-26. Koçla hedefe ulaşmak daha uzun sürer; High/Medium'da tek kuponda riske edilen en yüksek tutar ~%45 düşer ve hedefe varıldığında ayrıca 2.000 €'yu aşan bir güven payı birikmiş olur (güven payı hedefe sayılmaz).</t>
         </is>
       </c>
     </row>
@@ -3582,12 +3582,12 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Toplam varlık (€)</t>
+          <t>Oyundaki kasa (€)</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Kenara (€) / Kenarda toplam (€)</t>
+          <t>Kenara (€) / Güven payı toplam (€)</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -3639,7 +3639,7 @@
         </is>
       </c>
       <c r="C28" s="27" t="n">
-        <v>650</v>
+        <v>550</v>
       </c>
       <c r="D28" s="21" t="inlineStr">
         <is>
@@ -3667,7 +3667,7 @@
         </is>
       </c>
       <c r="C29" s="27" t="n">
-        <v>1014</v>
+        <v>724</v>
       </c>
       <c r="D29" s="21" t="inlineStr">
         <is>
@@ -3695,7 +3695,7 @@
         </is>
       </c>
       <c r="C30" s="27" t="n">
-        <v>1700</v>
+        <v>1410</v>
       </c>
       <c r="D30" s="21" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="C31" s="27" t="n">
-        <v>2902</v>
+        <v>2252</v>
       </c>
       <c r="D31" s="21" t="inlineStr">
         <is>
@@ -3751,7 +3751,7 @@
         </is>
       </c>
       <c r="C32" s="27" t="n">
-        <v>4791</v>
+        <v>3541</v>
       </c>
       <c r="D32" s="21" t="inlineStr">
         <is>
@@ -3769,22 +3769,50 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="28" t="inlineStr">
-        <is>
-          <t>Kullanıcının örneği (koçu dinlemeden 1.000 €'ya gelmiş, High): tek kupon 500 € = konforun 5 katı → seçenekler: 530 € kenara + High (11 gün), 530 € kenara + Medium (önerilen, 17 gün), 300 € kenara + Minimum (20 gün).</t>
+    <row r="33">
+      <c r="A33" s="21" t="n">
+        <v>45</v>
+      </c>
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>Hedef</t>
+        </is>
+      </c>
+      <c r="C33" s="27" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D33" s="21" t="inlineStr">
+        <is>
+          <t>— / 2.190</t>
+        </is>
+      </c>
+      <c r="E33" s="21" t="inlineStr">
+        <is>
+          <t>Minimum</t>
+        </is>
+      </c>
+      <c r="F33" s="21" t="inlineStr">
+        <is>
+          <t>oyundaki kasa 5.000 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="28" t="inlineStr">
+        <is>
+          <t>Kullanıcının örneği (koçu dinlemeden 1.000 €'ya gelmiş, High): tek kupon 500 € = konforun 5 katı → seçenekler: 530 € kenara + High (11 gün), 530 € kenara + Medium (önerilen, 17 gün), 300 € kenara + Minimum (21 gün).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A33:F33"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A34:F34"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B13:F13"/>
   </mergeCells>

</xml_diff>

<commit_message>
Sanal Kasa: Güven Payı sadeleştirildi — tek kural (kupon > rahat sınır → tek butonla kilitle), kilitli para hedefe sayılır, duraklı yol çizgisi, rahat sınır alanı; kapatılan kasayı yeniden aç / sil
İş listesi: #1 güncellendi, #14 (kapatılan kasa yeniden aç/sil) ve #15 (NL menü taşması, öneri) eklendi; Güven Payı Kuralları sayfası.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="İş Listesi" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Özet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Cash-out Kuralları" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Güven Payı Kuralları" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'İş Listesi'!$A$4:$N$500</definedName>
@@ -24,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
     <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +71,17 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -166,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -233,6 +244,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -825,7 +842,7 @@
       <c r="J5" s="8" t="inlineStr"/>
       <c r="K5" s="21" t="inlineStr">
         <is>
-          <t>Duygusal Denge Koçu olarak yapıldı; kurallar ve örnek yol haritası 'Cash-out Kuralları' sayfasında. Eşikler varsayımdır, kullanıcı testinden sonra ayarlanabilir.</t>
+          <t>Sadeleştirildi (2026-09-26): tek kural (bugünkü kupon &gt; rahat sınır → tek butonla kilitle), kilitli para hedefe sayılır, duraklı yol çizgisi. Kurallar 'Güven Payı Kuralları' sayfasında.</t>
         </is>
       </c>
       <c r="L5" s="19" t="n">
@@ -834,7 +851,7 @@
       <c r="M5" s="19" t="n"/>
       <c r="N5" s="21" t="inlineStr">
         <is>
-          <t>d8d4301 — Sanal Kasa'ya Duygusal Denge Koçu: stres eşiği / anapara / zirveden düşüş / kazanç serisi sinyalleri, risk profili seçenekli cash-out, elle kenara koyma, geri alma, yol haritası; tablo+grafikte 'Kenarda' (js/paper_engine.js, js/paper_ui.js). a6b9224 — güven payı kazanç eğrisi/hedef dışında; Güven Payı İşlemleri (kenara koy / kasaya geri al); Tab/Enter ile sonraki gün; girişte sayfa kaymıyor.</t>
+          <t>d8d4301 — Sanal Kasa'ya Duygusal Denge Koçu: stres eşiği / anapara / zirveden düşüş / kazanç serisi sinyalleri, risk profili seçenekli cash-out, elle kenara koyma, geri alma, yol haritası; tablo+grafikte 'Kenarda' (js/paper_engine.js, js/paper_ui.js). a6b9224 — güven payı kazanç eğrisi/hedef dışında; Güven Payı İşlemleri (kenara koy / kasaya geri al); Tab/Enter ile sonraki gün; girişte sayfa kaymıyor. Sadeleştirme: Güven Payı kartı (tek sayı + tek buton + yol çizgisi), rahat sınır alanı, Oyundaki/Kilitli sütunları.</t>
         </is>
       </c>
     </row>
@@ -1415,10 +1432,108 @@
       <c r="N17" s="7" t="n"/>
     </row>
     <row r="18">
-      <c r="L18" s="20" t="n"/>
+      <c r="A18" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Kapatılan kasayı yeniden aç / sil</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Yanlışlıkla oluşturulan veya hatalı girilen kasalar için Kapatılan Kasalar listesinde "Yeniden aç" (düzeltip tekrar kapatma) ve "Sil" butonları; senkronizasyonda silinen kasa geri gelmez.</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Murat</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>Claude (Murat)</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="n"/>
+      <c r="K18" s="7" t="n"/>
+      <c r="L18" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M18" s="19" t="n"/>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>Güven Payı sadeleştirmesiyle aynı commit (js/paper_engine.js reopenClosedPlan/deleteClosedPlan, js/auth_sync.js)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="L19" s="20" t="n"/>
+      <c r="A19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>NL dilinde üst menü taşması</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Hollandaca seçiliyken 1280 px genişlikte üst menüdeki hesap butonu sayfayı ~80 px yatay taşırıyor (tüm sekmelerde). Test sırasında bulundu.</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Öneri (Claude - test sırasında)</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Düşük</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="n"/>
+      <c r="J19" s="8" t="n"/>
+      <c r="K19" s="7" t="n"/>
+      <c r="L19" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M19" s="19" t="n"/>
+      <c r="N19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="L20" s="20" t="n"/>
@@ -3161,660 +3276,539 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sanal Kasa — Duygusal Denge Koçu (EI Cash-out) Kuralları</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="58" customHeight="1">
-      <c r="A2" s="22" t="inlineStr">
-        <is>
-          <t>Temel fikir: paranın insan üzerindeki etkisi kasanın yüzdesine değil, tek kuponda riske edilen MUTLAK tutara bağlıdır. Kişinin başlarken tamamını kaybetmeyi göze aldığı tutar (başlangıç kasası) 'konfor tutarı' kabul edilir. Koç her gün girilen gerçek kasaya bakar, öneri sunar; para hareketini kullanıcı onaylar (otomatik uygulamaz).</t>
+          <t>Sanal Kasa — Güven Payı Kuralları</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="29" t="inlineStr">
+        <is>
+          <t>Sitedeki cümle: "Kasan büyüdükçe bir kısmını kilitle. Kilitlediğin para bir daha riske girmez ama hedefine sayılır." Kullanıcı tek bir sayıya (bugünkü kupon ile rahat sınır) bakar ve tek bir butona basar. Para hareketini her zaman kullanıcı onaylar.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Öncelik</t>
+          <t>Kural</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Sinyal</t>
+          <t>Ne zaman</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Tetikleme koşulu</t>
+          <t>Ne olur</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Önerilen aksiyon</t>
+          <t>Psikolojik gerekçe</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Davranışsal gerekçe</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Varsayılan değer</t>
-        </is>
-      </c>
+          <t>Değer</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="n">
-        <v>1</v>
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>Rahat sınır</t>
+        </is>
       </c>
       <c r="B5" s="21" t="inlineStr">
         <is>
-          <t>Zirveden düşüş</t>
+          <t>Kasa açılırken sorulur: "Tek kupona en fazla ne kadar koymak seni rahatsız etmez?" Boş = başlangıç kasası.</t>
         </is>
       </c>
       <c r="C5" s="21" t="inlineStr">
         <is>
-          <t>Oyundaki kasa, son cash-out'tan beri görülen zirvesinin %30 altına indi (Minimum riskte değilken)</t>
+          <t>Kupon, bu sınırla karşılaştırılır. Sınır = seçilen tutar + kilitli para.</t>
         </is>
       </c>
       <c r="D5" s="21" t="inlineStr">
         <is>
-          <t>Risk bir kademe düşür, bugün mola ver (para kenara konmaz)</t>
+          <t>Stres kişiye özeldir; tahmin etmek yerine kişiye sormak en dürüst yol. Kilitli para güvende olduğu için kişi alışır, sınır onunla büyür.</t>
         </is>
       </c>
       <c r="E5" s="21" t="inlineStr">
         <is>
-          <t>Kaybı kovalama / başa baş etkisi: kayıptan sonra risk artırma eğilimi</t>
-        </is>
-      </c>
-      <c r="F5" s="21" t="inlineStr">
+          <t>limitGrowth = 1,0</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>Işık</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Her gün kasa girildiğinde</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>🟢 kupon ≤ %75 sınır · 🟡 %75–100 · 🔴 sınırı geçti</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>Tek bakışta anlaşılır; "konfor tutarının 2,5 katı" gibi hesap yok.</t>
+        </is>
+      </c>
+      <c r="E6" s="21" t="inlineStr">
+        <is>
+          <t>watchRatio = %75</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>Kilitle (tek kural)</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Bugünkü kupon &gt; rahat sınır</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>Tek buton: "🔒 X € kilitle". Kupon, sınırın dörtte birine iner. İsteğe bağlı: riski bir kademe düşür.</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>Kayıptan kaçınma: kaybın acısı kazancın keyfinden ~2 kat güçlü. Kuponu belirgin biçimde (4 kat) küçültmek bir sonraki durağa kadar rahat bir alan bırakır.</t>
+        </is>
+      </c>
+      <c r="E7" s="21" t="inlineStr">
+        <is>
+          <t>resetRatio = 0,25</t>
+        </is>
+      </c>
+      <c r="F7" s="21" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>Mola uyarısı</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Oyundaki kasa son kilitlemeden beri zirvesinin %30 altına indiğinde</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>Sadece mesaj: "Bugün mola vermeyi düşün". Para hareketi önerilmez.</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>Kaybı kovalama: kayıptan sonra risk artırma eğilimi en pahalı hatadır.</t>
+        </is>
+      </c>
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>drawdownPct = %30</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>Stres eşiği</t>
-        </is>
-      </c>
-      <c r="C6" s="21" t="inlineStr">
-        <is>
-          <t>Tek kupon riski ≥ 2 × konfor tutarı</t>
-        </is>
-      </c>
-      <c r="D6" s="21" t="inlineStr">
-        <is>
-          <t>Kasanın bir kısmını kenara koy + risk bir kademe düşür; tek kupon riski yeniden konfor tutarına iner. Her risk profili için ayrı seçenek gösterilir.</t>
-        </is>
-      </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>Kayıptan kaçınma: büyük mutlak kayıp, kazancın keyfinden ~2 kat daha güçlü hissedilir</t>
-        </is>
-      </c>
-      <c r="F6" s="21" t="inlineStr">
-        <is>
-          <t>stressMultiple = 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>Anapara güvencesi</t>
-        </is>
-      </c>
-      <c r="C7" s="21" t="inlineStr">
-        <is>
-          <t>Henüz hiç kenara konmadı ve oyundaki kasa ≥ 2 × başlangıç kasası</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr">
-        <is>
-          <t>Başlangıç parasını kenara koy (risk aynı veya bir kademe düşük)</t>
-        </is>
-      </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
-          <t>Masada yalnızca kazanç kalır; en kötü günde bile kendi para güvende</t>
-        </is>
-      </c>
-      <c r="F7" s="21" t="inlineStr">
-        <is>
-          <t>principalMultiple = 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="21" t="inlineStr">
-        <is>
-          <t>Kazanç serisi (heyecan)</t>
-        </is>
-      </c>
-      <c r="C8" s="21" t="inlineStr">
-        <is>
-          <t>3 gün üst üste büyüme ve bu sürede oyundaki kasa ≥ %50 arttı</t>
-        </is>
-      </c>
-      <c r="D8" s="21" t="inlineStr">
-        <is>
-          <t>Serinin kazancının yarısını kenara koy</t>
-        </is>
-      </c>
-      <c r="E8" s="21" t="inlineStr">
-        <is>
-          <t>'Kasa parası' etkisi: seri kazançta risk iştahı artar</t>
-        </is>
-      </c>
-      <c r="F8" s="21" t="inlineStr">
-        <is>
-          <t>streakDays = 3, streakGain = %50, streakSecure = %50</t>
-        </is>
-      </c>
+      <c r="F8" s="21" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>Hedef</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Her zaman</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>Hedef ve toplam büyüme = oyundaki + kilitli. Günlük değişim = oyundaki kasa. Grafik: mavi oyundaki + üstünde yeşil kilitli, yanında kırmızı hedef.</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>Kilitli para hedefe sayılmazsa kilitlemek cezalandırılmış olur ve kişi kilitlemekten kaçınır; sayılırsa ödül gibi hissedilir.</t>
+        </is>
+      </c>
+      <c r="E9" s="21" t="inlineStr"/>
+      <c r="F9" s="21" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Tanım</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Formül / değer</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr"/>
-      <c r="D10" s="3" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="3" t="inlineStr"/>
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>Yol çizgisi</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Her zaman</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>Başlangıçtan hedefe tek çizgi, üzerinde 🔒 durakları ve "Sıradaki durak: kasa ~X € olunca Y € kilitle".</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>Durakları baştan görmek sürprizi ve anlık heyecanla karar vermeyi azaltır. Çizgi logaritmiktir: 50→100 € ile 1.000→2.000 € aynı adım gibi hissedilir (Weber-Fechner).</t>
+        </is>
+      </c>
+      <c r="E10" s="21" t="inlineStr"/>
+      <c r="F10" s="21" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
         <is>
-          <t>Tek kupon riski</t>
+          <t>Kullanıcı kontrolü</t>
         </is>
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>Oyundaki kasa × (1 − Kasa Rezerv Oranı)  →  Minimum %25, Medium %50, High %50</t>
-        </is>
-      </c>
-      <c r="C11" s="24" t="n"/>
-      <c r="D11" s="24" t="n"/>
-      <c r="E11" s="24" t="n"/>
-      <c r="F11" s="25" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="23" t="inlineStr">
-        <is>
-          <t>Konfor tutarı</t>
-        </is>
-      </c>
-      <c r="B12" s="21" t="inlineStr">
-        <is>
-          <t>Başlangıç kasası + %25 × kenara konan toplam (kenara konan para güvence verdiği için konfor biraz büyür: alışma katsayısı = 0,25)</t>
-        </is>
-      </c>
-      <c r="C12" s="24" t="n"/>
-      <c r="D12" s="24" t="n"/>
-      <c r="E12" s="24" t="n"/>
-      <c r="F12" s="25" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="23" t="inlineStr">
-        <is>
-          <t>Stres seviyesi göstergesi</t>
-        </is>
-      </c>
-      <c r="B13" s="21" t="inlineStr">
-        <is>
-          <t>Sakin: risk ≤ 1,25 × konfor · Dikkat: 1,25–2 × konfor · Yüksek stres: ≥ 2 × konfor</t>
-        </is>
-      </c>
-      <c r="C13" s="24" t="n"/>
-      <c r="D13" s="24" t="n"/>
-      <c r="E13" s="24" t="n"/>
-      <c r="F13" s="25" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="23" t="inlineStr">
-        <is>
-          <t>Kenara konacak tutar (stres)</t>
-        </is>
-      </c>
-      <c r="B14" s="21" t="inlineStr">
-        <is>
-          <t>x = (f·W − S − 0,25·Kenarda) / (f + 0,25)  →  sonrasında f·(W−x) = konfor tutarı. 100 € üstü 10'luk yuvarlanır; kasanın %5'inden küçükse yalnızca risk değişir.</t>
-        </is>
-      </c>
-      <c r="C14" s="24" t="n"/>
-      <c r="D14" s="24" t="n"/>
-      <c r="E14" s="24" t="n"/>
-      <c r="F14" s="25" t="n"/>
+          <t>Her zaman</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
+          <t>Kilitle / Geri al (tutar sorulur) / Son işlemi geri al. Aynı gün işlem yapıldıysa o gün yeni öneri çıkmaz.</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
+        <is>
+          <t>Kontrol kişide kalır; sistem sadece önerir.</t>
+        </is>
+      </c>
+      <c r="E11" s="21" t="inlineStr"/>
+      <c r="F11" s="21" t="inlineStr"/>
+    </row>
+    <row r="13" ht="44" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Kilitleme tutarı: x = (f·W − r·L0 − r·a·Kilitli) / (f + r·a) → sonrasında kupon f·(W−x) = r·(L0 + a·(Kilitli+x)). f = oynanan pay (Minimum %25, Medium/High %50), W = oyundaki kasa, L0 = seçilen rahat sınır, r = 0,25, a = 1,0. 100 € üstü 10'luk aşağı yuvarlanır.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
-        <is>
-          <t>Güven payı ve hedef</t>
-        </is>
-      </c>
-      <c r="B15" s="21" t="inlineStr">
-        <is>
-          <t>Kenara konan para kişinin güven payıdır: kazanç eğrisine, büyüme yüzdelerine ve hedefe dahil edilmez (grafikte mavi sütunun üstünde yeşil olarak ayrıca gösterilir). Hedef, OYUNDAKİ kasanın hedef kasaya ulaşmasıdır. Cash-out günü yol haritası kalan oyundaki kasa ve yeni risk faktörüyle o günden yeniden kurulur: Hedef(gün) = W·(1+g)^(gün−d)</t>
-        </is>
-      </c>
-      <c r="C15" s="24" t="n"/>
-      <c r="D15" s="24" t="n"/>
-      <c r="E15" s="24" t="n"/>
-      <c r="F15" s="25" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="23" t="inlineStr">
-        <is>
-          <t>Tekrar önerme</t>
-        </is>
-      </c>
-      <c r="B16" s="21" t="inlineStr">
-        <is>
-          <t>Aynı gün kenara koyma/geri alma yapıldıysa o gün yeni öneri yok. "Şimdilik devam et" o günün önerisini gizler; ertesi gün yeniden değerlendirilir. Kullanıcı istediği zaman Güven Payı İşlemleri ile kenara koyabilir veya güven payından kasaya geri alabilir; son işlem geri alınabilir.</t>
-        </is>
-      </c>
-      <c r="C16" s="24" t="n"/>
-      <c r="D16" s="24" t="n"/>
-      <c r="E16" s="24" t="n"/>
-      <c r="F16" s="25" t="n"/>
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>Durak sayısı nasıl belirleniyor?</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="72" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>Durak sayısı sabit bir hedef değil; kuponun rahat sınırı geçtiği her an bir durak oluşur. Bu kurala göre duraklar kasanın her ~2,3 katına çıkışında gelir, yani para algısı açısından eşit aralıklıdır. Yolculuk ne kadar uzunsa (hedef/başlangıç oranı) o kadar durak çıkar: 20 kat → 2–3, 50 kat → 3–5, 200 kat → 4–6. Bu, kişiyi her gün rahatsız etmeden (en sık haftada bir) ama kupon büyüdükçe mutlaka durduracak bir sıklıktır. High riskte kasa hızlı büyüdüğü için duraklar daha sık gelir; hızlı yükselişin heyecanı da daha erken dengelenmiş olur. İlk durak çoğu planda kendiliğinden "anaparanı kilitle" olur (ör. 100 €'da 50 €).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="26" t="inlineStr">
-        <is>
-          <t>Örnek yol haritası: 100 € → 5.000 € (her gün teorik büyüme gerçekleşirse, önerilen seçenek uygulanarak)</t>
-        </is>
-      </c>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Plan (başlangıç → hedef, risk)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Koçsuz: hedefe gün / en yüksek kupon</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Güven Payı ile: hedefe gün / en yüksek kupon</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Durak sayısı</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Duraklar (toplam kasa → kilitlenen)</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Risk profili</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Koçsuz: hedefe gün</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Koçsuz: en yüksek tek kupon (€)</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Koçla: hedefe gün</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>Koçla: en yüksek tek kupon (€)</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Koçla: seviye sayısı</t>
-        </is>
-      </c>
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>50 → 10.000 €, Minimum</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>56 gün / 2.363 €</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="inlineStr">
+        <is>
+          <t>73 gün / 1.795 €</t>
+        </is>
+      </c>
+      <c r="D19" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
+          <t>209 → 79 · 621 → 200 · 1.710 → 550 · 4.507 → 1.390</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="21" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="B20" s="21" t="n">
-        <v>18</v>
-      </c>
-      <c r="C20" s="27" t="n">
-        <v>2220</v>
+          <t>50 → 10.000 €, Medium</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>38 gün / 4.403 €</t>
+        </is>
+      </c>
+      <c r="C20" s="21" t="inlineStr">
+        <is>
+          <t>65 gün / 3.078 €</t>
+        </is>
       </c>
       <c r="D20" s="21" t="n">
-        <v>45</v>
-      </c>
-      <c r="E20" s="27" t="n">
-        <v>1152</v>
-      </c>
-      <c r="F20" s="21" t="n">
         <v>6</v>
       </c>
+      <c r="E20" s="21" t="inlineStr">
+        <is>
+          <t>101 → 50 · 255 → 100 · 573 → 210 · 1.222 → 430 · 2.538 → 880 · 5.180 → 1.760</t>
+        </is>
+      </c>
+      <c r="F20" s="21" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="21" t="inlineStr">
         <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="B21" s="21" t="n">
-        <v>28</v>
-      </c>
-      <c r="C21" s="27" t="n">
-        <v>2177</v>
+          <t>50 → 10.000 €, High</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>24 gün / 4.235 €</t>
+        </is>
+      </c>
+      <c r="C21" s="21" t="inlineStr">
+        <is>
+          <t>40 gün / 2.547 €</t>
+        </is>
       </c>
       <c r="D21" s="21" t="n">
-        <v>54</v>
-      </c>
-      <c r="E21" s="27" t="n">
-        <v>1223</v>
-      </c>
-      <c r="F21" s="21" t="n">
         <v>6</v>
       </c>
+      <c r="E21" s="21" t="inlineStr">
+        <is>
+          <t>122 → 64 · 341 → 140 · 726 → 260 · 1.714 → 660 · 3.939 → 1.480 · 8.972 → 3.360</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="21" t="inlineStr">
         <is>
-          <t>Minimum</t>
-        </is>
-      </c>
-      <c r="B22" s="21" t="n">
-        <v>42</v>
-      </c>
-      <c r="C22" s="27" t="n">
-        <v>1245</v>
+          <t>100 → 5.000 €, Minimum</t>
+        </is>
+      </c>
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>42 gün / 1.245 €</t>
+        </is>
+      </c>
+      <c r="C22" s="21" t="inlineStr">
+        <is>
+          <t>52 gün / 804 €</t>
+        </is>
       </c>
       <c r="D22" s="21" t="n">
-        <v>61</v>
-      </c>
-      <c r="E22" s="27" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F22" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="21" t="inlineStr">
+        <is>
+          <t>418 → 150 · 1.167 → 380 · 3.190 → 1.010</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>100 → 5.000 €, Medium</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>28 gün / 2.177 €</t>
+        </is>
+      </c>
+      <c r="C23" s="21" t="inlineStr">
+        <is>
+          <t>46 gün / 1.484 €</t>
+        </is>
+      </c>
+      <c r="D23" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E23" s="21" t="inlineStr">
+        <is>
+          <t>201 → 100 · 509 → 200 · 1.146 → 430 · 2.413 → 840 · 4.982 → 1.710</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>100 → 5.000 €, High</t>
+        </is>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>18 gün / 2.220 €</t>
+        </is>
+      </c>
+      <c r="C24" s="21" t="inlineStr">
+        <is>
+          <t>28 gün / 1.177 €</t>
+        </is>
+      </c>
+      <c r="D24" s="21" t="n">
         <v>4</v>
       </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="28" t="inlineStr">
-        <is>
-          <t>Kaynak: js/paper_engine.js buildEIRoadmap, 2026-09-26. Koçla hedefe ulaşmak daha uzun sürer; High/Medium'da tek kuponda riske edilen en yüksek tutar ~%45 düşer ve hedefe varıldığında ayrıca 2.000 €'yu aşan bir güven payı birikmiş olur (güven payı hedefe sayılmaz).</t>
-        </is>
-      </c>
+      <c r="E24" s="21" t="inlineStr">
+        <is>
+          <t>244 → 120 · 594 → 240 · 1.474 → 580 · 3.485 → 1.340</t>
+        </is>
+      </c>
+      <c r="F24" s="21" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="26" t="inlineStr">
-        <is>
-          <t>Detay: High risk, 100 € → 5.000 €</t>
-        </is>
-      </c>
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>50 → 1.000 €, Minimum</t>
+        </is>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>32 gün / 240 €</t>
+        </is>
+      </c>
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>38 gün / 167 €</t>
+        </is>
+      </c>
+      <c r="D25" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="21" t="inlineStr">
+        <is>
+          <t>209 → 79 · 621 → 200</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Gün</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Tetikleyici</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Oyundaki kasa (€)</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>Kenara (€) / Güven payı toplam (€)</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>Risk</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>Tek kupon riski (€): önce → sonra</t>
-        </is>
-      </c>
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>50 → 1.000 €, Medium</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>22 gün / 471 €</t>
+        </is>
+      </c>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>33 gün / 283 €</t>
+        </is>
+      </c>
+      <c r="D26" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E26" s="21" t="inlineStr">
+        <is>
+          <t>101 → 50 · 255 → 100 · 573 → 210</t>
+        </is>
+      </c>
+      <c r="F26" s="21" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="21" t="n">
-        <v>4</v>
+      <c r="A27" s="21" t="inlineStr">
+        <is>
+          <t>50 → 1.000 €, High</t>
+        </is>
       </c>
       <c r="B27" s="21" t="inlineStr">
         <is>
-          <t>Anapara güvencesi</t>
-        </is>
-      </c>
-      <c r="C27" s="27" t="n">
-        <v>244</v>
-      </c>
-      <c r="D27" s="21" t="inlineStr">
-        <is>
-          <t>100 / 100</t>
-        </is>
+          <t>14 gün / 455 €</t>
+        </is>
+      </c>
+      <c r="C27" s="21" t="inlineStr">
+        <is>
+          <t>21 gün / 256 €</t>
+        </is>
+      </c>
+      <c r="D27" s="21" t="n">
+        <v>3</v>
       </c>
       <c r="E27" s="21" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="inlineStr">
-        <is>
-          <t>122 → 72</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="21" t="n">
-        <v>10</v>
-      </c>
-      <c r="B28" s="21" t="inlineStr">
-        <is>
-          <t>Stres eşiği</t>
-        </is>
-      </c>
-      <c r="C28" s="27" t="n">
-        <v>550</v>
-      </c>
-      <c r="D28" s="21" t="inlineStr">
-        <is>
-          <t>190 / 290</t>
-        </is>
-      </c>
-      <c r="E28" s="21" t="inlineStr">
-        <is>
-          <t>High → Medium</t>
-        </is>
-      </c>
-      <c r="F28" s="21" t="inlineStr">
-        <is>
-          <t>275 → 180</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="21" t="n">
-        <v>15</v>
-      </c>
-      <c r="B29" s="21" t="inlineStr">
-        <is>
-          <t>Stres eşiği</t>
-        </is>
-      </c>
-      <c r="C29" s="27" t="n">
-        <v>724</v>
-      </c>
-      <c r="D29" s="21" t="inlineStr">
-        <is>
-          <t>0 / 290</t>
-        </is>
-      </c>
-      <c r="E29" s="21" t="inlineStr">
-        <is>
-          <t>Medium → Minimum</t>
-        </is>
-      </c>
-      <c r="F29" s="21" t="inlineStr">
-        <is>
-          <t>362 → 181</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="21" t="n">
-        <v>22</v>
-      </c>
-      <c r="B30" s="21" t="inlineStr">
-        <is>
-          <t>Stres eşiği</t>
-        </is>
-      </c>
-      <c r="C30" s="27" t="n">
-        <v>1410</v>
-      </c>
-      <c r="D30" s="21" t="inlineStr">
-        <is>
-          <t>360 / 650</t>
-        </is>
-      </c>
-      <c r="E30" s="21" t="inlineStr">
-        <is>
-          <t>Minimum</t>
-        </is>
-      </c>
-      <c r="F30" s="21" t="inlineStr">
-        <is>
-          <t>353 → 263</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="21" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="21" t="inlineStr">
-        <is>
-          <t>Stres eşiği</t>
-        </is>
-      </c>
-      <c r="C31" s="27" t="n">
-        <v>2252</v>
-      </c>
-      <c r="D31" s="21" t="inlineStr">
-        <is>
-          <t>600 / 1.250</t>
-        </is>
-      </c>
-      <c r="E31" s="21" t="inlineStr">
-        <is>
-          <t>Minimum</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="inlineStr">
-        <is>
-          <t>563 → 413</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="21" t="n">
-        <v>38</v>
-      </c>
-      <c r="B32" s="21" t="inlineStr">
-        <is>
-          <t>Stres eşiği</t>
-        </is>
-      </c>
-      <c r="C32" s="27" t="n">
-        <v>3541</v>
-      </c>
-      <c r="D32" s="21" t="inlineStr">
-        <is>
-          <t>940 / 2.190</t>
-        </is>
-      </c>
-      <c r="E32" s="21" t="inlineStr">
-        <is>
-          <t>Minimum</t>
-        </is>
-      </c>
-      <c r="F32" s="21" t="inlineStr">
-        <is>
-          <t>885 → 650</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="21" t="n">
-        <v>45</v>
-      </c>
-      <c r="B33" s="21" t="inlineStr">
-        <is>
-          <t>Hedef</t>
-        </is>
-      </c>
-      <c r="C33" s="27" t="n">
-        <v>5000</v>
-      </c>
-      <c r="D33" s="21" t="inlineStr">
-        <is>
-          <t>— / 2.190</t>
-        </is>
-      </c>
-      <c r="E33" s="21" t="inlineStr">
-        <is>
-          <t>Minimum</t>
-        </is>
-      </c>
-      <c r="F33" s="21" t="inlineStr">
-        <is>
-          <t>oyundaki kasa 5.000 €</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="28" t="inlineStr">
-        <is>
-          <t>Kullanıcının örneği (koçu dinlemeden 1.000 €'ya gelmiş, High): tek kupon 500 € = konforun 5 katı → seçenekler: 530 € kenara + High (11 gün), 530 € kenara + Medium (önerilen, 17 gün), 300 € kenara + Minimum (21 gün).</t>
+          <t>122 → 64 · 341 → 140 · 726 → 260</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="inlineStr"/>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Kaynak: js/paper_engine.js getEICoach / eiProject, 2026-09-26; rahat sınır = başlangıç kasası, her gün teorik büyüme gerçekleşirse. Güven Payı ile hedefe ulaşmak daha uzun sürer; karşılığında en yüksek kupon %24–47 küçülür ve yol boyunca kasanın bir kısmı kalıcı olarak güvende olur.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="4">
+    <mergeCell ref="A13:F13"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A28:F28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
İş listesi: #1 ve #14 commit hash eklendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -851,7 +851,7 @@
       <c r="M5" s="19" t="n"/>
       <c r="N5" s="21" t="inlineStr">
         <is>
-          <t>d8d4301 — Sanal Kasa'ya Duygusal Denge Koçu: stres eşiği / anapara / zirveden düşüş / kazanç serisi sinyalleri, risk profili seçenekli cash-out, elle kenara koyma, geri alma, yol haritası; tablo+grafikte 'Kenarda' (js/paper_engine.js, js/paper_ui.js). a6b9224 — güven payı kazanç eğrisi/hedef dışında; Güven Payı İşlemleri (kenara koy / kasaya geri al); Tab/Enter ile sonraki gün; girişte sayfa kaymıyor. Sadeleştirme: Güven Payı kartı (tek sayı + tek buton + yol çizgisi), rahat sınır alanı, Oyundaki/Kilitli sütunları.</t>
+          <t>d8d4301 — Sanal Kasa'ya Duygusal Denge Koçu: stres eşiği / anapara / zirveden düşüş / kazanç serisi sinyalleri, risk profili seçenekli cash-out, elle kenara koyma, geri alma, yol haritası; tablo+grafikte 'Kenarda' (js/paper_engine.js, js/paper_ui.js). a6b9224 — güven payı kazanç eğrisi/hedef dışında; Güven Payı İşlemleri (kenara koy / kasaya geri al); Tab/Enter ile sonraki gün; girişte sayfa kaymıyor. f3e7679 — Sadeleştirme: Güven Payı kartı (tek sayı + tek buton + yol çizgisi), rahat sınır alanı, Oyundaki/Kilitli sütunları.</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1483,7 @@
       <c r="M18" s="19" t="n"/>
       <c r="N18" s="7" t="inlineStr">
         <is>
-          <t>Güven Payı sadeleştirmesiyle aynı commit (js/paper_engine.js reopenClosedPlan/deleteClosedPlan, js/auth_sync.js)</t>
+          <t>f3e7679 — (js/paper_engine.js reopenClosedPlan/deleteClosedPlan, js/auth_sync.js)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Üst menü: sığmadığında kompakt tek satır, yine sığmazsa iki satır (EN/NL yatay taşma giderildi); NL 'Wedstrijden'
İş listesi #15 → Tamamlandı.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1523,12 +1523,20 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Öneri</t>
-        </is>
-      </c>
-      <c r="I19" s="7" t="n"/>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>Claude (Murat)</t>
+        </is>
+      </c>
       <c r="J19" s="8" t="n"/>
-      <c r="K19" s="7" t="n"/>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>Tüm dillerde: menü sığmazsa önce kompakt (alt yazılar gizli), yine sığmazsa iki satır. EN artık tek satır, NL geniş ekranda iki satır; hiçbir genişlikte yatay taşma yok.</t>
+        </is>
+      </c>
       <c r="L19" s="19" t="n">
         <v>46291</v>
       </c>

</xml_diff>

<commit_message>
İş listesi #15: kapanış tarihi ve commit hash
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1540,8 +1540,14 @@
       <c r="L19" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M19" s="19" t="n"/>
-      <c r="N19" s="7" t="n"/>
+      <c r="M19" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>add4e73 — üst menü sığdırma (compact/wrapped) + NL Wedstrijden</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="L20" s="20" t="n"/>

</xml_diff>

<commit_message>
Güven Payı: güvenli sınır otomatik (başlangıç kasası + kilitli para; kişiye sorulmaz), kart tek satır durum + tek buton + 'Güvenli sınır nedir?' açıklaması; yol çizgisi ve rahat sınır alanı kaldırıldı
Dayanak: zihinsel muhasebe (Thaler 1999), kasanın parası etkisi (Thaler & Johnson 1990), kayıptan kaçınma (Tversky & Kahneman 1992), peanuts etkisi (Weber & Chapman 2005). İş listesi #1 ve Güven Payı Kuralları sayfası güncellendi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -842,7 +842,7 @@
       <c r="J5" s="8" t="inlineStr"/>
       <c r="K5" s="21" t="inlineStr">
         <is>
-          <t>Sadeleştirildi (2026-09-26): tek kural (bugünkü kupon &gt; rahat sınır → tek butonla kilitle), kilitli para hedefe sayılır, duraklı yol çizgisi. Kurallar 'Güven Payı Kuralları' sayfasında.</t>
+          <t>Sadeleştirildi (2026-09-26): güvenli sınır OTOMATİK (başlangıç kasası + kilitli para, kişiye sorulmaz; dayanak: zihinsel muhasebe, kasanın parası etkisi, kayıptan kaçınma). Tek satır durum + tek buton + 'Güvenli sınır nedir?' açıklaması. Kurallar 'Güven Payı Kuralları' sayfasında.</t>
         </is>
       </c>
       <c r="L5" s="19" t="n">
@@ -851,7 +851,7 @@
       <c r="M5" s="19" t="n"/>
       <c r="N5" s="21" t="inlineStr">
         <is>
-          <t>d8d4301 — Sanal Kasa'ya Duygusal Denge Koçu: stres eşiği / anapara / zirveden düşüş / kazanç serisi sinyalleri, risk profili seçenekli cash-out, elle kenara koyma, geri alma, yol haritası; tablo+grafikte 'Kenarda' (js/paper_engine.js, js/paper_ui.js). a6b9224 — güven payı kazanç eğrisi/hedef dışında; Güven Payı İşlemleri (kenara koy / kasaya geri al); Tab/Enter ile sonraki gün; girişte sayfa kaymıyor. f3e7679 — Sadeleştirme: Güven Payı kartı (tek sayı + tek buton + yol çizgisi), rahat sınır alanı, Oyundaki/Kilitli sütunları.</t>
+          <t>d8d4301 — Sanal Kasa'ya Duygusal Denge Koçu: stres eşiği / anapara / zirveden düşüş / kazanç serisi sinyalleri, risk profili seçenekli cash-out, elle kenara koyma, geri alma, yol haritası; tablo+grafikte 'Kenarda' (js/paper_engine.js, js/paper_ui.js). a6b9224 — güven payı kazanç eğrisi/hedef dışında; Güven Payı İşlemleri (kenara koy / kasaya geri al); Tab/Enter ile sonraki gün; girişte sayfa kaymıyor. f3e7679 — Sadeleştirme: Güven Payı kartı (tek sayı + tek buton + yol çizgisi), rahat sınır alanı, Oyundaki/Kilitli sütunları. SONRAKI: güvenli sınır OTOMATİK (kişiye sorulmaz), kart tek satır + tek buton + açıklama; yol çizgisi ve rahat sınır alanı kaldırıldı.</t>
         </is>
       </c>
     </row>
@@ -3290,12 +3290,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
     <col width="44" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="4" customWidth="1" min="6" max="6"/>
@@ -3315,6 +3315,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3346,22 +3347,22 @@
     <row r="5">
       <c r="A5" s="23" t="inlineStr">
         <is>
-          <t>Rahat sınır</t>
+          <t>Güvenli sınır (otomatik)</t>
         </is>
       </c>
       <c r="B5" s="21" t="inlineStr">
         <is>
-          <t>Kasa açılırken sorulur: "Tek kupona en fazla ne kadar koymak seni rahatsız etmez?" Boş = başlangıç kasası.</t>
+          <t>Her zaman; kişiye sorulmaz</t>
         </is>
       </c>
       <c r="C5" s="21" t="inlineStr">
         <is>
-          <t>Kupon, bu sınırla karşılaştırılır. Sınır = seçilen tutar + kilitli para.</t>
+          <t>Sınır = başlangıç kasası + kilitli para. Kart: "Bugünkü kuponun X €, güvenli sınırın Y €". "Güvenli sınır nedir?" altında kısa açıklama.</t>
         </is>
       </c>
       <c r="D5" s="21" t="inlineStr">
         <is>
-          <t>Stres kişiye özeldir; tahmin etmek yerine kişiye sormak en dürüst yol. Kilitli para güvende olduğu için kişi alışır, sınır onunla büyür.</t>
+          <t>Zihinsel muhasebe: başlangıç kasası kişinin kaybetmeyi baştan kabul ettiği bütçedir (Thaler 1999). Kasanın parası etkisi: kazançtan sonra risk fark edilmeden artar, bu yüzden sınır kazançla değil yalnızca kilitli parayla büyür (Thaler &amp; Johnson 1990). Tutar büyüdükçe beklenen hayal kırıklığı ve temkin artar (Weber &amp; Chapman 2005).</t>
         </is>
       </c>
       <c r="E5" s="21" t="inlineStr">
@@ -3412,12 +3413,12 @@
       </c>
       <c r="C7" s="21" t="inlineStr">
         <is>
-          <t>Tek buton: "🔒 X € kilitle". Kupon, sınırın dörtte birine iner. İsteğe bağlı: riski bir kademe düşür.</t>
+          <t>Tek buton: "🔒 X € kilitle". Kupon, sınırın dörtte birine iner.</t>
         </is>
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>Kayıptan kaçınma: kaybın acısı kazancın keyfinden ~2 kat güçlü. Kuponu belirgin biçimde (4 kat) küçültmek bir sonraki durağa kadar rahat bir alan bırakır.</t>
+          <t>Kayıptan kaçınma: kaybın acısı kazancın keyfinden ~2,25 kat güçlü (Tversky &amp; Kahneman 1992). Kuponu belirgin biçimde (4 kat) küçültmek bir sonraki durağa kadar rahat bir alan bırakır.</t>
         </is>
       </c>
       <c r="E7" s="21" t="inlineStr">
@@ -3482,22 +3483,22 @@
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
         <is>
-          <t>Yol çizgisi</t>
+          <t>Sonraki kilit</t>
         </is>
       </c>
       <c r="B10" s="21" t="inlineStr">
         <is>
-          <t>Her zaman</t>
+          <t>Kilitleme önerisi yokken</t>
         </is>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
-          <t>Başlangıçtan hedefe tek çizgi, üzerinde 🔒 durakları ve "Sıradaki durak: kasa ~X € olunca Y € kilitle".</t>
+          <t>Tek cümle: "Sonraki kilit: kasan ~X € olunca."</t>
         </is>
       </c>
       <c r="D10" s="21" t="inlineStr">
         <is>
-          <t>Durakları baştan görmek sürprizi ve anlık heyecanla karar vermeyi azaltır. Çizgi logaritmiktir: 50→100 € ile 1.000→2.000 € aynı adım gibi hissedilir (Weber-Fechner).</t>
+          <t>Sıradaki durağı önceden bilmek sürprizi ve anlık heyecanla karar vermeyi azaltır. Duraklar kasanın her ~2,3 katına çıkışında gelir; para algısı orantısal olduğu için (Weber-Fechner) eşit aralıklı hissedilir.</t>
         </is>
       </c>
       <c r="E10" s="21" t="inlineStr"/>
@@ -3527,6 +3528,7 @@
       <c r="E11" s="21" t="inlineStr"/>
       <c r="F11" s="21" t="inlineStr"/>
     </row>
+    <row r="12"/>
     <row r="13" ht="44" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
@@ -3534,6 +3536,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="26" t="inlineStr">
         <is>
@@ -3548,6 +3551,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
@@ -3813,16 +3817,172 @@
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Kaynak: js/paper_engine.js getEICoach / eiProject, 2026-09-26; rahat sınır = başlangıç kasası, her gün teorik büyüme gerçekleşirse. Güven Payı ile hedefe ulaşmak daha uzun sürer; karşılığında en yüksek kupon %24–47 küçülür ve yol boyunca kasanın bir kısmı kalıcı olarak güvende olur.</t>
+          <t>Kaynak: js/paper_engine.js getEICoach / eiProject, 2026-09-26; güvenli sınır = başlangıç kasası + kilitli para, her gün teorik büyüme gerçekleşirse. Güven Payı ile hedefe ulaşmak daha uzun sürer; karşılığında en yüksek kupon %24–47 küçülür ve yol boyunca kasanın bir kısmı kalıcı olarak güvende olur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="26" t="inlineStr">
+        <is>
+          <t>Dış kaynaklar</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Kaynak</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Ne için</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Bağlantı</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>Thaler &amp; Johnson (1990), Management Science 36(6)</t>
+        </is>
+      </c>
+      <c r="B32" s="21" t="inlineStr">
+        <is>
+          <t>Kasanın parası ve başa baş etkisi</t>
+        </is>
+      </c>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>https://pubsonline.informs.org/doi/abs/10.1287/mnsc.36.6.643</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="inlineStr"/>
+      <c r="E32" s="21" t="inlineStr"/>
+      <c r="F32" s="21" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>Thaler (1999), Mental Accounting Matters</t>
+        </is>
+      </c>
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>Zihinsel muhasebe: bütçe ve referans noktası</t>
+        </is>
+      </c>
+      <c r="C33" s="21" t="inlineStr">
+        <is>
+          <t>https://www-apache.anderson.ucla.edu/faculty_pages/keith.chen/negot.%20papers/Thaler_MentalAccounting99.pdf</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="inlineStr"/>
+      <c r="E33" s="21" t="inlineStr"/>
+      <c r="F33" s="21" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>Tversky &amp; Kahneman (1992); kayıptan kaçınma meta-analizi</t>
+        </is>
+      </c>
+      <c r="B34" s="21" t="inlineStr">
+        <is>
+          <t>Kayıp ≈ 2,25 × kazanç (bağlama göre değişir)</t>
+        </is>
+      </c>
+      <c r="C34" s="21" t="inlineStr">
+        <is>
+          <t>https://www.sciencedirect.com/science/article/pii/S0167487024000485</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="inlineStr"/>
+      <c r="E34" s="21" t="inlineStr"/>
+      <c r="F34" s="21" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="21" t="inlineStr">
+        <is>
+          <t>Weber &amp; Chapman (2005), OBHDP</t>
+        </is>
+      </c>
+      <c r="B35" s="21" t="inlineStr">
+        <is>
+          <t>Peanuts etkisi: tutar büyüdükçe temkin artar</t>
+        </is>
+      </c>
+      <c r="C35" s="21" t="inlineStr">
+        <is>
+          <t>https://www.sciencedirect.com/science/article/abs/pii/S0749597805000361</t>
+        </is>
+      </c>
+      <c r="D35" s="21" t="inlineStr"/>
+      <c r="E35" s="21" t="inlineStr"/>
+      <c r="F35" s="21" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="21" t="inlineStr">
+        <is>
+          <t>Lower-Risk Gambling Guidelines, CCSA (2021)</t>
+        </is>
+      </c>
+      <c r="B36" s="21" t="inlineStr">
+        <is>
+          <t>Hanehalkı gelirinin aylık en fazla %1'i, ayda en fazla 4 gün</t>
+        </is>
+      </c>
+      <c r="C36" s="21" t="inlineStr">
+        <is>
+          <t>https://gamblingguidelines.ca/lower-risk-gambling-guidelines/what-are-the-guidelines/</t>
+        </is>
+      </c>
+      <c r="D36" s="21" t="inlineStr"/>
+      <c r="E36" s="21" t="inlineStr"/>
+      <c r="F36" s="21" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="21" t="inlineStr">
+        <is>
+          <t>Bahis kasa yönetimi rehberleri (ör. Covers)</t>
+        </is>
+      </c>
+      <c r="B37" s="21" t="inlineStr">
+        <is>
+          <t>Profesyonel standart: bahis başına kasanın %1–5'i</t>
+        </is>
+      </c>
+      <c r="C37" s="21" t="inlineStr">
+        <is>
+          <t>https://www.covers.com/guides/sports-betting-bank-roll-management-and-roi</t>
+        </is>
+      </c>
+      <c r="D37" s="21" t="inlineStr"/>
+      <c r="E37" s="21" t="inlineStr"/>
+      <c r="F37" s="21" t="inlineStr"/>
+    </row>
+    <row r="38" ht="36" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Not: Sitenin büyüme modeli günlük kasanın %25–50'si ile oynar; bu, profesyonel %1–5 standardının çok üstündedir. Güven Payı bu yüksek tempoyu değiştirmez; tempo nedeniyle büyüyen kupon tutarının yarattığı stresi sınırlar.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A13:F13"/>
+  <mergeCells count="5">
+    <mergeCell ref="A38:F38"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A13:F13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
İş listesi #1: commit hash eklendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -851,7 +851,7 @@
       <c r="M5" s="19" t="n"/>
       <c r="N5" s="21" t="inlineStr">
         <is>
-          <t>d8d4301 — Sanal Kasa'ya Duygusal Denge Koçu: stres eşiği / anapara / zirveden düşüş / kazanç serisi sinyalleri, risk profili seçenekli cash-out, elle kenara koyma, geri alma, yol haritası; tablo+grafikte 'Kenarda' (js/paper_engine.js, js/paper_ui.js). a6b9224 — güven payı kazanç eğrisi/hedef dışında; Güven Payı İşlemleri (kenara koy / kasaya geri al); Tab/Enter ile sonraki gün; girişte sayfa kaymıyor. f3e7679 — Sadeleştirme: Güven Payı kartı (tek sayı + tek buton + yol çizgisi), rahat sınır alanı, Oyundaki/Kilitli sütunları. SONRAKI: güvenli sınır OTOMATİK (kişiye sorulmaz), kart tek satır + tek buton + açıklama; yol çizgisi ve rahat sınır alanı kaldırıldı.</t>
+          <t>d8d4301 — Sanal Kasa'ya Duygusal Denge Koçu: stres eşiği / anapara / zirveden düşüş / kazanç serisi sinyalleri, risk profili seçenekli cash-out, elle kenara koyma, geri alma, yol haritası; tablo+grafikte 'Kenarda' (js/paper_engine.js, js/paper_ui.js). a6b9224 — güven payı kazanç eğrisi/hedef dışında; Güven Payı İşlemleri (kenara koy / kasaya geri al); Tab/Enter ile sonraki gün; girişte sayfa kaymıyor. f3e7679 — Sadeleştirme: Güven Payı kartı (tek sayı + tek buton + yol çizgisi), rahat sınır alanı, Oyundaki/Kilitli sütunları. 1f2a385 — güvenli sınır OTOMATİK (kişiye sorulmaz), kart tek satır + tek buton + açıklama; yol çizgisi ve rahat sınır alanı kaldırıldı.</t>
         </is>
       </c>
     </row>
@@ -3315,7 +3315,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3528,7 +3527,6 @@
       <c r="E11" s="21" t="inlineStr"/>
       <c r="F11" s="21" t="inlineStr"/>
     </row>
-    <row r="12"/>
     <row r="13" ht="44" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
@@ -3536,7 +3534,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="26" t="inlineStr">
         <is>
@@ -3551,7 +3548,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
@@ -3821,7 +3817,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Testler: 10-16 bugünkü siteye göre yeniden yazıldı (menü, Güven Payı motoru ve ekranı, Tab ile gün geçişi, kapatılan kasa yeniden aç/sil + senkron, üst menü taşma); gizli sekmelerin eski ekran testleri kaldırıldı
İş listesi: #7 Tamamlandı; #5, #6, #11, #12, #13 Açık (plana alındı).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1035,7 +1035,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Öneri</t>
+          <t>Açık</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr"/>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Öneri</t>
+          <t>Açık</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr"/>
@@ -1131,16 +1131,26 @@
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Öneri</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr"/>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Claude (Murat)</t>
+        </is>
+      </c>
       <c r="J11" s="8" t="inlineStr"/>
-      <c r="K11" s="7" t="inlineStr"/>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>TEST 10 menü (4 sekme), 12 Güven Payı motoru, 13 Sanal Kasa ekranı + kilitleme + Tab, 14 kapatılan kasa yeniden aç/sil + senkron, 16 üst menü TR/EN/NL taşma. Gizli sekmelerin eski ekran testleri (sim-kupon, rec, cpn) kaldırıldı. 34 kontrol geçiyor.</t>
+        </is>
+      </c>
       <c r="L11" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M11" s="19" t="n"/>
+      <c r="M11" s="19" t="n">
+        <v>46291</v>
+      </c>
       <c r="N11" s="7" t="n"/>
     </row>
     <row r="12">
@@ -1323,7 +1333,7 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Öneri</t>
+          <t>Açık</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr"/>
@@ -1371,7 +1381,7 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Öneri</t>
+          <t>Açık</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr"/>
@@ -1419,7 +1429,7 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Öneri</t>
+          <t>Açık</t>
         </is>
       </c>
       <c r="I17" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
İş listesi #7: commit hash eklendi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1151,7 +1151,11 @@
       <c r="M11" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="N11" s="7" t="n"/>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>905890e — scripts/test_paper_betting.py testleri 10-16 yeniden yazıldı</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">

</xml_diff>

<commit_message>
Is listesi #6: tamamlandi (da16191, 952d698)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1083,17 +1083,27 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr"/>
       <c r="J10" s="8" t="inlineStr"/>
-      <c r="K10" s="7" t="inlineStr"/>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>İlk çalışmada bulgu: LaLiga Levante-Athletic 16.09 hiç notlanmamış (football-data/ESPN'de yok → ertelenmiş ya da hayalet fikstür). Uyarılar: GitHub → Actions → çalışma özeti.</t>
+        </is>
+      </c>
       <c r="L10" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M10" s="19" t="n"/>
-      <c r="N10" s="7" t="n"/>
+      <c r="M10" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N10" s="7" t="inlineStr">
+        <is>
+          <t>da16191 — scripts/validate_data.py: hata (yayını durdurur) + uyarı (Actions özeti) kontrolleri, test_validate_data.py 7 senaryo; CI'da yeşil | 952d698 — botun push öncesi rebase'i (çift push'ta kırmızı düşen çalışmalar)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">

</xml_diff>

<commit_message>
Is listesi #11 tamamlandi (80c00f6); #16 oneri: mobilde ust baslik alani
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1347,17 +1347,27 @@
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr"/>
       <c r="J15" s="8" t="inlineStr"/>
-      <c r="K15" s="7" t="inlineStr"/>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>Bulgu → #16 (mobilde üst başlık alanı). TR sayı biçimi tutarsızlığı (91.9% / %91,9) #13 kapsamında.</t>
+        </is>
+      </c>
       <c r="L15" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M15" s="19" t="n"/>
-      <c r="N15" s="7" t="n"/>
+      <c r="M15" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>80c00f6 — 3 dil × 360/390/414 px × 4 sekme otomatik tarandı (yatay taşma yok) + ekran görüntüleri incelendi; Sanal Kasa günlük tablosunda Gün sütunu yatay kaydırmada sabitlendi</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -1574,7 +1584,52 @@
       </c>
     </row>
     <row r="20">
-      <c r="L20" s="20" t="n"/>
+      <c r="A20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Mobilde üst başlık alanını küçült</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Telefonda (360 px) üst bar + sekmeler (~165 px) ve 'Betting Analysis, Variance &amp; Uncertainty System' bandı + 3 özellik çipi (~140 px) her sekmede tekrar ediyor; ilk içerik ekranın ~%40'ından sonra başlıyor. Öneri: telefonda bant/çipleri yalnızca Fikstür'de göster veya tek satıra indir. Ayrıca TR arayüzde çipler İngilizce (AI-powered vb.) — bilinçli mi?</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Claude (#11 mobil kontrolden)</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="n"/>
+      <c r="J20" s="8" t="n"/>
+      <c r="K20" s="7" t="n"/>
+      <c r="L20" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M20" s="19" t="n"/>
+      <c r="N20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="L21" s="20" t="n"/>

</xml_diff>

<commit_message>
Is listesi #12: Test (Supabase'de hesap_silme.sql bekliyor); CLAUDE.md: hash push'tan sonra, run_tests
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1405,17 +1405,25 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr"/>
       <c r="J16" s="8" t="inlineStr"/>
-      <c r="K16" s="7" t="inlineStr"/>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>CANLIDA ETKİN DEĞİL: Supabase panel erişimi olan kişi SQL Editor'de supabase/hesap_silme.sql'i bir kez çalıştırmalı (canlı projede fonksiyon yok, kontrol edildi). O zamana kadar buton 'henüz etkinleştirilmedi' der, hiçbir şey silmez. Çalıştırılınca Tamamlandı yapılabilir.</t>
+        </is>
+      </c>
       <c r="L16" s="19" t="n">
         <v>46291</v>
       </c>
       <c r="M16" s="19" t="n"/>
-      <c r="N16" s="7" t="n"/>
+      <c r="N16" s="7" t="inlineStr">
+        <is>
+          <t>27f7107 — Hesabım &gt; Hesabımı sil (kullanıcı adı onaylı, 'bu cihazdaki verileri de sil' seçeneği), supabase/hesap_silme.sql, gizlilik sayfası TR/EN/NL, test_delete_account.py 3 senaryo; canlıya yayında</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">

</xml_diff>

<commit_message>
Is listesi #13 tamamlandi (907518a)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1461,17 +1461,27 @@
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I17" s="7" t="inlineStr"/>
       <c r="J17" s="8" t="inlineStr"/>
-      <c r="K17" s="7" t="inlineStr"/>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>Anadili Hollandaca biri isterse ayrıca üslup kontrolü yapabilir; bariz hata kalmadı. TR'de tablo yüzdeleri '95.9%', şeritte '%91,9' — i18n.js'te bilinçli 'Türkçe görünüm değişmez' kararı, değiştirilmedi.</t>
+        </is>
+      </c>
       <c r="L17" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M17" s="19" t="n"/>
-      <c r="N17" s="7" t="n"/>
+      <c r="M17" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N17" s="7" t="inlineStr">
+        <is>
+          <t>907518a — NL/EN otomatik tarama (sekmeler + maç detayı + giriş penceresi): çevrilmemiş metin yok; 399 NL girişi okundu, 4 hata düzeltildi (puan tablosu 'G' çakışması, trefkans→trefpercentage, Totale start/sluiting, yaş mesajı 3 dilde)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">

</xml_diff>

<commit_message>
Is listesi #2: tamamlandi, sonuc negatif (799a2bf)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -891,17 +891,27 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr"/>
       <c r="J6" s="8" t="inlineStr"/>
-      <c r="K6" s="7" t="inlineStr"/>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>Sonuç negatif: geçmişte vurgusu tutmayan takımlar sonraki sezonda diğerleriyle aynı tutuyor (pazar içi fark anlamsız) → şans. Canlı koda dokunulmadı.</t>
+        </is>
+      </c>
       <c r="L6" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M6" s="19" t="n"/>
-      <c r="N6" s="7" t="n"/>
+      <c r="M6" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N6" s="7" t="inlineStr">
+        <is>
+          <t>799a2bf — scripts/tune_team_blacklist.py: 24 ayarlı ileriye dönük test, 13.133 vurgu. Kara liste isabeti artırmıyor (en iyi +0,03 puan, anlamsız; çoğu ayarda düşürüyor). YAYINA ALINMADI.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">

</xml_diff>

<commit_message>
Is listesi #3: backtest tamam, urun karari bekliyor (87e4154)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -949,17 +949,25 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Devam ediyor</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr"/>
       <c r="J7" s="8" t="inlineStr"/>
-      <c r="K7" s="7" t="inlineStr"/>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>BACKTEST SONUCU (karar bekliyor): bugünkü profillerin hedef oranları (1.28/1.42/1.35) kuponların gerçek tutma oranından çıkan adil orandan yüksek (Minimum adil 1.15, Yüksek 1.24). Piyasa oranlarıyla ROI −9% / −15% / −13%, kasa sezonda eriyor. 137 ayardan hiçbiri eğitim+doğrulamada kârlı değil; en iyiler ≈ −1% (tek maç ÇŞ ≥%85). Sayfa tasarımına geçmeden önce ürün kararı gerekli.</t>
+        </is>
+      </c>
       <c r="L7" s="19" t="n">
         <v>46291</v>
       </c>
       <c r="M7" s="19" t="n"/>
-      <c r="N7" s="7" t="n"/>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>87e4154 — adım 1/2 backtest: scripts/tune_coupon_profiles.py</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">

</xml_diff>

<commit_message>
Is listesi #3: beklemede, Gokhan ile konusulacak
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -949,14 +949,14 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Devam ediyor</t>
+          <t>Açık</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr"/>
       <c r="J7" s="8" t="inlineStr"/>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>BACKTEST SONUCU (karar bekliyor): bugünkü profillerin hedef oranları (1.28/1.42/1.35) kuponların gerçek tutma oranından çıkan adil orandan yüksek (Minimum adil 1.15, Yüksek 1.24). Piyasa oranlarıyla ROI −9% / −15% / −13%, kasa sezonda eriyor. 137 ayardan hiçbiri eğitim+doğrulamada kârlı değil; en iyiler ≈ −1% (tek maç ÇŞ ≥%85). Sayfa tasarımına geçmeden önce ürün kararı gerekli.</t>
+          <t>BEKLEMEDE (26.09, Murat): Gökhan ile konuşulacak. BACKTEST SONUCU (karar bekliyor): bugünkü profillerin hedef oranları (1.28/1.42/1.35) kuponların gerçek tutma oranından çıkan adil orandan yüksek (Minimum adil 1.15, Yüksek 1.24). Piyasa oranlarıyla ROI −9% / −15% / −13%, kasa sezonda eriyor. 137 ayardan hiçbiri eğitim+doğrulamada kârlı değil; en iyiler ≈ −1% (tek maç ÇŞ ≥%85). Karar: (a) risk seviyelerini ölçülen kurallarla ve gerçek tutma oranlarıyla gösteren, büyüme vaadi olmayan öneri sayfası (önerilen) ya da (b) mevcut profillerle devam. Sanal Kasa %10/15/25 büyüme hedefleri de aynı bulguya takılıyor.</t>
         </is>
       </c>
       <c r="L7" s="19" t="n">

</xml_diff>

<commit_message>
Is listesi #12: tamamlandi (Supabase fonksiyonu canlida dogrulandi)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1423,20 +1423,22 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr"/>
       <c r="J16" s="8" t="inlineStr"/>
       <c r="K16" s="7" t="inlineStr">
         <is>
-          <t>CANLIDA ETKİN DEĞİL: Supabase panel erişimi olan kişi SQL Editor'de supabase/hesap_silme.sql'i bir kez çalıştırmalı (canlı projede fonksiyon yok, kontrol edildi). O zamana kadar buton 'henüz etkinleştirilmedi' der, hiçbir şey silmez. Çalıştırılınca Tamamlandı yapılabilir.</t>
+          <t>26.09: supabase/hesap_silme.sql Supabase SQL Editor'de çalıştırıldı; canlıda doğrulandı (giriş yapmadan çağrı 'permission denied' veriyor = fonksiyon kurulu, yetki kısıtı doğru). Gerçek bir hesapla uçtan uca deneme henüz yapılmadı.</t>
         </is>
       </c>
       <c r="L16" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M16" s="19" t="n"/>
+      <c r="M16" s="19" t="n">
+        <v>46291</v>
+      </c>
       <c r="N16" s="7" t="inlineStr">
         <is>
           <t>27f7107 — Hesabım &gt; Hesabımı sil (kullanıcı adı onaylı, 'bu cihazdaki verileri de sil' seçeneği), supabase/hesap_silme.sql, gizlilik sayfası TR/EN/NL, test_delete_account.py 3 senaryo; canlıya yayında</t>

</xml_diff>

<commit_message>
Is listesi #1 ve #14: tamamlandi (Murat)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -831,7 +831,7 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -842,13 +842,15 @@
       <c r="J5" s="8" t="inlineStr"/>
       <c r="K5" s="21" t="inlineStr">
         <is>
-          <t>Sadeleştirildi (2026-09-26): güvenli sınır OTOMATİK (başlangıç kasası + kilitli para, kişiye sorulmaz; dayanak: zihinsel muhasebe, kasanın parası etkisi, kayıptan kaçınma). Tek satır durum + tek buton + 'Güvenli sınır nedir?' açıklaması. Kurallar 'Güven Payı Kuralları' sayfasında.</t>
+          <t>Sadeleştirildi (2026-09-26): güvenli sınır OTOMATİK (başlangıç kasası + kilitli para, kişiye sorulmaz; dayanak: zihinsel muhasebe, kasanın parası etkisi, kayıptan kaçınma). Tek satır durum + tek buton + 'Güvenli sınır nedir?' açıklaması. Kurallar 'Güven Payı Kuralları' sayfasında. | 26.09 Murat: kapatıldı.</t>
         </is>
       </c>
       <c r="L5" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M5" s="19" t="n"/>
+      <c r="M5" s="19" t="n">
+        <v>46291</v>
+      </c>
       <c r="N5" s="21" t="inlineStr">
         <is>
           <t>d8d4301 — Sanal Kasa'ya Duygusal Denge Koçu: stres eşiği / anapara / zirveden düşüş / kazanç serisi sinyalleri, risk profili seçenekli cash-out, elle kenara koyma, geri alma, yol haritası; tablo+grafikte 'Kenarda' (js/paper_engine.js, js/paper_ui.js). a6b9224 — güven payı kazanç eğrisi/hedef dışında; Güven Payı İşlemleri (kenara koy / kasaya geri al); Tab/Enter ile sonraki gün; girişte sayfa kaymıyor. f3e7679 — Sadeleştirme: Güven Payı kartı (tek sayı + tek buton + yol çizgisi), rahat sınır alanı, Oyundaki/Kilitli sütunları. 1f2a385 — güvenli sınır OTOMATİK (kişiye sorulmaz), kart tek satır + tek buton + açıklama; yol çizgisi ve rahat sınır alanı kaldırıldı.</t>
@@ -1539,7 +1541,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I18" s="7" t="inlineStr">
@@ -1548,11 +1550,17 @@
         </is>
       </c>
       <c r="J18" s="8" t="n"/>
-      <c r="K18" s="7" t="n"/>
+      <c r="K18" s="7" t="inlineStr">
+        <is>
+          <t>26.09 Murat: kapatıldı.</t>
+        </is>
+      </c>
       <c r="L18" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M18" s="19" t="n"/>
+      <c r="M18" s="19" t="n">
+        <v>46291</v>
+      </c>
       <c r="N18" s="7" t="inlineStr">
         <is>
           <t>f3e7679 — (js/paper_engine.js reopenClosedPlan/deleteClosedPlan, js/auth_sync.js)</t>

</xml_diff>

<commit_message>
Is listesi #8 tamamlandi (8199d3a); #17-#19 rakip analizinden oneriler
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1223,17 +1223,27 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr"/>
       <c r="J12" s="8" t="inlineStr"/>
-      <c r="K12" s="7" t="inlineStr"/>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>Çıkan öneriler: #9, #10, #17 gün şeridi, #18 biten maç tahmin yanında, #19 olasılık çubuğu; telefonda alt menü → #16.</t>
+        </is>
+      </c>
       <c r="L12" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M12" s="19" t="n"/>
-      <c r="N12" s="7" t="n"/>
+      <c r="M12" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N12" s="7" t="inlineStr">
+        <is>
+          <t>8199d3a — docs/rakip-analizi.md: 9 site masaüstü+telefon incelendi; korunacaklar, uygulanacaklar (öncelikli), yapılmamalılar</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -1670,7 +1680,11 @@
       </c>
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="8" t="n"/>
-      <c r="K20" s="7" t="n"/>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>#8 rakip analizi: Forebet telefonda sekmeleri alt menü çubuğuna almış; üst başlık küçülür, sekmeler başparmak altında.</t>
+        </is>
+      </c>
       <c r="L20" s="19" t="n">
         <v>46291</v>
       </c>
@@ -1678,13 +1692,148 @@
       <c r="N20" s="7" t="n"/>
     </row>
     <row r="21">
-      <c r="L21" s="20" t="n"/>
+      <c r="A21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Fikstür'de gün şeridi</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>'Tüm günler' takvim butonu yerine Bugün · Yarın · Cmt · Paz … düğmeleri, her günün maç sayısıyla (PredictZ, WinDrawWin, Over25Tips, Forebet). Bir dokunuşla gün seçimi.</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Claude (#8 rakip analizi)</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="n"/>
+      <c r="J21" s="8" t="n"/>
+      <c r="K21" s="7" t="n"/>
+      <c r="L21" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M21" s="19" t="n"/>
+      <c r="N21" s="7" t="n"/>
     </row>
     <row r="22">
-      <c r="L22" s="20" t="n"/>
+      <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Biten maçı tahminin yanında göster</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Fikstür'de oynanmış maçın skoru ve vurgunun tutup tutmadığı aynı satırda (Forebet). Geçmiş performans şeridini her maçta somutlaştırır. #4 ile birlikte düşünülmeli.</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Claude (#8 rakip analizi)</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="n"/>
+      <c r="J22" s="8" t="n"/>
+      <c r="K22" s="7" t="n"/>
+      <c r="L22" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M22" s="19" t="n"/>
+      <c r="N22" s="7" t="n"/>
     </row>
     <row r="23">
-      <c r="L23" s="20" t="n"/>
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Maç detayında olasılık çubuğu</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Yüzdelerin yanında ince çubuk (ThePuntersPage 1-X-2 çubuğu, Adam Choi yüzde çubuğu); bir bakışta okunur.</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Claude (#8 rakip analizi)</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Düşük</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="n"/>
+      <c r="J23" s="8" t="n"/>
+      <c r="K23" s="7" t="n"/>
+      <c r="L23" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M23" s="19" t="n"/>
+      <c r="N23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="L24" s="20" t="n"/>

</xml_diff>

<commit_message>
Is listesi #9: devam ediyor (83a4185)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1281,17 +1281,25 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Devam ediyor</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="8" t="inlineStr"/>
-      <c r="K13" s="7" t="inlineStr"/>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>26.09 Murat: asıl dert listenin Excel gibi (eski moda) görünmesi; filtre şeridi 1. adım, liste görünümü yenilenecek.</t>
+        </is>
+      </c>
       <c r="L13" s="19" t="n">
         <v>46291</v>
       </c>
       <c r="M13" s="19" t="n"/>
-      <c r="N13" s="7" t="n"/>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>83a4185 — 1. adım: bayraklı lig düğme şeridi (Fikstür + İstatistikler)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">

</xml_diff>

<commit_message>
Is listesi #9: geri alindi, Acik
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1281,25 +1281,21 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Devam ediyor</t>
+          <t>Açık</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="8" t="inlineStr"/>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>26.09 Murat: asıl dert listenin Excel gibi (eski moda) görünmesi; filtre şeridi 1. adım, liste görünümü yenilenecek.</t>
+          <t>26.09: bayraklı düğme şeridi denendi, Murat'ın isteğiyle geri alındı (b4e7365). Açılır liste eski hâlinde; yeni yön konuşulacak.</t>
         </is>
       </c>
       <c r="L13" s="19" t="n">
         <v>46291</v>
       </c>
       <c r="M13" s="19" t="n"/>
-      <c r="N13" s="7" t="inlineStr">
-        <is>
-          <t>83a4185 — 1. adım: bayraklı lig düğme şeridi (Fikstür + İstatistikler)</t>
-        </is>
-      </c>
+      <c r="N13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">

</xml_diff>

<commit_message>
Is listesi #9 tamamlandi (1d8c5d2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1281,21 +1281,27 @@
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="8" t="inlineStr"/>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>26.09: bayraklı düğme şeridi denendi, Murat'ın isteğiyle geri alındı (b4e7365). Açılır liste eski hâlinde; yeni yön konuşulacak.</t>
+          <t>26.09: bayraklı düğme şeridi denendi, Murat'ın isteğiyle geri alındı (b4e7365). Açılır liste eski hâlinde; yeni yön konuşulacak. | Murat onayladı.</t>
         </is>
       </c>
       <c r="L13" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M13" s="19" t="n"/>
-      <c r="N13" s="7" t="n"/>
+      <c r="M13" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>1d8c5d2 — 'Tüm ligler' açılır listesi modern panel (bayrak, maç sayısı, seçili işaret; telefonda alttan açılır), Fikstür + İstatistikler</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">

</xml_diff>

<commit_message>
Is listesi #10 tamamlandi (1076a19)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1339,17 +1339,27 @@
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr"/>
       <c r="J14" s="8" t="inlineStr"/>
-      <c r="K14" s="7" t="inlineStr"/>
+      <c r="K14" s="7" t="inlineStr">
+        <is>
+          <t>5 seçenek (A marka şeritleri, B yumuşak ışık, C taktik saha, D kümülatif artış, E saha+artış) önizlendi; Murat C'yi seçti. Esin: Hudl StatsBomb, Stats Perform, Understat, Opta Analyst.</t>
+        </is>
+      </c>
       <c r="L14" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M14" s="19" t="n"/>
-      <c r="N14" s="7" t="n"/>
+      <c r="M14" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
+          <t>1076a19 — seçenek C 'taktik saha' (silik saha, pas okları, şut noktaları, radar); açık/koyu tema, 1366/820/390 px kontrol</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">

</xml_diff>

<commit_message>
Is listesi #4 tamamlandi (4b82ff1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1007,17 +1007,27 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Öneri</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr"/>
       <c r="J8" s="8" t="inlineStr"/>
-      <c r="K8" s="7" t="inlineStr"/>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>Bulgu: vurgulu bölgede model hafif temkinli (0.5+: %94,9 dedi → %95,8; 1X: %83,9 → %87,6). Murat onayladı.</t>
+        </is>
+      </c>
       <c r="L8" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M8" s="19" t="n"/>
-      <c r="N8" s="7" t="n"/>
+      <c r="M8" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N8" s="7" t="inlineStr">
+        <is>
+          <t>4b82ff1 — İstatistikler'e kalibrasyon kartı: pazar seçmeli grafik + tablo, vurgulu özet, ortalama sapma; filtrelere uyar, günlük güncellenir</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">

</xml_diff>

<commit_message>
Is listesi #3 tamamlandi (c7b132a)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -951,23 +951,25 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr"/>
       <c r="J7" s="8" t="inlineStr"/>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>BEKLEMEDE (26.09, Murat): Gökhan ile konuşulacak. BACKTEST SONUCU (karar bekliyor): bugünkü profillerin hedef oranları (1.28/1.42/1.35) kuponların gerçek tutma oranından çıkan adil orandan yüksek (Minimum adil 1.15, Yüksek 1.24). Piyasa oranlarıyla ROI −9% / −15% / −13%, kasa sezonda eriyor. 137 ayardan hiçbiri eğitim+doğrulamada kârlı değil; en iyiler ≈ −1% (tek maç ÇŞ ≥%85). Karar: (a) risk seviyelerini ölçülen kurallarla ve gerçek tutma oranlarıyla gösteren, büyüme vaadi olmayan öneri sayfası (önerilen) ya da (b) mevcut profillerle devam. Sanal Kasa %10/15/25 büyüme hedefleri de aynı bulguya takılıyor.</t>
+          <t>BEKLEMEDE (26.09, Murat): Gökhan ile konuşulacak. BACKTEST SONUCU (karar bekliyor): bugünkü profillerin hedef oranları (1.28/1.42/1.35) kuponların gerçek tutma oranından çıkan adil orandan yüksek (Minimum adil 1.15, Yüksek 1.24). Piyasa oranlarıyla ROI −9% / −15% / −13%, kasa sezonda eriyor. 137 ayardan hiçbiri eğitim+doğrulamada kârlı değil; en iyiler ≈ −1% (tek maç ÇŞ ≥%85). Karar: (a) risk seviyelerini ölçülen kurallarla ve gerçek tutma oranlarıyla gösteren, büyüme vaadi olmayan öneri sayfası (önerilen) ya da (b) mevcut profillerle devam. Sanal Kasa %10/15/25 büyüme hedefleri de aynı bulguya takılıyor. | 26.09 Murat: 'ölçülmüş kurallar' yönü seçildi, onaylandı.</t>
         </is>
       </c>
       <c r="L7" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M7" s="19" t="n"/>
+      <c r="M7" s="19" t="n">
+        <v>46291</v>
+      </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>87e4154 — adım 1/2 backtest: scripts/tune_coupon_profiles.py</t>
+          <t>87e4154 — adım 1/2 backtest: scripts/tune_coupon_profiles.py | c7b132a — Sanal Kasa'da kupon önerisi kartı (ölçülmüş kurallar, geçmiş tutma oranı, adil oran, dürüst kâr notu); build_coupon_rules.py günlük</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Is listesi: #20 gol pazari oran verisi (park), hedef orana gore kupon (devam)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1868,10 +1868,104 @@
       <c r="N23" s="7" t="n"/>
     </row>
     <row r="24">
-      <c r="L24" s="20" t="n"/>
+      <c r="A24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Gol pazarları (0.5+/1.5+) için gerçek oran verisi</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Kupon önerisine gol kuponu eklemek için 0.5/1.5 Üst gerçek kapanış oranları gerekli (football-data'da yok). Aday: Footiqo tüm ligler veri seti €59,99 (1xBet kapanış, 2015/16+, O05/O15 sütunları doğrulandı). OddsPapi yalnız 2026+. Veri gelince tune_coupon_profiles ile gerçek oranlı test, sonra kartta Gol kuponu satırı.</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Murat (26.09)</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Açık</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="n"/>
+      <c r="J24" s="8" t="n"/>
+      <c r="K24" s="7" t="inlineStr">
+        <is>
+          <t>PARK EDİLDİ (26.09, Murat): satın alma kararı bekliyor, Murat geri dönecek.</t>
+        </is>
+      </c>
+      <c r="L24" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M24" s="19" t="n"/>
+      <c r="N24" s="7" t="n"/>
     </row>
     <row r="25">
-      <c r="L25" s="20" t="n"/>
+      <c r="A25" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Kupon önerisi: kasa hedef oranına göre kupon kur</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Sanal Kasa günlük büyüme hedefi için gereken oran (1 + hedef / kupon payı: Minimum 1,40 · Orta 1,30 · Yüksek 1,50) önerilen kuponlardan yüksek (1,07 / 1,23 / 1,38). Kasanın risk profiline göre gereken orana ulaşana kadar maç ekleyen kupon; kuralın geçmiş tutma oranı ve getirisi gerçek oranlarla gösterilir (beklenti eksi olabilir, açıkça yazılır).</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Murat (26.09)</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Devam ediyor</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="n"/>
+      <c r="J25" s="8" t="n"/>
+      <c r="K25" s="7" t="n"/>
+      <c r="L25" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M25" s="19" t="n"/>
+      <c r="N25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="L26" s="20" t="n"/>

</xml_diff>

<commit_message>
Is listesi #21 tamamlandi (aa45446)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1955,17 +1955,27 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Devam ediyor</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I25" s="7" t="n"/>
       <c r="J25" s="8" t="n"/>
-      <c r="K25" s="7" t="n"/>
+      <c r="K25" s="7" t="inlineStr">
+        <is>
+          <t>Murat onayladı. İlk 'geçmiş öneriler' sonuçları 9-10 Ekim maçlarından sonra. 0.5+/1.5+ oranları tahmini (#20).</t>
+        </is>
+      </c>
       <c r="L25" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M25" s="19" t="n"/>
-      <c r="N25" s="7" t="n"/>
+      <c r="M25" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N25" s="7" t="inlineStr">
+        <is>
+          <t>aa45446 — tüm vurgulu tahminlerden hedef orana ulaşan en olası kupon (≤5 maç), bot günlük kurar/dondurur/sonuçlandırır (data/coupons.json), kartta geçmiş öneriler</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="L26" s="20" t="n"/>

</xml_diff>

<commit_message>
Is listesi #17 #18 #19 tamamlandi (f7c1a29)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1759,17 +1759,27 @@
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Öneri</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I21" s="7" t="n"/>
       <c r="J21" s="8" t="n"/>
-      <c r="K21" s="7" t="n"/>
+      <c r="K21" s="7" t="inlineStr">
+        <is>
+          <t>Murat onayladı (26.09).</t>
+        </is>
+      </c>
       <c r="L21" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M21" s="19" t="n"/>
-      <c r="N21" s="7" t="n"/>
+      <c r="M21" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>f7c1a29</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -1807,17 +1817,27 @@
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Öneri</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I22" s="7" t="n"/>
       <c r="J22" s="8" t="n"/>
-      <c r="K22" s="7" t="n"/>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>Murat onayladı (26.09).</t>
+        </is>
+      </c>
       <c r="L22" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M22" s="19" t="n"/>
-      <c r="N22" s="7" t="n"/>
+      <c r="M22" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N22" s="7" t="inlineStr">
+        <is>
+          <t>f7c1a29</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -1855,17 +1875,27 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Öneri</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I23" s="7" t="n"/>
       <c r="J23" s="8" t="n"/>
-      <c r="K23" s="7" t="n"/>
+      <c r="K23" s="7" t="inlineStr">
+        <is>
+          <t>Murat onayladı (26.09).</t>
+        </is>
+      </c>
       <c r="L23" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M23" s="19" t="n"/>
-      <c r="N23" s="7" t="n"/>
+      <c r="M23" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N23" s="7" t="inlineStr">
+        <is>
+          <t>f7c1a29</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">

</xml_diff>

<commit_message>
Is listesi #16 tamamlandi (0ace88d)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1707,7 +1707,7 @@
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Öneri</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I20" s="7" t="n"/>
@@ -1720,8 +1720,14 @@
       <c r="L20" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M20" s="19" t="n"/>
-      <c r="N20" s="7" t="n"/>
+      <c r="M20" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>0ace88d — telefonda menü 165→96 px, başlık bandı yalnız Fikstür'de; İstatistikler/FAQ ilk içerik 321→100 px</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">

</xml_diff>

<commit_message>
Is listesi #5 tamamlandi (f762bc7); #22 oneri: kupalar yalniz 0.5+
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1067,17 +1067,27 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr"/>
       <c r="J9" s="8" t="inlineStr"/>
-      <c r="K9" s="7" t="inlineStr"/>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>Sonuç: yalnız 0.5+ lig seviyesinde tutuyor (%95,9); 1.5+/2.5+/Çifte Şans vurguları kupalarda belirgin düşük (%62–83). Kapsam %27 (iki takım da 10 ligimizde). Canlıya alınmadı; öneri → #22.</t>
+        </is>
+      </c>
       <c r="L9" s="19" t="n">
         <v>46291</v>
       </c>
-      <c r="M9" s="19" t="n"/>
-      <c r="N9" s="7" t="n"/>
+      <c r="M9" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>f762bc7 — ESPN'den 2.314 kupa maçı, lig katsayılı ayrı model, 520 maçlık ileriye dönük test</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -2014,7 +2024,52 @@
       </c>
     </row>
     <row r="26">
-      <c r="L26" s="20" t="n"/>
+      <c r="A26" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Kupa maçlarını Fikstür'e yalnız 0.5+ vurgusuyla eklemek</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>#5 backtest'ine göre kupalarda yalnız 0.5+ vurgusu lig seviyesinde tutuyor (243 vurgu, %95,9). Öneri: iki takımı da 10 ligimizden olan kupa maçlarını Fikstür'e 'Kupa' etiketiyle eklemek; yalnız 0.5+ vurgulanır, diğer olasılıklar gösterilir ama vurgulanmaz. Fikstür kaynağı ESPN (scripts/fetch_euro_results.py genişletilir), model scripts/tune_euro_backtest.py'deki lig katsayılı model.</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Claude (#5 backtest'ten)</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="n"/>
+      <c r="J26" s="8" t="n"/>
+      <c r="K26" s="7" t="n"/>
+      <c r="L26" s="19" t="n">
+        <v>46291</v>
+      </c>
+      <c r="M26" s="19" t="n"/>
+      <c r="N26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="L27" s="20" t="n"/>

</xml_diff>

<commit_message>
Is listesi #23 kilitleme uyarisi (3e65649)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2072,7 +2072,58 @@
       <c r="N26" s="7" t="n"/>
     </row>
     <row r="27">
-      <c r="L27" s="20" t="n"/>
+      <c r="A27" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Tutar girilince kilitleme uyarısı</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Sanal Kasa tablosuna tutar girilince kilitleme gerekiyorsa, Güven Payı kartı yukarıda kaldığı için kullanıcı görmüyordu; ekranın altında uyarı + tek dokunuşla kilitle.</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Murat (27.09)</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="n"/>
+      <c r="J27" s="8" t="n"/>
+      <c r="K27" s="7" t="n"/>
+      <c r="L27" s="19" t="n">
+        <v>46292</v>
+      </c>
+      <c r="M27" s="19" t="n">
+        <v>46292</v>
+      </c>
+      <c r="N27" s="7" t="inlineStr">
+        <is>
+          <t>3e65649 — tabloya tutar girilince kilitleme önerisi ekranın altında (kilitle / Güven Payı / kapat)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="L28" s="20" t="n"/>

</xml_diff>

<commit_message>
Is listesi #24 (177795b)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2126,7 +2126,58 @@
       </c>
     </row>
     <row r="28">
-      <c r="L28" s="20" t="n"/>
+      <c r="A28" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Kupon kartı: sabit kurallar kaldır, shuffle ekle</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Kartta yalnız kasa hedefine göre kupon kalsın; 'Başka kombinasyon' ile aynı risk için farklı kupon kombinasyonları gezilebilsin. Tutma olasılığını yükseltme denemesi (geçmiş isabete göre seçim) test edildi, fark gürültü düzeyinde.</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Murat (27.09)</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="n"/>
+      <c r="J28" s="8" t="n"/>
+      <c r="K28" s="7" t="n"/>
+      <c r="L28" s="19" t="n">
+        <v>46292</v>
+      </c>
+      <c r="M28" s="19" t="n">
+        <v>46292</v>
+      </c>
+      <c r="N28" s="7" t="inlineStr">
+        <is>
+          <t>177795b — sabit kurallar kaldırıldı; bot gün+profil başına ≤5 kombinasyon üretir, kartta 🔀 ile gezilir</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="L29" s="20" t="n"/>

</xml_diff>

<commit_message>
Is listesi #25: Guven Payi hedef sonrasi kilit (9fdc18f)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2180,7 +2180,58 @@
       </c>
     </row>
     <row r="29">
-      <c r="L29" s="20" t="n"/>
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Güven Payı: hedef sonrası kilitleme önerisi</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Hedefe ulaşılınca kilit önerisi ve düşüş uyarısı kesiliyordu; oynamaya devam edenin kazancı korumasız kalıyordu (Murat'ın tablosu: 4. günden sonra 220 € kilitli kaldı). Artık hedef bandı ışık + kilitle butonuyla birlikte görünür.</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Murat (27.09)</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="n"/>
+      <c r="J29" s="8" t="n"/>
+      <c r="K29" s="7" t="n"/>
+      <c r="L29" s="19" t="n">
+        <v>46292</v>
+      </c>
+      <c r="M29" s="19" t="n">
+        <v>46292</v>
+      </c>
+      <c r="N29" s="7" t="inlineStr">
+        <is>
+          <t>9fdc18f hedefe ulaşmak artık kilit önerisini engellemiyor + test</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="L30" s="20" t="n"/>

</xml_diff>

<commit_message>
Is listesi #26: arayuz onerisi (ornekler artifact'te)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2234,7 +2234,56 @@
       </c>
     </row>
     <row r="30">
-      <c r="L30" s="20" t="n"/>
+      <c r="A30" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Futuristik görünüm + kullanıcı dostu dokunuşlar</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Görünüm yönü (birini seç): A Aurora (açık tema + kayan ışık, buzlu cam) / B Koyu neon (cam paneller, parıltı) / C Saha çizgisi deseni (paralaks). Kolaylıklar: 1 mobil alt menü, 2 günün öne çıkanları kartı, 3 yükleniyor iskeleti + dolan çubuklar, 4 ilk giriş rehberi. Çalışan örnekler: https://claude.ai/artifact/6t215zEcNoZUpRh4HFWzqd</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Murat (27.09)</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I30" s="7" t="n"/>
+      <c r="J30" s="8" t="n"/>
+      <c r="K30" s="7" t="inlineStr">
+        <is>
+          <t>Murat örneklere bakıp seçecek.</t>
+        </is>
+      </c>
+      <c r="L30" s="19" t="n">
+        <v>46292</v>
+      </c>
+      <c r="M30" s="19" t="n"/>
+      <c r="N30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="L31" s="20" t="n"/>

</xml_diff>

<commit_message>
Is listesi #26 tamamlandi (43f7728)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2269,21 +2269,27 @@
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Öneri</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I30" s="7" t="n"/>
       <c r="J30" s="8" t="n"/>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>Murat örneklere bakıp seçecek.</t>
+          <t>Murat seçti: A Aurora + 1,2,3,4; ek istek: tüm göstergeler açılışta dolsun.</t>
         </is>
       </c>
       <c r="L30" s="19" t="n">
         <v>46292</v>
       </c>
-      <c r="M30" s="19" t="n"/>
-      <c r="N30" s="7" t="n"/>
+      <c r="M30" s="19" t="n">
+        <v>46292</v>
+      </c>
+      <c r="N30" s="7" t="inlineStr">
+        <is>
+          <t>43f7728 Aurora + alt menü + günün öne çıkanları + dolan göstergeler/sayaç + ilk giriş rehberi (canlıda doğrulandı)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="L31" s="20" t="n"/>

</xml_diff>

<commit_message>
Is listesi: #20 Test (bot bagli, oranlar 9-10 Ekim), #27 donen top onerisi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -1949,21 +1949,25 @@
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="I24" s="7" t="n"/>
       <c r="J24" s="8" t="n"/>
       <c r="K24" s="7" t="inlineStr">
         <is>
-          <t>PARK EDİLDİ (26.09, Murat): satın alma kararı bekliyor, Murat geri dönecek. | 27.09: Ücretsiz geçmiş 0.5/1.5 oran kaynağı bulunamadı (Kaggle/football-data.org/SharpAPI yok). Ücretsiz ileriye dönük seçenek: 5dollarfootballapi.com (Bet365 O0.5–9.5, yalnız 26.09.2026'dan beri, ücretsiz planda büyük 5 lig, maç başına sorgu). Murat hesap açıp anahtarı GitHub secret FIVEDOLLAR_API_KEY olarak eklerse bot bağlanacak. Alternatif: Footiqo €59,99 geçmiş veri. | 27.09 12:09 UTC: FIVEDOLLAR_API_KEY Actions secret'ı eklendi (doğrulandı). Sıradaki adım: bota 5DollarFootballAPI O0.5/O1.5 çekme adımı eklemek.</t>
+          <t>PARK EDİLDİ (26.09, Murat): satın alma kararı bekliyor, Murat geri dönecek. | 27.09: Ücretsiz geçmiş 0.5/1.5 oran kaynağı bulunamadı (Kaggle/football-data.org/SharpAPI yok). Ücretsiz ileriye dönük seçenek: 5dollarfootballapi.com (Bet365 O0.5–9.5, yalnız 26.09.2026'dan beri, ücretsiz planda büyük 5 lig, maç başına sorgu). Murat hesap açıp anahtarı GitHub secret FIVEDOLLAR_API_KEY olarak eklerse bot bağlanacak. Alternatif: Footiqo €59,99 geçmiş veri. | 27.09 12:09 UTC: FIVEDOLLAR_API_KEY Actions secret'ı eklendi (doğrulandı). Sıradaki adım: bota 5DollarFootballAPI O0.5/O1.5 çekme adımı eklemek. | 27.09: bot bağlandı (95957ef, 7d27614): scripts/fetch_goal_odds.py saatte ≤40 istek, 5 lig kimliği bulundu, oranlar data/goal-odds.json, kupon 0.5+/1.5+ için gerçek Bet365 oranını kullanıyor. Uluslararası ara: ilk gerçek oranlar 9–10 Ekim maçlarında; o hafta goal-odds.json dolu mu ve kuponda "tahmini" yazısı kalkıyor mu kontrol edilecek, sonra Tamamlandı.</t>
         </is>
       </c>
       <c r="L24" s="19" t="n">
         <v>46291</v>
       </c>
       <c r="M24" s="19" t="n"/>
-      <c r="N24" s="7" t="n"/>
+      <c r="N24" s="7" t="inlineStr">
+        <is>
+          <t>95957ef + 7d27614 Bet365 O0.5/O1.5 çekme adımı + kupona bağlama</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -2292,7 +2296,56 @@
       </c>
     </row>
     <row r="31">
-      <c r="L31" s="20" t="n"/>
+      <c r="A31" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Fikstür başlığında dönen futbol topu + lig yörüngesi</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Başlığın sağında 3B dönen top (canvas, kesik ikosahedron, kütüphanesiz), etrafında 10 lig bayrağı yörüngede; bayrağa tıklayınca Fikstür o lige filtrelenir; kutularda canlı sayılar (bu ayki maç, vurgu isabeti, sıradaki gün) sayarak yükselir. Örnek: https://claude.ai/artifact/BK7JszNNrtiifGcp8ocsi2</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Murat (27.09, Tofiko esinli)</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I31" s="7" t="n"/>
+      <c r="J31" s="8" t="n"/>
+      <c r="K31" s="7" t="inlineStr">
+        <is>
+          <t>Murat örneğe bakıp karar verecek.</t>
+        </is>
+      </c>
+      <c r="L31" s="19" t="n">
+        <v>46292</v>
+      </c>
+      <c r="M31" s="19" t="n"/>
+      <c r="N31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="L32" s="20" t="n"/>

</xml_diff>

<commit_message>
Is listesi #27 tamamlandi (959cbdb)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2331,21 +2331,27 @@
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>Öneri</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="I31" s="7" t="n"/>
       <c r="J31" s="8" t="n"/>
       <c r="K31" s="7" t="inlineStr">
         <is>
-          <t>Murat örneğe bakıp karar verecek.</t>
+          <t>Murat: hızı düşür; sonra "kopuk duruyor" → yalnız Fikstür, küçük, sayı kutuları kaldırıldı (bandı tekrar ediyordu). Aynı turda Kasa Gelişim Grafiği de futuristik yapıldı (dolarak yükselen sütunlar, hedef eğrisi).</t>
         </is>
       </c>
       <c r="L31" s="19" t="n">
         <v>46292</v>
       </c>
-      <c r="M31" s="19" t="n"/>
-      <c r="N31" s="7" t="n"/>
+      <c r="M31" s="19" t="n">
+        <v>46292</v>
+      </c>
+      <c r="N31" s="7" t="inlineStr">
+        <is>
+          <t>77db376 + 959cbdb dönen top + lig yörüngesi (yalnız Fikstür), kasa grafiği yenilendi</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="L32" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: #28 kupon kartı sadeleştirme tamamlandı (67347ba)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -20,9 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
     <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -2354,7 +2355,58 @@
       </c>
     </row>
     <row r="32">
-      <c r="L32" s="20" t="n"/>
+      <c r="A32" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Kupon kartı: Gerçekçi beklenti ve Geçmiş öneriler kaldır</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Kupon önerisi kartındaki 'Gerçekçi beklenti' (1 yıllık simülasyon) ve 'Geçmiş öneriler' bölümleri kaldırılsın; kartta yalnız kupon ve özet satırı kalsın.</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I32" s="7" t="n"/>
+      <c r="J32" s="8" t="n"/>
+      <c r="K32" s="7" t="n"/>
+      <c r="L32" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M32" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N32" s="7" t="inlineStr">
+        <is>
+          <t>67347ba — coupon_suggest.js: iki bölüm ve kullanılmayan simulate/ruleFor/historyHtml kaldırıldı</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="L33" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: Süper Lig fikstür düzeltmesi (324835f)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2409,7 +2409,62 @@
       </c>
     </row>
     <row r="33">
-      <c r="L33" s="20" t="n"/>
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Süper Lig fikstürde ve yörüngede görünmüyor</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Fikstür lig menüsünde Turkish Süper Lig 0 maç, başlıktaki lig yörüngesinde bayrak yok. Neden: tff.org fikstür sayfası 18-20 Eylül haftasında takılı; bot bir aylık pencerede maç bulamıyor.</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="n"/>
+      <c r="J33" s="8" t="n"/>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>Bot saatlik çalışınca predictions.json Süper Lig maçlarıyla dolar (ilk maçlar 9 Ekim, milli ara). Sitede görünmesi kontrol edilecek.</t>
+        </is>
+      </c>
+      <c r="L33" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M33" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N33" s="7" t="inlineStr">
+        <is>
+          <t>324835f — Süper Lig fikstürü ESPN tur.1'den (27 maç / 30 gün), TFF yalnız yedek; Başakşehir takma adı</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="L34" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: olasılık çekirdeği tamamlandı (73f95c2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2467,7 +2467,62 @@
       </c>
     </row>
     <row r="34">
-      <c r="L34" s="20" t="n"/>
+      <c r="A34" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>Fikstür başlığı: top yerine olasılık çekirdeği</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Lig yörüngesinin ortasındaki futbol topu basit duruyordu. 4 öneri (holografik, olasılık çekirdeği, nokta bulutu, neon cam) önizlemede gösterildi; olasılık çekirdeği seçildi: iç içe üç halka vurgu isabet oranlarıyla dolar (genel, 1X, 2.5+), ortada genel isabet, tıklayınca İstatistikler.</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I34" s="7" t="n"/>
+      <c r="J34" s="8" t="n"/>
+      <c r="K34" s="7" t="inlineStr">
+        <is>
+          <t>Murat yerelde görüp onayladı, sonra push.</t>
+        </is>
+      </c>
+      <c r="L34" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M34" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N34" s="7" t="inlineStr">
+        <is>
+          <t>73f95c2 — js/ball_orbit.js çekirdek (data/stats-summary.json), açık tema tonları, TR/EN/NL</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="L35" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: yaklaşan öne çıkan maçlar tamamlandı (c2505bd)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2525,7 +2525,58 @@
       </c>
     </row>
     <row r="35">
-      <c r="L35" s="20" t="n"/>
+      <c r="A35" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Öne çıkanlar: "Yaklaşan öne çıkan maçlar", yalnız H2H’lı maçlar</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>'Günün öne çıkanları' bugünün maçı olmayan günleri gösterince yanıltıyordu (ör. 9 Ekim). Başlık 'Yaklaşan öne çıkan maçlar' oldu; listeye yalnız H2H + form (●●●) verili maçlar giriyor, yalnız formlu (●●) ve kısıtlı veriler girmiyor.</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="n"/>
+      <c r="J35" s="8" t="n"/>
+      <c r="K35" s="7" t="n"/>
+      <c r="L35" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M35" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N35" s="7" t="inlineStr">
+        <is>
+          <t>c2505bd — js/ux_extras.js H2H filtresi + başlık, TR/EN/NL, test_ux_extras kontrolü</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="L36" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: gün seçiliyken Vurgu tamamlandı (64516d7)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2579,7 +2579,58 @@
       </c>
     </row>
     <row r="36">
-      <c r="L36" s="20" t="n"/>
+      <c r="A36" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Fikstür: gün seçiliyken Vurgu filtresi</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Fikstür'de bir gün seçilince Vurgu düğmesi kilitleniyordu. Artık gün seçiliyken de açılıyor ve o günün maçlarını vurgulu olanlara indiriyor (sayaç: n / gün toplamı). Takım aramasında kapalı kalıyor.</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I36" s="7" t="n"/>
+      <c r="J36" s="8" t="n"/>
+      <c r="K36" s="7" t="n"/>
+      <c r="L36" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M36" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N36" s="7" t="inlineStr">
+        <is>
+          <t>64516d7 — index.html visible()/renderPred kilidi kaldırıldı, test_ux_extras kontrolü</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="L37" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: logo Nöral Radar (0c1664a) + nihai logo için açık iş
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2633,10 +2633,110 @@
       </c>
     </row>
     <row r="37">
-      <c r="L37" s="20" t="n"/>
+      <c r="A37" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Logo: Nöral Radar (geçici)</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Yeni logo: 3 tur öneri (5 konsept → radar varyasyonları → yapay zekâ varyasyonları, scratch/logo_*.html). Seçilen: Nöral Radar — altıgen, 6 pazar = 6 nöron, ortada yapay zekâ çekirdeği; sloganda AI rozeti. Sekme ikonu ve brand/ PNG'leri güncellendi.</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="n"/>
+      <c r="J37" s="8" t="n"/>
+      <c r="K37" s="7" t="inlineStr">
+        <is>
+          <t>Murat: "şimdilik" seçildi, konuya tekrar dönülecek (ayrı satır).</t>
+        </is>
+      </c>
+      <c r="L37" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M37" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N37" s="7" t="inlineStr">
+        <is>
+          <t>0c1664a — üst menü logosu, brand/betavus-mark.svg favicon (index/backtest/gizlilik), brand PNG'ler</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="L38" s="20" t="n"/>
+      <c r="A38" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Logo: nihai tasarıma tekrar dönülecek</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Nöral Radar geçici seçim. Daha analitik / AI-driven hissi için tekrar ele alınacak; adaylar: Nöral Radar + AI Çip birleşimi, yazı karakteri/wordmark. Giriş ekranı (gate) ve gizlilik sayfasındaki eski sarı-mavi BETAVUS yazısı da yeni stile çekilmeli.</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>Açık</t>
+        </is>
+      </c>
+      <c r="I38" s="7" t="n"/>
+      <c r="J38" s="8" t="n"/>
+      <c r="K38" s="7" t="n"/>
+      <c r="L38" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M38" s="19" t="n"/>
+      <c r="N38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="L39" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: kasa tablosu bugün vurgusu kaldırıldı (4766c44)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2739,7 +2739,58 @@
       <c r="N38" s="7" t="n"/>
     </row>
     <row r="39">
-      <c r="L39" s="20" t="n"/>
+      <c r="A39" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Günlük kasa tablosu: "Bugün" vurgusu kaldır</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Tablo takvim gününe göre bir satırı 'BUGÜN' diye vurguluyordu; kullanıcı arada birkaç gün oynamayınca vurgu yanlış satırda kalıyor. Satır vurgusu, BUGÜN etiketi ve başlıktaki 'bugün N. gün' kaldırıldı. Kasa Gelişim Grafiği'ndeki 'Bugün' çizgisi şimdilik duruyor.</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="n"/>
+      <c r="J39" s="8" t="n"/>
+      <c r="K39" s="7" t="n"/>
+      <c r="L39" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M39" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N39" s="7" t="inlineStr">
+        <is>
+          <t>4766c44 — paper_ui.js tablo + başlık, ilgili CSS ve çeviri</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="L40" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: kasa tablosu yapışkan başlık düzeltildi (1cb0320)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2793,7 +2793,58 @@
       </c>
     </row>
     <row r="40">
-      <c r="L40" s="20" t="n"/>
+      <c r="A40" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Günlük kasa tablosu: kaydırınca satırlar başlığa giriyor</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Tablo kaydırılınca satırlar yapışkan başlık satırının arkasından görünüyordu (başlık arka planı saydamdı). Başlık opak yapıldı ve satırların üstünde kalıyor.</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I40" s="7" t="n"/>
+      <c r="J40" s="8" t="n"/>
+      <c r="K40" s="7" t="n"/>
+      <c r="L40" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M40" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N40" s="7" t="inlineStr">
+        <is>
+          <t>1cb0320 — index.html .kasa-sim-table th opak; test_paper_betting kaydırma kontrolü</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="L41" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: kasa trend çizgisi tamamlandı (de51bae)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2847,7 +2847,62 @@
       </c>
     </row>
     <row r="41">
-      <c r="L41" s="20" t="n"/>
+      <c r="A41" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Kasa Gelişim Grafiği: trend çizgisi + belirsizlik bandı</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Gerçek kasa gelişimine göre trend: son 7 oynanan günün kasasına (oyundaki + kilitli) üstel eğri; oynanan kısım düz, gelecek kesikli + tahmin bandı. Altında trend büyüme (plana göre), bu gidişle son gün kasası (bant) ve hedefe varış günü. 3 yöntem önizlemede karşılaştırıldı (scratch/kasa_trend.html), son 7 gün seçildi.</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I41" s="7" t="n"/>
+      <c r="J41" s="8" t="n"/>
+      <c r="K41" s="7" t="inlineStr">
+        <is>
+          <t>Oynanmayan günler atlanır; 3 oynanmış günden azsa trend gösterilmez. Az veriyle (ör. 5 gün) uzak gelecek tahmini çok geniş/yüksek çıkabilir.</t>
+        </is>
+      </c>
+      <c r="L41" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M41" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N41" s="7" t="inlineStr">
+        <is>
+          <t>de51bae — paper_ui.js kasaTrend + grafik + kutular, TR/EN/NL, test_paper_betting kontrolü</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="L42" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: kasa grafiği trend penceresi (32cfb27)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -2905,7 +2905,62 @@
       </c>
     </row>
     <row r="42">
-      <c r="L42" s="20" t="n"/>
+      <c r="A42" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Kasa grafiği: Bugün çizgisi kaldır + güne göre trend penceresi</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Grafikteki 'Bugün' çizgisi kaldırıldı (oynanmayan günlerde yanlış yerde kalıyordu). Trend penceresi son oynanan güne (D) göre: D ≤ 7 tüm günler, D ≤ 14 son 7 gün, D ≥ 15 son ⌊D/2⌋ gün (20. gün → 10, 26. gün → 13). Lejantta pencere yazıyor.</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I42" s="7" t="n"/>
+      <c r="J42" s="8" t="n"/>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>Pencerede 3 oynanmış günden az kalırsa son 3 oynanan gün alınır.</t>
+        </is>
+      </c>
+      <c r="L42" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M42" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N42" s="7" t="inlineStr">
+        <is>
+          <t>32cfb27 — paper_ui.js trendWindow + Bugün çizgisi kaldırıldı, test güncellendi</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="L43" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: #39 yeni logo tamamlandı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -20,10 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd.mm.yyyy"/>
     <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -2963,7 +2962,62 @@
       </c>
     </row>
     <row r="43">
-      <c r="L43" s="20" t="n"/>
+      <c r="A43" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Yeni logo: VC-10 kıvrık şerit + neon top</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>scratch/vc10-ribbon-ball logosu siteye işlendi: sekme simgesi (SVG + 32px PNG), telefon simgesi (180px), üst menü logosu (koyu zemin, kırpılmış yatay işaret). Yazılı logo (koyu/açık) ve açık zemin işareti brand/ klasöründe hazır. Eski betavus-logo-120/512.png kaldırıldı.</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I43" s="7" t="n"/>
+      <c r="J43" s="8" t="n"/>
+      <c r="K43" s="7" t="inlineStr">
+        <is>
+          <t>Menü logosu tarayıcıda görsel olarak kontrol edilmeli (otomatik ekran görüntüsü alınamadı). animated.gif eklenmedi (1 MB).</t>
+        </is>
+      </c>
+      <c r="L43" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M43" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N43" s="7" t="inlineStr">
+        <is>
+          <t>d219b43 — brand/ yeni simge ve logolar; index/backtest/gizlilik favicon + menü logosu</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="L44" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: #40 animasyonlu gerçekçi top tamamlandı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3020,7 +3020,62 @@
       </c>
     </row>
     <row r="44">
-      <c r="L44" s="20" t="n"/>
+      <c r="A44" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Logo: gerçekçi animasyonlu top + giriş ekranı logosu</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Menü logosu animasyonsuzdu (statik SVG) ve top düz sarı daire gibi duruyordu. Top gölgeli beyaz futbol topu oldu (beşgen yamalar, dikişler, parlama); yamalar döner, hale nabız gibi atar (SVG içinde SMIL). Erişim kodu ekranında BETAVUS yazısı yerine yeni logo (koyu/açık tema). Favicon ve uygulama simgesi de aynı topla yeniden üretildi.</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I44" s="7" t="n"/>
+      <c r="J44" s="8" t="n"/>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>Tarayıcı önbelleği eski favicon'u bir süre gösterebilir.</t>
+        </is>
+      </c>
+      <c r="L44" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M44" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N44" s="7" t="inlineStr">
+        <is>
+          <t>b684dc4 — brand/ SVG'lerde yeni top + animasyon, index.html giriş ekranı logosu, simge PNG'leri</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="L45" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: #41 logo dalga animasyonu tamamlandı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3078,7 +3078,62 @@
       </c>
     </row>
     <row r="45">
-      <c r="L45" s="20" t="n"/>
+      <c r="A45" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Logo animasyonu: şerit dalgası akar, top döner</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Canlıda logo animasyonsuz görünüyordu: yalnızca küçük top dönüyordu, 36px'de fark edilmiyor. animated.gif'teki gibi şerit de dalgalanıyor (mevcut şeritten uydurulan dalga formülü, 12 kare SMIL). Top 3 sn'de bir tur döner, hale nabız gibi atar.</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I45" s="7" t="n"/>
+      <c r="J45" s="8" t="n"/>
+      <c r="K45" s="7" t="inlineStr">
+        <is>
+          <t>Favicon ve PNG simgeler hareketsiz (tarayıcılar favicon animasyonu oynatmaz).</t>
+        </is>
+      </c>
+      <c r="L45" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M45" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N45" s="7" t="inlineStr">
+        <is>
+          <t>2ab6554 — ribbon dalga animasyonu brand/ 4 SVG'de, top dönüşü 3 sn, viewBox genişletildi</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="L46" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: #42 logo büyütüldü
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3136,7 +3136,58 @@
       </c>
     </row>
     <row r="46">
-      <c r="L46" s="20" t="n"/>
+      <c r="A46" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Logo biraz küçük: menüde ve giriş ekranında büyüt</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Dalga animasyonu için çerçeve genişleyince menü logosu küçülmüştü. Menü işareti 36→50px (telefonda 40/34/28px), erişim kodu ekranındaki logo 300→340px.</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>Düşük</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I46" s="7" t="n"/>
+      <c r="J46" s="8" t="n"/>
+      <c r="K46" s="7" t="n"/>
+      <c r="L46" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M46" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N46" s="7" t="inlineStr">
+        <is>
+          <t>0f02eb0 — index.html .bv-mark ve .gate-brand img boyutları</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="L47" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: #43 logo topu büyütüldü
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3190,7 +3190,58 @@
       </c>
     </row>
     <row r="47">
-      <c r="L47" s="20" t="n"/>
+      <c r="A47" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Logo: top küçük kalıyor, büyüt</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Logo büyütülünce top şeride göre küçük kaldı. Top (hale ve parıltı dahil) merkezinden 1,5 kat büyütüldü; menü işaretinin çerçevesi sağa genişletildi, favicon/uygulama simgesi PNG'leri yeniden üretildi.</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Düşük</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I47" s="7" t="n"/>
+      <c r="J47" s="8" t="n"/>
+      <c r="K47" s="7" t="n"/>
+      <c r="L47" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M47" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N47" s="7" t="inlineStr">
+        <is>
+          <t>2e271de — brand/ 5 SVG'de top ölçeği 1,5, simge PNG'leri, index.html işaret genişliği</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="L48" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: #44 futuristik maç kartı tamamlandı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3244,7 +3244,58 @@
       </c>
     </row>
     <row r="48">
-      <c r="L48" s="20" t="n"/>
+      <c r="A48" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>Maç kartı: futuristik tasarım</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>Maça tıklayınca açılan kart sade/eski görünüyordu. Başlık: takım monogramları + sıra/puan, ortada beklenen gol (λ) halka göstergesi, lig/tarih çipleri. Cam paneller, köşe braketleri, ızgara zemin, kademeli açılma. Olasılık çubukları neon dolgu + parıltı, puan durumu satır kartları, H2H galibiyet dağılım çubuğu + skorbord skorlar, parlayan gol grafiği. Koyu/açık tema + telefon.</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I48" s="7" t="n"/>
+      <c r="J48" s="8" t="n"/>
+      <c r="K48" s="7" t="n"/>
+      <c r="L48" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M48" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N48" s="7" t="inlineStr">
+        <is>
+          <t>ac20920 — index.html matchHero + .sheet/.s-card HUD stilleri, goalChart parıltı, i18n 4 yeni metin</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="L49" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: #45 takım armaları tamamlandı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3298,7 +3298,62 @@
       </c>
     </row>
     <row r="49">
-      <c r="L49" s="20" t="n"/>
+      <c r="A49" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Maç kartı: takım armaları</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Maç kartındaki takım altıgenlerinde baş harfler yerine armalar. scripts/fetch_team_logos.py ESPN takım listesinden 10 ligin 192 takımını eşleştirir (data/team-logos.json); yalnızca arması eksik takımı olan lig yeniden çekilir, bot her saat çalıştırır. Amedspor ESPN'de yok: tr.wikipedia armasından brand/crests/amedspor.png. Arma yüklenemezse baş harfler görünür.</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I49" s="7" t="n"/>
+      <c r="J49" s="8" t="n"/>
+      <c r="K49" s="7" t="inlineStr">
+        <is>
+          <t>Yeni yükselen takım ESPN'de arma olmadan gelirse MANUAL listesine eklenmeli (fetch_team_logos.py).</t>
+        </is>
+      </c>
+      <c r="L49" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M49" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N49" s="7" t="inlineStr">
+        <is>
+          <t>a1139c3 — fetch_team_logos.py + team-logos.json, index.html arma gösterimi, update.yml adımı</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="L50" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: #46 arma boyutu ve hover efekti tamamlandı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3356,7 +3356,62 @@
       </c>
     </row>
     <row r="50">
-      <c r="L50" s="20" t="n"/>
+      <c r="A50" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Maç kartı armaları: çerçevesiz, büyük, üstüne gelince öne çıksın</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>Arma varsa altıgen çerçeve kaldırıldı, arma 68px (telefonda 50px). Fareyle üstüne gelince arma yukarı kalkıp 1,3 kat büyür ve takım renginde parlar; fare çekilince yumuşakça yerine döner. Arma yoksa baş harfli altıgen kalır.</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Düşük</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I50" s="7" t="n"/>
+      <c r="J50" s="8" t="n"/>
+      <c r="K50" s="7" t="inlineStr">
+        <is>
+          <t>Dokunmatik ekranlarda üstüne gelme olmadığı için büyüme efekti yok.</t>
+        </is>
+      </c>
+      <c r="L50" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M50" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N50" s="7" t="inlineStr">
+        <is>
+          <t>94c1791 — index.html .mx-crest has-logo boyutu + hover efekti</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="L51" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: #47 futuristik arayüz tamamlandı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3414,7 +3414,62 @@
       </c>
     </row>
     <row r="51">
-      <c r="L51" s="20" t="n"/>
+      <c r="A51" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Futuristik arayüz: bayraklı dil seçici + site geneli</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Dil seçici SVG bayraklı neon açılır menü (TR/EN/NL). Maç kartındaki tasarım dili tüm siteye tek CSS katmanıyla: cam paneller + neon saç çizgisi (kartlar, maç listesi, KPI, kasa blokları, FAQ, üyelik penceresi), parlayan filtre/arama/seçim kontrolleri, gün şeridi, HUD tablo başlıkları, satır tarama çizgisi; Sanal Kasa mavi şerit başlıklar neon etikete döndü. Koyu/açık tema.</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Murat (28.09)</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I51" s="7" t="n"/>
+      <c r="J51" s="8" t="n"/>
+      <c r="K51" s="7" t="inlineStr">
+        <is>
+          <t>Kapsam dışı kaldı: ayrı sayfalar backtest.html ve gizlilik.html (kendi stilleri var), Rehber turu balonları.</t>
+        </is>
+      </c>
+      <c r="L51" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="M51" s="19" t="n">
+        <v>46293</v>
+      </c>
+      <c r="N51" s="7" t="inlineStr">
+        <is>
+          <t>c3b1e56 — js/i18n.js mountSwitcher, index.html futuristik katman</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="L52" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: #47 kalan sayfalar tamamlandı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3456,7 +3456,7 @@
       <c r="J51" s="8" t="n"/>
       <c r="K51" s="7" t="inlineStr">
         <is>
-          <t>Kapsam dışı kaldı: ayrı sayfalar backtest.html ve gizlilik.html (kendi stilleri var), Rehber turu balonları.</t>
+          <t>backtest.html, gizlilik.html (logo + bayraklı dil düğmeleri), Rehber turu balonu ve 'Tüm vurgular' filtresi de 1cab1c4 ile aynı stile getirildi.</t>
         </is>
       </c>
       <c r="L51" s="19" t="n">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="N51" s="7" t="inlineStr">
         <is>
-          <t>c3b1e56 — js/i18n.js mountSwitcher, index.html futuristik katman</t>
+          <t>c3b1e56 — dil seçici + site geneli katman; 1cab1c4 — backtest/gizlilik sayfaları, Rehber turu, istatistik filtresi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
İş listesi: #48 holografik logo topu tamamlandı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3472,7 +3472,58 @@
       </c>
     </row>
     <row r="52">
-      <c r="L52" s="20" t="n"/>
+      <c r="A52" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>Logo topu: holografik</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Gelen yorum: beyaz gerçekçi top logoya sadelik katmış. 4 seçenek (düz neon, neon 3B, holografik, beyaz) yan yana karşılaştırıldı; holografik (beyazdan turkuaza, koyu yamalar, neon sarı hale) seçildi. Animasyon aynı; menü, giriş ekranı, favicon/simge güncellendi.</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>Murat (29.09)</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I52" s="7" t="n"/>
+      <c r="J52" s="8" t="n"/>
+      <c r="K52" s="7" t="n"/>
+      <c r="L52" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="M52" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="N52" s="7" t="inlineStr">
+        <is>
+          <t>249331b — brand/ 5 SVG'de top C seçeneği, simge PNG'leri</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="L53" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: #49 logo neon hedef tamamlandı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3526,7 +3526,58 @@
       </c>
     </row>
     <row r="53">
-      <c r="L53" s="20" t="n"/>
+      <c r="A53" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Logo: top yerine neon hedef</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Holografik top (#48) menü boyutunda beyaz görünüyordu; top fikri de beğenilmedi. Menü boyutunda karşılaştırılan seçeneklerden neon hedef seçildi: dönen kesikli halka + nabız gibi atan parlak çekirdek + genişleyen hale (tasarımcının ilk 'glowing target' fikri). Dalga animasyonu aynı; menü, giriş ekranı, favicon/simge güncellendi.</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Murat (29.09)</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I53" s="7" t="n"/>
+      <c r="J53" s="8" t="n"/>
+      <c r="K53" s="7" t="n"/>
+      <c r="L53" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="M53" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="N53" s="7" t="inlineStr">
+        <is>
+          <t>fe8cfc2 — brand/ 5 SVG'de E seçeneği, simge PNG'leri</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="L54" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: #50 logo mini saha tamamlandı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3580,7 +3580,62 @@
       </c>
     </row>
     <row r="54">
-      <c r="L54" s="20" t="n"/>
+      <c r="A54" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>Logo: mini saha + kırmızı neon top</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>Logo ucu için 11 seçenek (neon hedef, radar, altıgen, yörünge, yüzde halkası, tel çerçeve top, Poisson, çan eğrisi, kale, %, mini saha) scratch/logo-oneriler altında canlı önizlemeyle sunuldu. Mini saha seçildi; istekle top kırmızı neon, saha ~%14 büyük. Menü, giriş ekranı logoları ve favicon/simge güncellendi.</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>Murat (29.09)</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I54" s="7" t="n"/>
+      <c r="J54" s="8" t="n"/>
+      <c r="K54" s="7" t="inlineStr">
+        <is>
+          <t>Önizleme ve diğer seçenekler: scratch/logo-oneriler (yalnız Murat'ın bilgisayarında). #34 (logo nihai tasarım) ile ilgili.</t>
+        </is>
+      </c>
+      <c r="L54" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="M54" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="N54" s="7" t="inlineStr">
+        <is>
+          <t>8b55376 — brand/ 5 SVG'de S2 seçeneği, simge PNG'leri</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="L55" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi: #50 saha büyütme düzeltmesi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3595,7 +3595,7 @@
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Logo ucu için 11 seçenek (neon hedef, radar, altıgen, yörünge, yüzde halkası, tel çerçeve top, Poisson, çan eğrisi, kale, %, mini saha) scratch/logo-oneriler altında canlı önizlemeyle sunuldu. Mini saha seçildi; istekle top kırmızı neon, saha ~%14 büyük. Menü, giriş ekranı logoları ve favicon/simge güncellendi.</t>
+          <t>Logo ucu için 11 seçenek (neon hedef, radar, altıgen, yörünge, yüzde halkası, tel çerçeve top, Poisson, çan eğrisi, kale, %, mini saha) scratch/logo-oneriler altında canlı önizlemeyle sunuldu. Mini saha seçildi; istekle top kırmızı neon, saha ~%14 büyük. Menü, giriş ekranı logoları ve favicon/simge güncellendi. Düzeltme: menüde çok küçük görünüyordu; saha 2,2 kat ölçek, kırmızı top iri, giriş ekranı logosunda işaret yazıdan uzaklaştırıldı.</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="N54" s="7" t="inlineStr">
         <is>
-          <t>8b55376 — brand/ 5 SVG'de S2 seçeneği, simge PNG'leri</t>
+          <t>8b55376 — brand/ 5 SVG'de S2 seçeneği, simge PNG'leri; 07e0130 — saha büyütüldü</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
İş listesi: #51 radar logo tamamlandı
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3638,7 +3638,62 @@
       </c>
     </row>
     <row r="55">
-      <c r="L55" s="20" t="n"/>
+      <c r="A55" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Logo: radar + kırmızı neon noktalar</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Mini saha (#50) onaydan geçmedi; 4 önizleme turunda 23 seçenek sunuldu (scratch/logo-oneriler, tur3, tur4). Radar (F) seçildi: dönen tarama ışını, halkalar; merkez nokta ve belirip kaybolan nokta kırmızı neon. Büyük ölçek korundu. Menü, giriş ekranı, favicon/simge güncellendi.</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Murat (29.09)</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>Tamamlandı</t>
+        </is>
+      </c>
+      <c r="I55" s="7" t="n"/>
+      <c r="J55" s="8" t="n"/>
+      <c r="K55" s="7" t="inlineStr">
+        <is>
+          <t>Diğer seçenekler scratch/logo-oneriler altında (yalnız Murat'ın bilgisayarında).</t>
+        </is>
+      </c>
+      <c r="L55" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="M55" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="N55" s="7" t="inlineStr">
+        <is>
+          <t>83085cb — brand/ 5 SVG'de radar (F), simge PNG'leri</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="L56" s="20" t="n"/>

</xml_diff>

<commit_message>
İş listesi #52: İlk yarı / maç sonucu (İY/MS) istatistiksel çalışması eklendi (Açık)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3696,7 +3696,56 @@
       </c>
     </row>
     <row r="56">
-      <c r="L56" s="20" t="n"/>
+      <c r="A56" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>İlk yarı ve maç sonucu (İY/MS) istatistiksel çalışması</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Siteye dokunmadan, önce istatistiksel çalışma: İlk yarı 1X2, maç sonu 1X2 ve birleşik İY/MS (9 sonuç: 1/1, X/1, 2/1 …) olasılıklarının modellenmesi ve 2021/22–2026/27 walk-forward backtest'i. Veri: football-data CSV'lerindeki ilk yarı skorları (HTHG/HTAG) ve maç sonu 1X2 oranları (İY/MS oranı CSV'de yok → kaynak araştırılacak). Ölçüler: kalibrasyon, Brier/log-loss, marjsız piyasaya karşı karşılaştırma, eşik bazında isabet + başabaş + ROI (Wilson aralığıyla); eşikler yalnız eski sezonlarda seçilip yeni sezonlarda doğrulanacak (örneklem-dışı). Çıktı: rapor + karar (yayına alınır mı?).</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>Murat (02.10)</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>Açık</t>
+        </is>
+      </c>
+      <c r="I56" s="7" t="n"/>
+      <c r="J56" s="8" t="n"/>
+      <c r="K56" s="7" t="inlineStr">
+        <is>
+          <t>Murat: henüz siteye dokunulmayacak; önce istatistiksel çalışma. SISTEM_RAPORU.md bulguları (model 1X2/ÇŞ'de piyasadan zayıf) dikkate alınmalı.</t>
+        </is>
+      </c>
+      <c r="L56" s="19" t="n">
+        <v>46297</v>
+      </c>
+      <c r="M56" s="19" t="n"/>
+      <c r="N56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="L57" s="20" t="n"/>

</xml_diff>

<commit_message>
Karşılaştırma raporları docs/karsilastirma-2026-10 altında; iş listesine #53-#66 öneri
Ufuk Özbek'in BETAVUS-SistemGol karşılaştırması (ilk sürüm + R01),
kaynağı olan SISTEM_RAPORU.md ve BETAVUS'un savunma raporu (PDF + HTML,
41 iddia için doğru/kabul kararı) tek klasörde, README ile. docs/
Vercel'e yüklenmez. SISTEMGOL_RAPORU.md repo açık olduğu için bilerek
eklenmedi.

Savunma raporundaki iyileştirmeler B1-B14, BETAVUS_Is_Listesi.xlsx'e
#53-#66 olarak "Öneri" durumunda eklendi; hiçbiri uygulanmadı.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BETAVUS_Is_Listesi.xlsx
+++ b/BETAVUS_Is_Listesi.xlsx
@@ -3748,46 +3748,732 @@
       <c r="N56" s="7" t="n"/>
     </row>
     <row r="57">
-      <c r="L57" s="20" t="n"/>
+      <c r="A57" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Kasa planı: büyüme hedefi yerine edge temelli stake</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Günlük büyüme hedefini ve ondan türetilen gerekli kupon oranını (R = 1 + g/f) kaldırmak. Stake kasanın %1–3'ü ya da kesirli Kelly; edge ≤ 0 ise "oynanmaz". Gerekçe: Dengeli profilde kasanın büyümesi için %80,4 kupon isabeti gerekiyor, geçmişte gerçekleşen %68,6; bootstrap'ta 90 kupon sonra kasa %97 olasılıkla %10'un altında.</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>Ufuk R01 / Claude (Murat) 03.10</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I57" s="7" t="n"/>
+      <c r="J57" s="8" t="n"/>
+      <c r="K57" s="7" t="inlineStr">
+        <is>
+          <t>Savunma raporu B1: docs/karsilastirma-2026-10/BETAVUS_SistemGol_Savunma_Raporu.pdf</t>
+        </is>
+      </c>
+      <c r="L57" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="M57" s="19" t="n"/>
+      <c r="N57" s="7" t="n"/>
     </row>
     <row r="58">
-      <c r="L58" s="20" t="n"/>
+      <c r="A58" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="B58" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>Kupon kartı ile Güven Payı tutarlı olsun</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Kart "Kupona yatacak 150 €" derken Güven Payı aynı anda "180 € kilitle" uyarısı veriyor; kart kilidi hesaba katmıyor. Önce kilit, sonra stake. Gerçek hata.</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>Ufuk R01 / Claude (Murat) 03.10</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I58" s="7" t="n"/>
+      <c r="J58" s="8" t="n"/>
+      <c r="K58" s="7" t="inlineStr">
+        <is>
+          <t>Savunma raporu B2: docs/karsilastirma-2026-10/BETAVUS_SistemGol_Savunma_Raporu.pdf</t>
+        </is>
+      </c>
+      <c r="L58" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="M58" s="19" t="n"/>
+      <c r="N58" s="7" t="n"/>
     </row>
     <row r="59">
-      <c r="L59" s="20" t="n"/>
+      <c r="A59" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Gerçekçi beklenti simülasyonu geri gelsin</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>#28 ile kaldırılan simülasyon doğru göstergelerle geri gelsin: kupon başına beklenen log büyüme, N kupon sonra kasanın %10'un altına düşme olasılığı, gerekli isabet / gerçekleşen isabet. Profiller geçmiş kuponlarla test edilip ekranda gösterilsin.</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>Ufuk R01 / Claude (Murat) 03.10</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I59" s="7" t="n"/>
+      <c r="J59" s="8" t="n"/>
+      <c r="K59" s="7" t="inlineStr">
+        <is>
+          <t>Savunma raporu B3: docs/karsilastirma-2026-10/BETAVUS_SistemGol_Savunma_Raporu.pdf</t>
+        </is>
+      </c>
+      <c r="L59" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="M59" s="19" t="n"/>
+      <c r="N59" s="7" t="n"/>
     </row>
     <row r="60">
-      <c r="L60" s="20" t="n"/>
+      <c r="A60" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="B60" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>Arşiv: son maç öncesi tahmin + motor sürümü</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>predictions-archive yalnız ilk görülen tahmini (maçtan medyan 4,2 gün önce, oran gelmeden) saklıyor. Son maç öncesi tahmini de, engine_version ve market_used ile kaydetmek; canlı başarıyı son tahminden ölçmek. Ayrıca λ_ev/λ_dep yazılırsa ÇŞ canlı ölçülebilir.</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>Ufuk R01 / Claude (Murat) 03.10</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I60" s="7" t="n"/>
+      <c r="J60" s="8" t="n"/>
+      <c r="K60" s="7" t="inlineStr">
+        <is>
+          <t>Savunma raporu B4: docs/karsilastirma-2026-10/BETAVUS_SistemGol_Savunma_Raporu.pdf</t>
+        </is>
+      </c>
+      <c r="L60" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="M60" s="19" t="n"/>
+      <c r="N60" s="7" t="n"/>
     </row>
     <row r="61">
-      <c r="L61" s="20" t="n"/>
+      <c r="A61" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="B61" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>Alt lig tarihlerini ISO'ya çevir</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>update_predictions.py:641 alt lig satırlarına "dd/mm/YYYY" yazıyor; goals_model dize sıralaması yaptığı için (259, 409) "28/04/2026" &gt; "2026-09-13" sayılıyor. Yükselen takımlarda yakınlık ağırlığı ve H2H seçimi bozuluyor (~11 maç). Gerçek hata, çok küçük iş.</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>Ufuk R01 / Claude (Murat) 03.10</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I61" s="7" t="n"/>
+      <c r="J61" s="8" t="n"/>
+      <c r="K61" s="7" t="inlineStr">
+        <is>
+          <t>Savunma raporu B5: docs/karsilastirma-2026-10/BETAVUS_SistemGol_Savunma_Raporu.pdf</t>
+        </is>
+      </c>
+      <c r="L61" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="M61" s="19" t="n"/>
+      <c r="N61" s="7" t="n"/>
     </row>
     <row r="62">
-      <c r="L62" s="20" t="n"/>
+      <c r="A62" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="B62" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>Eskimiş 0-0 yorumunu düzelt</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>_league_rho docstring ve SISTEM_RAPORU.md "openfootball 0-0'ları eksik" diyor; doğru değil, kaynakta "score": [0, 0] biçiminde duruyorlar ve db2f1d0'dan (20.09) beri okunuyor. Yorum düzeltilsin; bu biçimi kapsayan bir regresyon testi eklensin.</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>Ufuk R01 / Claude (Murat) 03.10</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I62" s="7" t="n"/>
+      <c r="J62" s="8" t="n"/>
+      <c r="K62" s="7" t="inlineStr">
+        <is>
+          <t>Savunma raporu B6: docs/karsilastirma-2026-10/BETAVUS_SistemGol_Savunma_Raporu.pdf</t>
+        </is>
+      </c>
+      <c r="L62" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="M62" s="19" t="n"/>
+      <c r="N62" s="7" t="n"/>
     </row>
     <row r="63">
-      <c r="L63" s="20" t="n"/>
+      <c r="A63" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="B63" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>Oran yokken vurguya "ön tahmin" etiketi</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Ü/A 2,5 oranı henüz gelmemiş maçlarda tahmin piyasasız; vurgu "ön tahmin / piyasasız" diye ayırt edilsin. Piyasasız vurguların başarısı ayrıca ölçülsün, kötüyse kapatılsın.</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Ufuk R01 / Claude (Murat) 03.10</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I63" s="7" t="n"/>
+      <c r="J63" s="8" t="n"/>
+      <c r="K63" s="7" t="inlineStr">
+        <is>
+          <t>Savunma raporu B7: docs/karsilastirma-2026-10/BETAVUS_SistemGol_Savunma_Raporu.pdf</t>
+        </is>
+      </c>
+      <c r="L63" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="M63" s="19" t="n"/>
+      <c r="N63" s="7" t="n"/>
     </row>
     <row r="64">
-      <c r="L64" s="20" t="n"/>
+      <c r="A64" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="B64" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>Eşikleri örneklem-dışı seç, 0,5 eşiğini test et</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>Eşikleri yalnız ≤ 2023/24 ile seçip sonraki sezonlarda dondurulmuş haliyle ölçmek; sitede bu sayıyı göstermek. 0,5 eşiğini %93,5'ten ≥ %95'e almak test edilsin (tabanın yalnız 2,2 puan üstünde).</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>Ufuk R01 / Claude (Murat) 03.10</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I64" s="7" t="n"/>
+      <c r="J64" s="8" t="n"/>
+      <c r="K64" s="7" t="inlineStr">
+        <is>
+          <t>Savunma raporu B8: docs/karsilastirma-2026-10/BETAVUS_SistemGol_Savunma_Raporu.pdf</t>
+        </is>
+      </c>
+      <c r="L64" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="M64" s="19" t="n"/>
+      <c r="N64" s="7" t="n"/>
     </row>
     <row r="65">
-      <c r="L65" s="20" t="n"/>
+      <c r="A65" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="B65" s="9" t="inlineStr">
+        <is>
+          <t>2 - Arayüz: Kullanılabilirlik &amp; Profesyonel Görünüm</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>Başarı şeridine başabaş ve ROI; etiketleri yumuşat</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>Şerit yalnız isabet gösteriyor; %92 isabet ortalama 1,06 oranla zarar demek (başabaş %94,2). Başabaş ve ROI yan yana gösterilsin. "AI-powered" ve "Doğrulanmış" etiketleri ne anlama geldikleri açıklanarak yumuşatılsın.</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>Ufuk R01 / Claude (Murat) 03.10</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>Faz 2</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I65" s="7" t="n"/>
+      <c r="J65" s="8" t="n"/>
+      <c r="K65" s="7" t="inlineStr">
+        <is>
+          <t>Savunma raporu B9: docs/karsilastirma-2026-10/BETAVUS_SistemGol_Savunma_Raporu.pdf</t>
+        </is>
+      </c>
+      <c r="L65" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="M65" s="19" t="n"/>
+      <c r="N65" s="7" t="n"/>
     </row>
     <row r="66">
-      <c r="L66" s="20" t="n"/>
+      <c r="A66" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="B66" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>Gerçek oran gelene kadar 0,5/1,5 kupondan çıksın</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>Bugünkü kuponlarda 77 bacağın 77'si tahmini oranlı. Gerçek fiyat (#20) gelene kadar 0,5 ve 1,5 kupon motorundan çıkarılsın; 1,01 altı oran hiç seçilmesin.</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>Ufuk R01 / Claude (Murat) 03.10</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I66" s="7" t="n"/>
+      <c r="J66" s="8" t="n"/>
+      <c r="K66" s="7" t="inlineStr">
+        <is>
+          <t>Savunma raporu B10: docs/karsilastirma-2026-10/BETAVUS_SistemGol_Savunma_Raporu.pdf</t>
+        </is>
+      </c>
+      <c r="L66" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="M66" s="19" t="n"/>
+      <c r="N66" s="7" t="n"/>
     </row>
     <row r="67">
-      <c r="L67" s="20" t="n"/>
+      <c r="A67" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="B67" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>Çifte Şans: piyasayla harmanla ya da kaldır</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>Model ÇŞ'de piyasadan belirgin zayıf (Brier farkı 1X +0,014, X2 +0,016). Piyasadan ayrıştığı maçlarda (oran ≥ 1,40) isabet %57,7. 1X2 piyasa harmanı denensin; olmazsa pazar kaldırılsın.</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>Ufuk R01 / Claude (Murat) 03.10</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I67" s="7" t="n"/>
+      <c r="J67" s="8" t="n"/>
+      <c r="K67" s="7" t="inlineStr">
+        <is>
+          <t>Savunma raporu B11: docs/karsilastirma-2026-10/BETAVUS_SistemGol_Savunma_Raporu.pdf</t>
+        </is>
+      </c>
+      <c r="L67" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="M67" s="19" t="n"/>
+      <c r="N67" s="7" t="n"/>
     </row>
     <row r="68">
-      <c r="L68" s="20" t="n"/>
+      <c r="A68" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="B68" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>Alarm: iş akışı hatası ve sessiz sonuç</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>İş akışı düştüğünde veya birkaç gündür yeni sonuç gelmediğinde bildirim. validate_data.py var ama bildirim kanalı yok.</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>Ufuk R01 / Claude (Murat) 03.10</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I68" s="7" t="n"/>
+      <c r="J68" s="8" t="n"/>
+      <c r="K68" s="7" t="inlineStr">
+        <is>
+          <t>Savunma raporu B12: docs/karsilastirma-2026-10/BETAVUS_SistemGol_Savunma_Raporu.pdf</t>
+        </is>
+      </c>
+      <c r="L68" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="M68" s="19" t="n"/>
+      <c r="N68" s="7" t="n"/>
     </row>
     <row r="69">
-      <c r="L69" s="20" t="n"/>
+      <c r="A69" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="B69" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>Ertelenen maç için kupon iade kuralı</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>Ertelenen maç içeren kupon sonsuza dek "bekliyor" kalıyor (180 gün sonra siliniyor). İade (bacak oranı 1,00) kuralı eklensin.</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Ufuk R01 / Claude (Murat) 03.10</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Düşük</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I69" s="7" t="n"/>
+      <c r="J69" s="8" t="n"/>
+      <c r="K69" s="7" t="inlineStr">
+        <is>
+          <t>Savunma raporu B13: docs/karsilastirma-2026-10/BETAVUS_SistemGol_Savunma_Raporu.pdf</t>
+        </is>
+      </c>
+      <c r="L69" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="M69" s="19" t="n"/>
+      <c r="N69" s="7" t="n"/>
     </row>
     <row r="70">
-      <c r="L70" s="20" t="n"/>
+      <c r="A70" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="B70" s="9" t="inlineStr">
+        <is>
+          <t>1 - Teknik: Veri Doğruluğu</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>Piyasa düşük gol / favori filtresini gölgede ölç</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>Canlıdaki 8 adet 0,5 kaybının 8'inde piyasa düşük gol bekliyordu (Ü2,5 1,33–2,13). SistemGol'de 1X2 favori ≤ 1,25 filtresi dış testte 0,5'i %94,4 → %99,1 çıkarıyor. Önce gölgede, kazanan seçimlerle birlikte ölçülsün; walk-forward ile doğrulanmadan yayına alınmasın.</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>Ufuk R01 / Claude (Murat) 03.10</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>Düşük</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>Faz 1</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="I70" s="7" t="n"/>
+      <c r="J70" s="8" t="n"/>
+      <c r="K70" s="7" t="inlineStr">
+        <is>
+          <t>Savunma raporu B14: docs/karsilastirma-2026-10/BETAVUS_SistemGol_Savunma_Raporu.pdf</t>
+        </is>
+      </c>
+      <c r="L70" s="19" t="n">
+        <v>46298</v>
+      </c>
+      <c r="M70" s="19" t="n"/>
+      <c r="N70" s="7" t="n"/>
     </row>
     <row r="71">
       <c r="L71" s="20" t="n"/>

</xml_diff>